<commit_message>
docs: atualiza arquivos 'Planilha Textos Alternativos'
</commit_message>
<xml_diff>
--- a/Planilha Textos Alternativos.xlsx
+++ b/Planilha Textos Alternativos.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="364">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="576" uniqueCount="440">
   <si>
     <t>ID</t>
   </si>
@@ -46,19 +46,37 @@
     <t>Resumo da Noticia</t>
   </si>
   <si>
-    <t>Prompt sem Contexto</t>
+    <t>Prompt para Gemini Sem Gems</t>
+  </si>
+  <si>
+    <t>Prompt com URL</t>
   </si>
   <si>
     <t>Prompt com Contexto</t>
   </si>
   <si>
-    <t>Alt Text IA 1 - Tese da Carolina</t>
+    <t>Alt Text 1 - Tese da Carolina</t>
+  </si>
+  <si>
+    <t>Alt Text 1 URL - Tese da Carolina</t>
+  </si>
+  <si>
+    <t>Alt Text IA 1 Contexto - Tese da Carolina</t>
+  </si>
+  <si>
+    <t>Alt Text 2 URL - BBC</t>
   </si>
   <si>
     <t>Alt Text IA 2 - BBC</t>
   </si>
   <si>
-    <t>Alt Text IA 3 - Section 508</t>
+    <t>Alt Text 3 - Section 508</t>
+  </si>
+  <si>
+    <t>Alt Text 3 URL - Section 508</t>
+  </si>
+  <si>
+    <t>Alt Text IA 3 Contexto - Section 508</t>
   </si>
   <si>
     <t>Governo suspende 3,4 milhões de multas de pedágios 'free flow'; entenda</t>
@@ -89,16 +107,34 @@
   </si>
   <si>
     <t>Contexto: O Ministério dos Transportes suspendeu 3,4 milhões de multas aplicadas por evasão de pedágio no sistema free flow (pedágio eletrônico sem cancelas) em rodovias federais e estaduais. A decisão fundamenta-se na falta de clareza na sinalização dos pórticos e no nome estrangeiro do sistema, o que dificultava a compreensão dos motoristas.</t>
+  </si>
+  <si>
+    <t>URL: https://noticias.uol.com.br/cotidiano/ultimas-noticias/2026/04/28/free-flow-ministerio-dos-transportes.ghtm
+Tipo de Imagem: Imagem Informativa</t>
   </si>
   <si>
     <t xml:space="preserve">Contexto: O Ministério dos Transportes suspendeu 3,4 milhões de multas aplicadas por evasão de pedágio no sistema free flow (pedágio eletrônico sem cancelas) em rodovias federais e estaduais. A decisão fundamenta-se na falta de clareza na sinalização dos pórticos e no nome estrangeiro do sistema, o que dificultava a compreensão dos motoristas.
 Tipo de Imagem: Imagem Informativa </t>
+  </si>
+  <si>
+    <t>Descrição Principal (Simplificada)
+    Fotografia aérea de um pórtico do sistema de pedágio eletrônico Free Flow instalado em uma rodovia movimentada.
+    Uso recomendado: Ideal para o alt text principal (comunicação rápida e direta do fato jornalístico).
+Descrição Detalhada
+    Fotografia aérea e diagonal de um pórtico metálico do sistema de pedágio eletrônico Free Flow, que cruza as faixas de uma rodovia. O pórtico cinza estende-se sobre três faixas de rolagem da esquerda, sustentando sensores, câmeras e uma placa azul retangular com a inscrição "PEDÁGIO ELETRÔNICO" em letras brancas, além de uma placa circular de limite de altura de 5,5 metros. Na coluna direita da estrutura, há uma placa vertical vermelha com o texto "Free Flow Pedágio eletrônico". Sob o pórtico, transitam um caminhão vermelho carregado e uma picape branca. À direita, há uma placa laranja de obras na pista. O plano de fundo mostra o restante da rodovia asfaltada com fluxo de veículos sob a luz do dia, cercada por áreas gramadas e vegetação nas laterais.
+    Uso recomendado: Ideal para recursos de acessibilidade expandidos onde o usuário solicita o detalhamento minucioso da imagem.</t>
   </si>
   <si>
     <t>Opção 1: Texto Alternativo (Principal)
     Pórtico de pedágio eletrônico com câmeras e sensores sobre a rodovia. Acima da pista, uma placa azul indica "Pagamento Eletrônico Automático" com o logotipo de uma antena e ondas de sinal.
 Opção 2: Descrição Longa (Se o portal permitir detalhamento)
     Descrição da imagem: Fotografia em ângulo baixo de um pórtico metálico que atravessa as faixas de uma rodovia. No topo da estrutura, há diversos sensores e câmeras apontados para a pista. Uma placa informativa azul destaca-se com o símbolo de sinal de rádio e o texto informativo sobre o pagamento automático. Ao fundo, o céu está claro e a estrada segue em linha reta.</t>
+  </si>
+  <si>
+    <t>**Opção 1 (Informativa/Principal):**
+Pórtico metálico do sistema de pedágio eletrônico Free Flow instalado sobre as faixas de uma rodovia movimentada, com câmeras e sensores direcionados para a pista onde trafegam carros e caminhões. À direita, uma placa vertical vermelha exibe a inscrição "Free Flow Pedágio eletrônico".
+**Opção 2 (Foco nos elementos de sinalização/texto):**
+Vista aérea de trecho de rodovia com estrutura metálica automatizada de pedágio sem cancelas. No topo do pórtico, há uma placa azul onde se lê "PEDÁGIO ELETRÔNICO" ao lado de uma sinalização de limite de altura de 5,5 metros, com veículos passando por baixo dos sensores.</t>
   </si>
   <si>
     <t>Opção 1: Texto Alternativo Ideal (Foco em Informação e Concisão)
@@ -107,6 +143,20 @@
 Opção 2: Descrição Longa (Se houver campo extra no CMS)
 Caso o nosso sistema permita uma descrição detalhada para complementar o entendimento do contexto de falta de clareza na sinalização:
     Fotografia em plano médio mostra um pórtico metálico cinza instalado sobre as faixas de uma rodovia asfaltada. Na parte superior da estrutura, há cabos, sensores e múltiplas câmeras de monitoramento direcionadas para baixo, capturando o fluxo da pista. Fixadas na coluna direita do pórtico, duas placas azuis de sinalização vertical trazem inscrições em branco: a superior indica "FREE FLOW" com setas apontando para a pista, e a inferior traz o termo "PEDÁGIO AUTOMÁTICO". O dia está ensolarado e o céu, azul claro.</t>
+  </si>
+  <si>
+    <t>Opção 1: Imagem Informativa (Uso Principal)
+Esta opção cumpre a função de transmitir o fato central da notícia e o que está ilustrado, direto ao ponto e respeitando o limite ideal de caracteres para leitores de tela.
+    Texto Alternativo (Alt Text):
+    Carro passa por baixo de pórtico do sistema de pedágio eletrônico Free Flow em rodovia, com câmeras e sensores instalados na estrutura metálica.
+Opção 2: Imagem Decorativa
+Se esta mesma imagem estivesse em um bloco do portal onde o texto ao redor (como a legenda ou o corpo da matéria) já descrevesse exatamente essa cena, ela seria considerada redundante.
+    Código de Acessibilidade:
+    alt="" (Atributo alt vazio, permitindo que o leitor de tela ignore a imagem e evite repetição cansativa para você).
+Opção 3: Descrição Longa (Contexto Ampliado)
+Caso o artigo exija um detalhamento visual maior sobre como funciona a tecnologia mencionada na reportagem:
+    Descrição Detalhada:
+    Imagem em ângulo contra-plongé mostra um veículo utilitário branco trafegando sob um pórtico metálico cinza do sistema Free Flow. A estrutura, instalada sobre as faixas da rodovia, possui diversos dispositivos eletrônicos acoplados, incluindo câmeras de monitoramento, sensores de presença e antenas de leitura de tags, iluminados pela luz do dia.</t>
   </si>
   <si>
     <t>Opção 1: Texto Alternativo Principal (Ideal para o atributo alt do HTML)
@@ -151,14 +201,28 @@
     <t>Contexto: A Lei 15.397/2026, sancionada em maio de 2026, endurece as penas para crimes patrimoniais e digitais no Brasil, elevando a punição mínima do furto de um para seis anos e estabelecendo até dez anos de reclusão para o roubo de celulares e veículos. A legislação também cria o crime de "conta laranja" e amplia as penas para fraudes em redes sociais, visando combater a criminalidade eletrônica e o mercado de receptação. O presidente Lula vetou apenas o aumento de pena para roubo com lesão grave para manter a proporcionalidade jurídica em relação ao crime de homicídio.</t>
   </si>
   <si>
+    <t>URL: https://noticias.uol.com.br/ultimas-noticias/agencia-estado/2026/05/04/lula-sanciona-lei-que-endurece-penas-para-roubo-furto-e-fraudes-digitais.htm
+Tipo de Imagem: Imagem Informativa</t>
+  </si>
+  <si>
     <t>Contexto: A Lei 15.397/2026, sancionada em maio de 2026, endurece as penas para crimes patrimoniais e digitais no Brasil, elevando a punição mínima do furto de um para seis anos e estabelecendo até dez anos de reclusão para o roubo de celulares e veículos. A legislação também cria o crime de "conta laranja" e amplia as penas para fraudes em redes sociais, visando combater a criminalidade eletrônica e o mercado de receptação. O presidente Lula vetou apenas o aumento de pena para roubo com lesão grave para manter a proporcionalidade jurídica em relação ao crime de homicídio.
 Tipo de Imagem: Imagem Informativa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opção 1: Descrição Principal (Ideal para o Alt Text Principal)Fotografia do presidente Luiz Inácio Lula da Silva com expressão reflexiva e séria, com a mão direita tocando sutilmente os lábios. Ao fundo, as cores verde e amarela desfocadas da bandeira do Brasil ambientam o cenário oficial.  Por que essa escolha? Conforme as diretrizes, fomos direto ao ponto sem usar termos redundantes como "foto de". Identificamos o sujeito famoso, sua localização implícita (ambiente oficial), seu comportamento (expressão reflexiva) e a ação corporal sutil.  
+Opção 2: Descrição Detalhada (Para recursos de expansão de tela)Fotografia em plano médio e fechado do presidente Luiz Inácio Lula da Silva, um homem idoso de pele clara, cabelos brancos curtos e barba com bigode também brancos e aparados. Ele está posicionado do peito para cima, ligeiramente voltado para a esquerda. Sua expressão é concentrada e séria, com o olhar direcionado para a lateral. A mão direita está erguida, com os dedos indicador e médio apoiados levemente sobre o lábio inferior e o queixo; na mesma mão, é visível uma aliança dourada no dedo anelar. Lula veste um paletó de terno escuro, camisa social branca e gravata escura com pequenos detalhes discretos. À sua frente, no canto inferior esquerdo, aparece a ponta de um microfone de mesa preto com um detalhe em anel vermelho. O plano de fundo está altamente desfocado, revelando as formas e cores verde, amarela e azul da bandeira nacional.  Por que essa escolha? Esse nível aprofunda as características físicas do sujeito (barba, cabelos, aliança), o vestuário jornalístico formal, elementos periféricos (microfone) e o estilo visual de profundidade de campo (fundo desfocado), respeitando a ordem de varredura visual e a neutralidade interpretativa.  </t>
   </si>
   <si>
     <t>Opção 1: Texto Alternativo (Principal)
     O presidente Lula, um homem branco de barba grisalha usando terno e gravata, assina a nova lei de crimes patrimoniais. Ele está sentado à mesa, sorrindo e segurando uma caneta sobre o documento oficial.
 Opção 2: Descrição Longa (Ideal para detalhamento do cenário)
     Descrição da imagem: Fotografia em plano médio do Presidente da República, Luiz Inácio Lula da Silva, durante a sanção da Lei 15.397/2026. Lula é um homem idoso, branco, de cabelos e barba curta grisalhos. Ele veste terno azul escuro, camisa branca e gravata azul. Está sentado atrás de uma mesa de madeira escura com o brasão da República, segurando uma caneta enquanto assina o documento. Ao fundo, as bandeiras do Brasil e da Presidência estão posicionadas verticalmente. O ambiente é iluminado e formal.</t>
+  </si>
+  <si>
+    <t>Opção 1 (Informativa/Principal):
+O presidente Luiz Inácio Lula da Silva em primeiro plano, com expressão séria e pensativa, tocando os lábios com os dedos da mão direita. Ele usa paletó escuro, camisa branca e gravata escura. Ao fundo, fora de foco, está a bandeira do Brasil.
+Opção 2 (Foco no semblante/Expressão institucional):
+Close-up do presidente Lula vestindo terno e gravata, com olhar direcionado para a esquerda e semblante concentrado, enquanto leva a mão com aliança ao queixo. A bandeira nacional aparece desfocada ao fundo do cenário.</t>
   </si>
   <si>
     <t>Opção 1: Texto Alternativo Ideal (Foco em Informação e Concisão)
@@ -167,6 +231,14 @@
 Opção 2: Descrição Longa (Para maior detalhamento no CMS)
 Ideal se o nosso template exigir uma contextualização visual mais profunda sobre o ambiente institucional onde as decisões de Estado ocorrem.
     Fotografia em plano médio do presidente Luiz Inácio Lula da Silva sentado à sua mesa oficial. Ele é um homem branco de cabelos e barba grisalhos, veste terno escuro, camisa branca e gravata azul-clara. Com uma caneta na mão direita, ele analisa papéis dispostos sobre a mesa de madeira escura, onde também há uma pasta de couro e um notebook fechado. Ao fundo, através de uma parede de vidro, avista-se a arquitetura externa do Palácio da Alvorada e copas de árvores sob iluminação diurna natural.</t>
+  </si>
+  <si>
+    <t>Opção 1: Alt Text Principal (Informativo e Direto)
+Ideal para o campo "alt" padrão da plataforma de notícias, focando no fato jornalístico central logo no início.  Presidente Lula assina documento oficial em uma mesa de madeira. Ele veste terno escuro e gravata, concentrado no ato da sanção presidencial.
+Opção 2: Descrição Longa / Contextualizada
+Indicada se o portal permitir uma descrição mais detalhada no corpo do texto ou via link longdesc, contextualizando o ambiente político e institucional.  Em plano médio, o presidente Luiz Inácio Lula da Silva aparece sentado à mesa presidencial de madeira escura, focado enquanto assina, com uma caneta preta, os papéis da nova lei de segurança digital. Ele usa um terno azul-marinho e gravata cinza. Ao fundo, detalhes discretos do gabinete oficial completam a cena com um tom de formalidade e seriedade.
+Opção 3: Versão Curta / Alternativa (Foco Institucional)
+Uma variação mais sucinta focado estritamente na ação executiva.  Luiz Inácio Lula da Silva assina sanção da nova lei que endurece penas para crimes e fraudes digitais em seu gabinete.</t>
   </si>
   <si>
     <t>Opções de Texto Alternativo (Alt Text)
@@ -305,8 +377,40 @@
     <t>Contexto: A Polícia Civil do Paraná prendeu preventivamente Márcio Talaska, de 38 anos, sob a suspeita de ter provocado a queda de um veículo no Rio Paraná, em Porto Rico, resultando nas mortes de sua esposa, Iria Djanira Ramon Costa Talaska, de 36 anos, e de sua filha, Maria Laura Ramon Talaska, de 3 anos. O incidente ocorreu na noite de 2 de maio de 2026, quando o carro submergiu após descer uma rampa de acesso ao rio; embora o suspeito tenha alegado inicialmente que a esposa conduzia o veículo e se perdera no caminho, investigações baseadas em imagens de câmeras de segurança indicam que era ele quem dirigia desde a saída de uma confraternização familiar até o momento do acidente. O investigado, que foi o único sobrevivente, permanece detido enquanto a defesa aguarda acesso integral aos autos para se manifestar, e o inquérito policial segue para apurar as tipificações de feminicídio e homicídio.</t>
   </si>
   <si>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+        <sz val="11.0"/>
+      </rPr>
+      <t>URL: https://noticias.uol.com.br/cotidiano/ultimas-noticias/2026/05/09/homem-e-preso-sob-suspeita-de-matar-mulher-e-filha-encontradas-em-rio-no-pr.ghtm</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color rgb="FF1155CC"/>
+        <sz val="11.0"/>
+        <u/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+        <sz val="11.0"/>
+      </rPr>
+      <t>Tipo de Imagem: Imagem Informativa</t>
+    </r>
+  </si>
+  <si>
     <t>Contexto: A Polícia Civil do Paraná prendeu preventivamente Márcio Talaska, de 38 anos, sob a suspeita de ter provocado a queda de um veículo no Rio Paraná, em Porto Rico, resultando nas mortes de sua esposa, Iria Djanira Ramon Costa Talaska, de 36 anos, e de sua filha, Maria Laura Ramon Talaska, de 3 anos. O incidente ocorreu na noite de 2 de maio de 2026, quando o carro submergiu após descer uma rampa de acesso ao rio; embora o suspeito tenha alegado inicialmente que a esposa conduzia o veículo e se perdera no caminho, investigações baseadas em imagens de câmeras de segurança indicam que era ele quem dirigia desde a saída de uma confraternização familiar até o momento do acidente. O investigado, que foi o único sobrevivente, permanece detido enquanto a defesa aguarda acesso integral aos autos para se manifestar, e o inquérito policial segue para apurar as tipificações de feminicídio e homicídio.
 Tipo de Imagem: Imagem Informativa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opção 1: Descrição Principal (Texto Alternativo Curto para Leitores de Tela)Fotografia em plano fechado de uma mulher adulta e uma criança pequena sorrindo juntas, com os rostos colados em um momento de carinho.  Por que essa escolha? Conforme as normas, evitamos frases redundantes como "olhando para a câmera" e priorizamos imediatamente a ação central e o sentimento evocado pela imagem (afetividade/sorriso) no início do texto.  
+Opção 2: Descrição Detalhada (Nível Avançado de Acessibilidade)Fotografia em plano médio fechado, em ângulo levemente inclinado, mostrando uma mulher e uma menina em um momento afetuoso. Em primeiro plano, à esquerda, a mulher de pele clara, cabelos longos e castanhos sorri de forma serena. Ela usa um colar fino dourado e brincos pequenos. Atrás dela e ligeiramente à direita, uma criança pequena, de pele clara e cabelos castanhos, sorri abertamente mostrando os dentes. A menina veste um vestido rosa estampado e está com o rosto encostado carinhosamente na bochecha da mulher. O plano de fundo é escuro e indefinido, mantendo o foco inteiramente na expressão de felicidade das duas.  Por que essa escolha? Este nível responde de forma estruturada a perguntas essenciais ("Quem são?", "Como se portam?", "O que fazem?") e adiciona os detalhes físicos detalhados (vestuário, adornos, tom de pele) necessários para criar uma imagem mental fidedigna do arquivo "3.webp" sem misturar opiniões subjetivas.  </t>
   </si>
   <si>
     <t>1. Texto Alternativo (Principal)
@@ -314,6 +418,12 @@
     Por que esta opção? Cumpre a regra de identificação de raça e gênero de forma objetiva, conectando os nomes aos rostos, o que é essencial para a autonomia do leitor em uma notícia de cunho investigativo.
 2. Descrição Longa (Se o sistema permitir um campo longdesc ou legenda expandida)
     Sugestão: Retrato familiar em ambiente externo. À esquerda, Márcio Talaska, homem de pele clara e cabelos castanhos curtos, veste camisa polo escura. No centro, Iria Djanira, mulher de pele clara, cabelos longos e loiros, sorri para a câmera. À direita, a filha do casal, Maria Laura, criança de 3 anos com cabelos loiros. O fundo da imagem está levemente desfocado, sugerindo um momento de confraternização.</t>
+  </si>
+  <si>
+    <t>**Opção 1 (Informativa/Principal):**
+Mulher e sua filha pequena sorriem juntas em uma selfie. A mulher tem cabelos escuros e compridos, e a criança, com cabelos claros, veste um vestido rosa estampado.
+**Opção 2 (Foco no contexto jornalístico/Afeição):**
+Close de uma mulher com cabelos longos e escuros sorrindo ao lado da filha pequena, uma menina que sorri alegremente usando um vestido rosa com estampas. Ambas aparecem unidas e felizes na imagem de arquivo pessoal.</t>
   </si>
   <si>
     <t>Opção 1: Texto Alternativo Ideal (Foco em Informação e Concisão)
@@ -354,9 +464,21 @@
     <t>Contexto: O Ministério da Saúde restabeleceu, em 9 de junho de 2020, a divulgação dos dados acumulados de casos e mortes por covid-19 em seu painel oficial, após uma decisão do Supremo Tribunal Federal (STF) que determinou a retomada da publicidade integral dos indicadores. A plataforma havia sido alterada para exibir apenas registros das últimas 24 horas, o que gerou críticas sobre falta de transparência e possíveis manobras estatísticas. Com a atualização, o portal voltou a consolidar o impacto total da pandemia no país, detalhando números por estados e regiões para facilitar o acompanhamento da curva epidemiológica pela sociedade e órgãos de controle.</t>
   </si>
   <si>
+    <t>URL: https://noticias.uol.com.br/saude/ultimas-noticias/redacao/2020/06/09/covid-19-saude-volta-a-divulgar-numeros-totais-de-casos-e-mortes-em-portal.htm
+Tipo de Imagem: Imagem Complexa</t>
+  </si>
+  <si>
     <t xml:space="preserve">Contexto: O Ministério da Saúde restabeleceu, em 9 de junho de 2020, a divulgação dos dados acumulados de casos e mortes por covid-19 em seu painel oficial, após uma decisão do Supremo Tribunal Federal (STF) que determinou a retomada da publicidade integral dos indicadores. A plataforma havia sido alterada para exibir apenas registros das últimas 24 horas, o que gerou críticas sobre falta de transparência e possíveis manobras estatísticas. Com a atualização, o portal voltou a consolidar o impacto total da pandemia no país, detalhando números por estados e regiões para facilitar o acompanhamento da curva epidemiológica pela sociedade e órgãos de controle.
 Tipo de Imagem: Imagem Complexa
 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opção 1: Descrição Principal (Ideal para o Alt Text Principal)
+Diagrama do Painel Coronavírus do Ministério da Saúde, atualizado em 8 de junho de 2020 às 18h30, exibindo os dados acumulados e novos de casos, óbitos e recuperados da covid-19 no Brasil.  
+Por que essa escolha? Conforme as regras da Seção 7.2 de "2021-tese-diretrizes_alt_text_carolina-dividido_2.pdf", o texto evita termos como "foto de" e indica logo no início a natureza técnica da imagem (Diagrama), seu tema central, os sujeitos institucionais envolvidos e o recorte temporal jornalístico de forma concisa.  
+Opção 2: Descrição Detalhada (Essencial para Imagens Complexas/De Texto)
+Diagrama da interface web intitulada "COVID19 Painel Coronavírus", com a indicação de "Atualizado em: 08/06/2020 18:30". A imagem exibe três blocos principais de cartões informativos lado a lado com os seguintes dados numéricos:  Bloco 1 (Fundo verde com letras brancas): Casos recuperados: 290.040. Em acompanhamento: 380.238.  Bloco 2 (Fundo branco com textos em preto e verde): Título "CASOS CONFIRMADOS". Acumulado: 707.412. Casos novos: 15.654. Incidência: 336,6.  Bloco 3 (Fundo branco com textos em preto e roxo): Título "ÓBITOS CONFIRMADOS". Óbitos acumulados: 37.134. Casos novos: 679. Letalidade: 5,2%. Mortalidade: 17,7.  Na parte inferior da imagem, há o início de uma tabela intitulada "Síntese de casos, óbitos, incidência e mortalidade". A primeira linha da tabela traz os dados consolidados do "Brasil", repetindo os valores de 707.412 casos e 37.134 óbitos.  
+Por que essa escolha? Imagens complexas com dados numéricos e textuais exigem transcrição completa e organização espacial lógica (da esquerda para a direita, de cima para baixo) para que nenhuma informação seja perdida pelo usuário de leitor de telas, conforme instruído na seção de Imagens de Texto e Diagramas da tese.  </t>
   </si>
   <si>
     <t>1. Texto Alternativo (Para leitura rápida)
@@ -376,6 +498,16 @@
     O rodapé indica que os dados foram atualizados às 18:30 do dia 08/06/2020.</t>
   </si>
   <si>
+    <t>Alt text principal (conforme diretrizes do arquivo "BBC GEL _ Complex images.pdf" para síntese de dados complexos):
+Infográfico do Painel Coronavírus do Ministério da Saúde atualizado em 08/06/2020. Exibe três blocos de dados sobre a covid-19 no Brasil: 290.040 casos recuperados e 380.238 em acompanhamento; 707.412 casos confirmados acumulados (15.654 novos); e 37.134 óbitos acumulados (679 novos), com taxa de letalidade em 5,2%.
+Descrição longa (conforme diretrizes do arquivo "BBC GEL _ Complex images.pdf" para fornecer todas as informações disponíveis aos usuários de leitores de tela):
+Captura de tela do Painel Coronavírus no Brasil, atualizado em 08 de junho de 2020 às 18:30. Na parte superior, três cartões principais organizam os indicadores da pandemia:
+    Card verde à esquerda: "Casos recuperados" destaca o número 290.040. Abaixo, "Em acompanhamento" registra 380.238.
+    Card central: "Casos confirmados" mostra 707.412 no acumulado, 15.654 casos novos e o índice de incidência em 336,6.
+    Card à direita: "Óbitos confirmados" apresenta 37.134 óbitos acumulados, 679 casos novos, taxa de letalidade de 5,2% e taxa de mortalidade de 17,7.
+    Na parte inferior, inicia-se uma tabela intitulada "Síntese de casos, óbitos, incidência e mortalidade", replicando a linha de dados totais do Brasil com 707.412 casos e 37.134 óbitos.</t>
+  </si>
+  <si>
     <t>1. Texto Alternativo Principal (Atributo Alt)
 Focado na informação editorial mais importante logo no início, sem usar "foto de" ou "imagem de", mantendo-se conciso.
     Painel interativo do SUS com dados acumulados da Covid-19 no Brasil, registrando 707.412 casos confirmados e 37.134 óbitos acumulados até 9 de junho de 2020.
@@ -421,8 +553,21 @@
     <t>Contexto: O estado de São Paulo abriga a maior população de imigrantes do Brasil, concentrando fluxos históricos e contemporâneos que moldaram sua demografia e economia. Dados oficiais indicam que a capital paulista é o principal destino, recebendo grupos tradicionais como portugueses, italianos e japoneses, além de uma crescente presença de bolivianos, chineses e haitianos. Esse movimento migratório é impulsionado pela oferta de emprego e serviços, embora os novos imigrantes frequentemente enfrentem desafios relacionados à regularização documental e condições de trabalho.</t>
   </si>
   <si>
+    <t>URL: https://noticias.uol.com.br/infograficos/2014/01/21/imigrantes-sp.htm
+Tipo de Imagem: Imagem Complexa</t>
+  </si>
+  <si>
     <t>Contexto: O estado de São Paulo abriga a maior população de imigrantes do Brasil, concentrando fluxos históricos e contemporâneos que moldaram sua demografia e economia. Dados oficiais indicam que a capital paulista é o principal destino, recebendo grupos tradicionais como portugueses, italianos e japoneses, além de uma crescente presença de bolivianos, chineses e haitianos. Esse movimento migratório é impulsionado pela oferta de emprego e serviços, embora os novos imigrantes frequentemente enfrentem desafios relacionados à regularização documental e condições de trabalho.
 Tipo de Imagem: Imagem Complexa</t>
+  </si>
+  <si>
+    <t>Opção 1: Descrição Principal (Texto Alternativo Curto para Leitores de Tela)
+Infográfico com dados estatísticos sobre imigrantes legalizados no Brasil e na cidade de São Paulo, destacando Portugal e Bolívia como as principais nacionalidades da capital paulista.  Por que essa escolha? Iniciamos diretamente especificando o formato relevante para a compreensão da notícia (Infográfico), apontando os sujeitos (imigrantes), a localização geográfica e o fato principal de destaque no topo da hierarquia visual, sem usar termos redundantes.  
+Opção 2: Descrição Detalhada (Nível Avançado de Acessibilidade)
+Infográfico composto por dois gráficos e um texto explicativo sobre o panorama de imigrantes legalizados, com fundo branco e elementos em tons de azul e cinza.  Lado esquerdo - Gráfico de barras verticais: Sob o título "IMIGRANTES LEGALIZADOS - Na cidade de São Paulo, por nacionalidade, em %", o gráfico exibe barras decrescentes representando as seguintes nacionalidades (identificadas por pequenas bandeiras circulares e nomes abaixo de cada barra, ordenadas da esquerda para a direita):  Portugal (a barra mais alta, destacada ao lado com os números acumulados de 368.188 imigrantes e 29.7%);  Bolívia;  Japão;  Itália;  Espanha;  China;  Coreia do Sul;  Argentina;  Chile;  EUA (a menor barra da listagem).  Centro - Bloco de texto informativo:
+"Fundadores da cidade de São Paulo, os portugueses continuaram vindo para a cidade ao longo de cinco séculos, sendo o maior grupo de estrangeiros na capital atualmente".  Lado direito - Gráfico de pizza:
+Sob o título "NO BRASIL", um gráfico circular apresenta o total geral de 1.088.517 imigrantes legalizados, dividido em três fatias de distribuição regional:  51,6% estão no estado de São Paulo (SP);  27% estão distribuídos em Outros estados;  21,4% estão no estado do Rio de Janeiro (RJ).  
+Por que essa escolha? Conforme as regras da Seção 7.2 (Quadro 7 e Tabela 48) para gráficos e diagramas complexos, a descrição decompõe detalhadamente cada elemento informacional de forma sequencial (da esquerda para a direita), transcrevendo todo o texto "queimado" na imagem para assegurar que nenhum dado estatístico seja omitido do leitor de telas.  Se a imagem fosse usada em um contexto puramente estético ou de plano de fundo sem relevância para a matéria (o que não ocorre aqui), a diretriz recomendaria ocultá-la usando o atributo nulo (alt="").</t>
   </si>
   <si>
     <t>1. Texto Alternativo (Para leitura rápida)
@@ -496,8 +641,44 @@
     <t>Contexto: O Zika vírus, a Dengue e a Febre Chikungunya, doenças transmitidas pelo mosquito Aedes aegypti, apresentam quadros clínicos distintos que exigem atenção para o diagnóstico correto: a Dengue caracteriza-se por febre alta súbita e dores musculares intensas; a Chikungunya destaca-se por dores articulares severas e persistentes; e o Zika manifesta-se frequentemente com febre baixa, manchas vermelhas na pele e coceira intensa, possuindo uma associação grave com casos de microcefalia em recém-nascidos e a síndrome de Guillain-Barré. Embora compartilhem sintomas como dor de cabeça e mal-estar, a intensidade e a localização das dores, bem como a presença de conjuntivite (comum no Zika) ou o risco de hemorragias (presente na Dengue), são critérios fundamentais para a diferenciação e para o direcionamento do tratamento adequado, que foca primordialmente no alívio dos sintomas e na hidratação.</t>
   </si>
   <si>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+        <sz val="11.0"/>
+      </rPr>
+      <t>URL: https://noticias.uol.com.br/saude/infograficos/2016/03/16/conhecas-as-diferencas-entre-zika-dengue-e-chikungunya.htm</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color rgb="FF1155CC"/>
+        <sz val="11.0"/>
+        <u/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+        <sz val="11.0"/>
+      </rPr>
+      <t>Tipo de Imagem: Imagem Complexa</t>
+    </r>
+  </si>
+  <si>
     <t>Contexto: O Zika vírus, a Dengue e a Febre Chikungunya, doenças transmitidas pelo mosquito Aedes aegypti, apresentam quadros clínicos distintos que exigem atenção para o diagnóstico correto: a Dengue caracteriza-se por febre alta súbita e dores musculares intensas; a Chikungunya destaca-se por dores articulares severas e persistentes; e o Zika manifesta-se frequentemente com febre baixa, manchas vermelhas na pele e coceira intensa, possuindo uma associação grave com casos de microcefalia em recém-nascidos e a síndrome de Guillain-Barré. Embora compartilhem sintomas como dor de cabeça e mal-estar, a intensidade e a localização das dores, bem como a presença de conjuntivite (comum no Zika) ou o risco de hemorragias (presente na Dengue), são critérios fundamentais para a diferenciação e para o direcionamento do tratamento adequado, que foca primordialmente no alívio dos sintomas e na hidratação.
 Tipo de Imagem: Imagem Complexa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opção 1: Descrição Principal (Ideal para o Alt Text Principal)
+Infográfico comparativo intitulado "É ZIKA, DENGUE OU CHIKUNGUNYA?", ilustrando a intensidade e a localização dos sintomas de cada doença no corpo humano.  
+Por que essa escolha? Conforme as regras da Seção 7.2 de "2021-tese-diretrizes_alt_text_carolina-dividido_4.pdf", o texto evita termos redundantes e indica logo no início a natureza técnica da imagem (Infográfico), seu tema central e o propósito jornalístico de forma concisa.  
+Opção 2: Descrição Detalhada (Essencial para Imagens Complexas/De Texto)
+Infográfico intitulado "É ZIKA, DENGUE OU CHIKUNGUNYA? Sintomas das doenças transmitidas pelo Aedes aegypti são parecidos". A imagem exibe lado a lado três silhuetas do corpo humano masculino, de frente, com manchas e texturas avermelhadas que apontam a localização e a intensidade dos sintomas. Abaixo de cada corpo há a ilustração de um termômetro apontando a temperatura da febre. A organização dos dados da esquerda para a direita é a seguinte:  Silhueta 1 - ZIKA: Apresenta manchas vermelhas espalhadas por todo o corpo. Linhas indicativas apontam para os sintomas de "DOR DE CABEÇA", "VERMELHIDÃO NOS OLHOS" e "MANCHAS VERMELHAS NA PELE". Na base, o termômetro indica "Febre baixa 37,5°". No canto inferior esquerdo há a nota: "*Só 1 em cada 5 infectados tem sintomas".  Silhueta 2 - DENGUE: Apresenta uma mancha vermelha concentrada na cabeça e outra na região do abdômen. Linhas indicativas apontam para "DOR DE CABEÇA", "DOR ATRÁS DO OLHO", "DOR MUSCULAR", "DOR NA BARRIGA E NÁUSEA" e "MANCHAS VERMELHAS NA PELE". Na base, o termômetro indica "Febre muito alta 39°".  Silhueta 3 - CHIKUNGUNYA: Apresenta manchas vermelhas concentradas nas articulações (ombro, cotovelo, pulsos, joelhos e tornozelos). Linhas indicativas apontam para "DOR MUSCULAR", "DORES NAS ARTICULAÇÕES", "MANCHAS VERMELHAS NA PELE" e "INCHAÇO" (com forte sombreado vermelho no tornozelo esquerdo). Na base, o termômetro indica "Febre alta 38,5°".  Legenda inferior central:Um copo de água azul indica "Dificuldade na ingestão de líquidos".  Uma gota de sangue vermelha indica "Possibilidade de hemorragia".  Ao final da imagem, lê-se em texto menor: "Fonte: Hospital São Luiz". 
+Por que essa escolha? Imagens complexas com dados médicos e anatômicos exigem transcrição completa e organização espacial lógica (da esquerda para a direita) para que nenhuma informação ou sintoma comparativo seja perdido pelo usuário de leitor de telas, conforme instruído na seção de Imagens de Texto e Diagramas da tese.  </t>
   </si>
   <si>
     <t>1. Texto Alternativo (Alt principal - Conciso)
@@ -617,8 +798,25 @@
     <t>Contexto: O portal UOL celebrou seu 25º aniversário em 28 de abril de 2021 com o lançamento de uma nova identidade visual e a expansão de sua grade de programação em vídeo e conteúdo digital. A mudança estratégica focou em modernizar a marca e reforçar os pilares de conteúdo, serviços e entretenimento, incluindo a estreia de novos programas com apresentadores renomados e o fortalecimento do Canal UOL. Com a atualização, a empresa buscou consolidar sua liderança no mercado de comunicação brasileiro, destacando sua trajetória iniciada em 1996 e sua evolução tecnológica para atender às novas demandas de consumo de informação.</t>
   </si>
   <si>
+    <t>URL: https://economia.uol.com.br/noticias/redacao/2021/04/28/uol-completa-25-anos-com-nova-marca-e-novidades-na-programacao.htm
+Tipo de Imagem: Imagem de Texto</t>
+  </si>
+  <si>
     <t>Contexto: O portal UOL celebrou seu 25º aniversário em 28 de abril de 2021 com o lançamento de uma nova identidade visual e a expansão de sua grade de programação em vídeo e conteúdo digital. A mudança estratégica focou em modernizar a marca e reforçar os pilares de conteúdo, serviços e entretenimento, incluindo a estreia de novos programas com apresentadores renomados e o fortalecimento do Canal UOL. Com a atualização, a empresa buscou consolidar sua liderança no mercado de comunicação brasileiro, destacando sua trajetória iniciada em 1996 e sua evolução tecnológica para atender às novas demandas de consumo de informação.
 Tipo de Imagem: Imagem de Texto</t>
+  </si>
+  <si>
+    <t>Opção 1: Descrição Principal (Texto Alternativo Curto para Leitores de Tela)
+    Nova identidade visual do UOL com o tradicional elemento circular estilizado em tons de amarelo, laranja e vermelho, seguido pelo nome do portal em letras minúsculas pretas.
+    Por que essa escolha? Seguindo as orientações para o nível principal, evitamos termos redundantes como "Imagem de" e descrevemos diretamente o sujeito da imagem e suas características essenciais para uma leitura rápida no fluxo da notícia.
+Opção 2: Descrição Detalhada (Nível Avançado de Acessibilidade)
+    Logotipo da nova marca do portal UOL centralizado sobre um fundo totalmente branco.
+    A composição visual é dividida em duas partes dispostas horizontalmente:
+        À esquerda: Um símbolo circular composto pela sobreposição de formas translúcidas que criam uma gradação de cores quentes. A parte superior esquerda é amarela, transitando para o laranja no centro e finalizando com uma curva vermelha intensa na base inferior direita.
+        À direita: A palavra "uol" escrita em letras minúsculas com uma tipografia preta, sólida e de traços grossos. As letras estão dispostas de forma compacta e linear.
+    Por que essa escolha? Conforme as regras para Imagens de Texto e logotipos que possuem relevância editorial, o nível detalhado responde às perguntas de estilo visual, disposição espacial (da esquerda para a direita) e paleta de cores. Isso garante que a descrição transmita o conceito de modernização e rejuvenescimento que a matéria jornalística aborda.
+Opção 3: Abordagem Funcional (Se a imagem fosse puramente Decorativa)
+    Caso este logotipo estivesse inserido no topo ou no rodapé do site apenas para marcar o leiaute da página, sem relação direta com o texto da notícia, a diretriz recomendaria ocultá-lo usando o atributo nulo (alt="") para não sobrecarregar sua leitura. Como aqui ele é o fato noticiado, a descrição informativa (Opção 1 ou 2) é obrigatória.</t>
   </si>
   <si>
     <t>1. Texto Alternativo (Principal)
@@ -633,6 +831,12 @@
 2. Variação Funcional (Caso a logo seja usada como botão ou link de navegação)
     Diretriz BBC News para Imagens Funcionais: Se essa imagem for inserida no topo de uma página especial e servir como o link para retornar à home ou à editoria do aniversário, o leitor de tela precisa saber a função do clique, e não a descrição estética.
 Proposta: Página inicial UOL 25 anos.</t>
+  </si>
+  <si>
+    <t>**Texto alternativo principal (Curto):**
+Embalagem de detergente Ypê em close destaca a data de fabricação de fevereiro de 2026 (FAB FEV26) e lote circulados em vermelho, lote este afetado pela suspensão da Anvisa.
+**Descrição longa (Para maior detalhamento do texto contido na imagem):**
+Fotografia em primeiro plano de uma garrafa plástica transparente de detergente líquido Ypê amarelo. Um círculo vermelho destaca as informações impressas no plástico: "FAB FEV26 VAL FEV28", seguido pelo número de lote "L 042101" e o horário "05:14". Ao fundo, de forma desfocada, aparecem outras embalagens de produtos de limpeza da mesma marca.</t>
   </si>
   <si>
     <t>Opções de Texto Alternativo (Alt Text)
@@ -665,8 +869,20 @@
     <t>Contexto: A fabricante de produtos de limpeza Ypê apresentou à Anvisa um plano com 239 medidas corretivas após a suspensão cautelar de diversos lotes de seus produtos por risco de contaminação biológica. As ações detalhadas pela empresa buscam adequar os processos de fabricação e controle de qualidade às normas sanitárias vigentes, visando garantir a segurança dos consumidores e a retomada integral das vendas. A agência reguladora analisa o cronograma de implementação dessas medidas para decidir sobre a liberação definitiva dos itens afetados, enquanto a companhia reforça que as falhas foram pontuais e estão sendo rigorosamente tratadas.</t>
   </si>
   <si>
+    <t>URL: https://www1.folha.uol.com.br/mercado/2026/05/ype-apresenta-239-medidas-de-correcao-apos-suspensao-de-produtos-diz-anvisa.shtml
+Tipo de Imagem: Imagem de Texto</t>
+  </si>
+  <si>
     <t>Contexto: A fabricante de produtos de limpeza Ypê apresentou à Anvisa um plano com 239 medidas corretivas após a suspensão cautelar de diversos lotes de seus produtos por risco de contaminação biológica. As ações detalhadas pela empresa buscam adequar os processos de fabricação e controle de qualidade às normas sanitárias vigentes, visando garantir a segurança dos consumidores e a retomada integral das vendas. A agência reguladora analisa o cronograma de implementação dessas medidas para decidir sobre a liberação definitiva dos itens afetados, enquanto a companhia reforça que as falhas foram pontuais e estão sendo rigorosamente tratadas.
 Tipo de Imagem: Imagem de Texto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opção 1: Descrição Principal (Ideal para o Alt Text Principal)
+Detalhe do lote e da data de fabricação impressos em uma embalagem plástica transparente de detergente Ypê neutro, circulados por uma linha vermelha.
+Opção 2: Descrição Detalhada (Essencial para Imagens de Texto e Informativas)
+Fotografia em plano detalhe que foca na parte inferior do rótulo de uma garrafa plástica transparente de detergente Ypê de cor amarela líquida.  No centro, sobre o plástico transparente abaixo do rótulo impresso, há letras e números gravados diretamente na embalagem. Um círculo vermelho desenhado digitalmente destaca as seguintes informações textuais:  Na primeira linha: "FAB. FEV 26" (indicando a fabricação em fevereiro de 2026).  Na segunda linha: "L 042101" (indicando o número do lote do produto).  À direita, fora do círculo vermelho, constam a validade "VAL. FEV 28" e o horário "05:14". O rótulo amarelo acima exibe selos informativos como "Biodegradável" e "Testado Dermatologicamente". Ao fundo, fora de foco, aparecem outras embalagens de produtos de limpeza da mesma marca.
+Opção 3: Abordagem Funcional (Se a imagem fosse Decorativa)
+Se esta imagem estivesse inserida no portal apenas como uma ilustração genérica de fundo sobre lavagem de louças, sem relação direta com a numeração dos lotes suspensos abordados no texto, a diretriz de tecnologia recomendaria o uso de um atributo nulo (alt=""). Contudo, como ela serve para instruir o consumidor a verificar o lote do produto em sua casa, a descrição textual detalhada das informações impressas é fundamental para manter a utilidade pública da notícia.  </t>
   </si>
   <si>
     <t>1. Texto Alternativo (Principal)
@@ -715,8 +931,21 @@
     <t>Contexto: Mensagens com frases de desânimo e pensamentos suicidas escritas por alunos nas portas dos banheiros de uma escola pública em Recife foram respondidas com palavras de apoio e acolhimento por outros estudantes, gerando uma mobilização positiva que viralizou nas redes sociais. A iniciativa, que transformou um espaço de desabafo silencioso em uma rede de solidariedade, levou a gestão da escola a reforçar o acompanhamento psicológico e as atividades de valorização da vida, destacando a importância da escuta ativa e da empatia no ambiente escolar para a prevenção do autoextermínio entre jovens.</t>
   </si>
   <si>
+    <t>URL: https://noticias.uol.com.br/cotidiano/ultimas-noticias/2019/09/24/mensagens-de-suicidio-em-escola-sao-respondidas-e-imagens-viralizam.htm
+Tipo de Imagem: Imagem de Texto</t>
+  </si>
+  <si>
     <t>Contexto: Mensagens com frases de desânimo e pensamentos suicidas escritas por alunos nas portas dos banheiros de uma escola pública em Recife foram respondidas com palavras de apoio e acolhimento por outros estudantes, gerando uma mobilização positiva que viralizou nas redes sociais. A iniciativa, que transformou um espaço de desabafo silencioso em uma rede de solidariedade, levou a gestão da escola a reforçar o acompanhamento psicológico e as atividades de valorização da vida, destacando a importância da escuta ativa e da empatia no ambiente escolar para a prevenção do autoextermínio entre jovens.
 Tipo de Imagem: Imagem de Texto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opção 1: Descrição Principal (Texto Alternativo Curto para Leitores de Tela)
+Mensagem escrita à mão em um azulejo de banheiro com o desabafo "Se todo mundo desiste de mim pq eu não posso? PORQUE?", seguido da resposta acolhedora "Pq vc é especial pra alguém!" e o desenho de um coração vermelho.  Por que essa escolha? 
+Conforme as diretrizes para o nível principal, evitamos termos redundantes como "Imagem de" e fornecemos os dados textuais essenciais imediatamente, inserindo o usuário diretamente no contexto central da matéria.  
+Opção 2: Descrição Detalhada (Nível Avançado de Acessibilidade)
+Fotografia em plano médio focada em um azulejo quadrado branco de uma parede de banheiro. No azulejo central, há uma interação escrita à mão com caneta hidrográfica que simula uma conversa:  Pergunta inicial (em letras menores): "SE TODO MUNDO DESISTE DE MIM PQ EU NÃO POSSO?"  Palavra de questionamento (em letras maiúsculas, grossas e sublinhadas): "PORQUE?"  Resposta (escrita logo abaixo, por outra caligrafia): "PQ VC É ESPECIAL PRA ALGUÉM!"  Logo abaixo da resposta, há o desenho de um coração pintado de vermelho, cercado por pequenos traços pretos que simulam feixes de luz ou pulsação. Os azulejos ao redor estão limpos e sem marcas.  
+Por que essa escolha? Para Imagens de Texto com forte carga editorial, o nível detalhado responde às perguntas de estilo visual, disposição espacial (de cima para baixo) e elementos gráficos adjacentes (como o coração pulsante). Isso garante que o usuário compreenda tanto o impacto verbal quanto a sensibilidade estética do ato retratado. 
+Opção 3: Abordagem Funcional (Se a imagem fosse puramente Decorativa)Caso essa imagem estivesse inserida em um artigo genérico sobre arquitetura escolar ou azulejos, sem relevância para o texto, a recomendação seria ocultá-la usando o atributo nulo (alt=""). Contudo, por se tratar do elemento principal que dá sentido e materialidade à reportagem, a descrição detalhada é indispensável.  </t>
   </si>
   <si>
     <t>1. Texto Alternativo (Alt principal - Focado no fato)
@@ -758,8 +987,22 @@
     <t>Contexto: O concurso 3006 da Mega-Sena, sorteado em 9 de maio de 2026 pelas Loterias Caixa, apresentou um prêmio acumulado estimado em R$ 45 milhões devido à ausência de ganhadores na faixa principal do sorteio anterior. As apostas para o certame, que possui valor mínimo de R$ 6 para seis dezenas, foram encerradas às 19h do dia do sorteio, com a divulgação oficial dos números realizada às 21h via canais digitais da instituição. O evento mobilizou apostadores em todo o país através de casas lotéricas e plataformas online, mantendo as opções de apostas automáticas e repetidas para os participantes que buscavam o prêmio milionário.</t>
   </si>
   <si>
+    <t>URL: https://economiareal.uol.com.br/noticia/loterias/resultado-da-mega-sena-3006-veja-os-numeros-sorteados-e-se-voce-ganhou-1784?utm_source=Feed%20UOL&amp;utm_medium=site&amp;xid=0700
+Tipo de Imagem: Imagem Decorativa</t>
+  </si>
+  <si>
     <t>Contexto: O concurso 3006 da Mega-Sena, sorteado em 9 de maio de 2026 pelas Loterias Caixa, apresentou um prêmio acumulado estimado em R$ 45 milhões devido à ausência de ganhadores na faixa principal do sorteio anterior. As apostas para o certame, que possui valor mínimo de R$ 6 para seis dezenas, foram encerradas às 19h do dia do sorteio, com a divulgação oficial dos números realizada às 21h via canais digitais da instituição. O evento mobilizou apostadores em todo o país através de casas lotéricas e plataformas online, mantendo as opções de apostas automáticas e repetidas para os participantes que buscavam o prêmio milionário.
 Tipo de Imagem: Imagem Decorativa</t>
+  </si>
+  <si>
+    <t>Opção 1: Tratamento Funcional Padrão (Recomendado para o Contexto)
+    Se a imagem cumpre uma função puramente estética ou ilustrativa no topo da página de resultados (sendo redundante ao texto que já traz as dezenas sorteadas), a melhor prática técnica é ocultá-la dos leitores de tela. Isso evita o excesso de informações repetitivas e agiliza sua leitura.
+        Código técnico: alt="" (Atributo alt vazio, fazendo com que o leitor de tela passe direto pela imagem).
+Opção 2: Descrição Principal (Caso mude a função para Informativa)
+    Vários bilhetes de apostas da Mega-Sena sobrepostos, com uma caneta esferográfica preta assinalando alguns números nos quadrantes de jogo.
+    Por que essa escolha? Caso o portal decida que a imagem precisa ser lida, este texto vai direto ao ponto em menos de 150 caracteres. Evitamos termos óbvios como "Foto de" e destacamos os elementos centrais: os volantes do jogo e o ato de apostar.
+Opção 3: Descrição Detalhada (Acessibilidade Avançada)
+    Em primeiro plano e ligeiramente inclinada, a ponta de uma caneta esferográfica de corpo transparente aponta para um bilhete de apostas oficial da Mega-Sena. No papel, algumas dezenas estão marcadas com pequenos traços pretos feitos à caneta. Ao fundo, em desalinho, aparecem partes de outros volantes de apostas idênticos. O design dos bilhetes destaca o logotipo verde e dourado da "Mega-Sena", acompanhado de um trevo de quatro folhas e tabelas numéricas que vão do 01 ao 60 em tom amarelo-claro.</t>
   </si>
   <si>
     <t>1. Texto Alternativo (Principal)
@@ -794,8 +1037,22 @@
     <t>Contexto: O consumo diário de cerveja, mesmo em quantidades moderadas, desencadeia uma série de efeitos sistêmicos que vão além dos danos hepáticos tradicionais, afetando órgãos como o cérebro, os rins e o sistema digestivo. De acordo com especialistas e estudos recentes, a ingestão frequente compromete a microbiota intestinal e prejudica a absorção de nutrientes essenciais, como o magnésio e as vitaminas do complexo B, além de causar uma sobrecarga renal devido ao efeito diurético do álcool, que pode levar à desidratação crônica. No campo neurológico, o hábito está associado à redução da densidade cerebral e à lentidão dos reflexos a longo prazo, enquanto no sistema cardiovascular pode contribuir para o aumento da pressão arterial e da gordura visceral. Embora a bebida possua compostos antioxidantes, a comunidade médica ressalta que os riscos inflamatórios e a toxicidade do álcool para as células superam eventuais benefícios, recomendando intervalos de pelo menos 48 horas sem consumo para permitir a regeneração dos tecidos e a desintoxicação do organismo.</t>
   </si>
   <si>
+    <t>URL: https://www.uol.com.br/vivabem/noticias/redacao/2026/05/12/impacto-alem-do-figado-o-que-uma-cerveja-por-dia-faz-com-seu-corpo.htm
+Tipo de Imagem: Imagem Decorativa</t>
+  </si>
+  <si>
     <t>Contexto: O consumo diário de cerveja, mesmo em quantidades moderadas, desencadeia uma série de efeitos sistêmicos que vão além dos danos hepáticos tradicionais, afetando órgãos como o cérebro, os rins e o sistema digestivo. De acordo com especialistas e estudos recentes, a ingestão frequente compromete a microbiota intestinal e prejudica a absorção de nutrientes essenciais, como o magnésio e as vitaminas do complexo B, além de causar uma sobrecarga renal devido ao efeito diurético do álcool, que pode levar à desidratação crônica. No campo neurológico, o hábito está associado à redução da densidade cerebral e à lentidão dos reflexos a longo prazo, enquanto no sistema cardiovascular pode contribuir para o aumento da pressão arterial e da gordura visceral. Embora a bebida possua compostos antioxidantes, a comunidade médica ressalta que os riscos inflamatórios e a toxicidade do álcool para as células superam eventuais benefícios, recomendando intervalos de pelo menos 48 horas sem consumo para permitir a regeneração dos tecidos e a desintoxicação do organismo.
 Tipo de Imagem: Imagem Decorativa</t>
+  </si>
+  <si>
+    <t>Opção 1: Tratamento Funcional Padrão (Recomendado para Imagem Decorativa)
+    Quando uma imagem tem função puramente estética ou ilustrativa — servindo apenas para preencher espaço visual sem acrescentar dados novos ao texto da notícia —, a diretriz técnica ideal de acessibilidade web é ocultá-la dos leitores de tela para tornar a sua navegação mais ágil e fluida.
+        Código técnico: alt="" (Atributo alt vazio, fazendo com que o leitor de tela ignore a imagem de forma limpa).
+Opção 2: Descrição Principal (Caso mude a função para Informativa)
+    Homem de camiseta cinza segura um copo de cerveja com espuma e olha para ele com expressão reflexiva e séria.
+    Por que essa escolha? Caso o editor opte por torná-la informativa, este texto vai direto ao ponto em menos de 120 caracteres, destacando o sujeito, o objeto central e o sentimento de dúvida/reflexão que conversa diretamente com o tema da matéria ("o que a cerveja faz com seu corpo").
+Opção 3: Descrição Detalhada (Acessibilidade Avançada)
+    Homem de pele clara, cabelos escuros e barba curta grisalha, vestindo camiseta cinza de mangas curtas. Ele está com a mão direita sob o queixo e o olhar direcionado para baixo, observando com semblante pensativo o copo de vidro americano cheio de cerveja clara e com colarinho de espuma branca que segura com a mão esquerda. O fundo da imagem é uma parede lisa em tom claro e neutro.</t>
   </si>
   <si>
     <t>1. Texto Alternativo (Principal)
@@ -830,8 +1087,22 @@
     <t>Contexto: A decisão do governo brasileiro de extinguir o imposto federal de 20% sobre compras internacionais de até US$ 50, popularmente conhecida como "taxa das blusinhas", coloca o país em uma direção oposta às recentes políticas adotadas por grandes economias globais, como os Estados Unidos e a União Europeia. Enquanto o Brasil justifica a medida como uma forma de beneficiar o consumo popular e regularizar o setor após o combate ao contrabando, os EUA implementaram tarifas de 30% ou um valor fixo de US$ 25 por item em remessas de baixo valor, e a União Europeia prepara-se para introduzir, em julho, uma taxa adicional de 3 euros para encomendas de até 150 euros, visando proteger indústrias locais e trabalhadores diante da expansão das plataformas de e-commerce estrangeiras. Por outro lado, a Argentina de Javier Milei segue uma linha similar à brasileira, tendo ampliado significativamente os limites de isenção para importações para fomentar a competitividade de preços, evidenciando uma divergência de estratégias econômicas entre o protecionismo de blocos desenvolvidos e a abertura comercial em determinados mercados sul-americanos.</t>
   </si>
   <si>
+    <t>URL: https://economia.uol.com.br/noticias/redacao/2026/05/15/taxa-das-blusinhas---internacional.ghtm
+Tipo de Imagem: Imagem Decorativa</t>
+  </si>
+  <si>
     <t>Contexto: A decisão do governo brasileiro de extinguir o imposto federal de 20% sobre compras internacionais de até US$ 50, popularmente conhecida como "taxa das blusinhas", coloca o país em uma direção oposta às recentes políticas adotadas por grandes economias globais, como os Estados Unidos e a União Europeia. Enquanto o Brasil justifica a medida como uma forma de beneficiar o consumo popular e regularizar o setor após o combate ao contrabando, os EUA implementaram tarifas de 30% ou um valor fixo de US$ 25 por item em remessas de baixo valor, e a União Europeia prepara-se para introduzir, em julho, uma taxa adicional de 3 euros para encomendas de até 150 euros, visando proteger indústrias locais e trabalhadores diante da expansão das plataformas de e-commerce estrangeiras. Por outro lado, a Argentina de Javier Milei segue uma linha similar à brasileira, tendo ampliado significativamente os limites de isenção para importações para fomentar a competitividade de preços, evidenciando uma divergência de estratégias econômicas entre o protecionismo de blocos desenvolvidos e a abertura comercial em determinados mercados sul-americanos.
 Tipo de Imagem: Imagem Decorativa</t>
+  </si>
+  <si>
+    <t>Opção 1: Tratamento Funcional Padrão (Recomendado para Imagem Decorativa)
+    Quando uma imagem tem função puramente estética ou ilustrativa — servindo para preencher espaço visual sem acrescentar dados inéditos ou cruciais ao texto da notícia —, a diretriz técnica ideal de acessibilidade web é ocultá-la dos leitores de tela. Isso evita redundâncias e torna a sua leitura do artigo mais ágil e focada no texto jornalístico.
+        Código técnico: alt="" (Atributo alt vazio, fazendo com que o leitor de tela ignore a imagem de forma limpa).
+Opção 2: Descrição Principal (Caso mude a função para Informativa)
+    Pessoa segura um cartão de crédito azul enquanto digita em um celular, com um notebook aberto ao fundo sobre a mesa.
+    Por que essa escolha? Caso o editor do portal decida que a imagem deve contextualizar visualmente o consumo e as compras em sites internacionais, este texto vai direto ao ponto em 121 caracteres, destacando as ferramentas da ação (cartão, smartphone e computador) sem rodeios ou termos redundantes.
+Opção 3: Descrição Detalhada (Acessibilidade Avançada)
+    Em primeiro plano e em foco, as mãos de uma pessoa realizam uma compra online. A mão direita segura um smartphone moderno que exibe um aplicativo com interface de pagamento, onde o polegar toca a tela. Ao fundo, ligeiramente desfocada, a outra mão segura um cartão de crédito de cor azul com uma faixa magnética escura. Um notebook cinza aberto está sobre a mesa de madeira, completando o cenário de comércio eletrônico.</t>
   </si>
   <si>
     <t>Opção 1: Texto Alternativo Curto (Recomendado para Imagem Informativa/Ilustrativa)
@@ -874,8 +1145,19 @@
     <t>Contexto: O presidente da Rússia, Vladimir Putin, declarou em 9 de maio de 2026 que o conflito com a Ucrânia está "chegando ao fim", ressaltando que, embora agradeça as mediações internacionais, o acordo final diz respeito apenas às duas nações envolvidas. A afirmação ocorreu no contexto do Dia da Vitória, durante o qual um cessar-fogo de três dias foi mediado pelo presidente dos Estados Unidos, Donald Trump, incluindo uma troca de 1.000 prisioneiros e sinais de que o presidente ucraniano, Volodymyr Zelensky, estaria disposto a um encontro pessoal. Apesar do tom otimista sobre o encerramento das hostilidades, Putin utilizou seu discurso oficial para reforçar as justificativas da "operação militar especial", criticando a agressividade da Otan e mantendo a exigência de que qualquer encontro bilateral ocorra somente após a formalização de um "acordo de paz duradouro".</t>
   </si>
   <si>
+    <t>URL: https://g1.globo.com/mundo/noticia/2026/05/09/putin-russia-ucrania.ghtml
+Tipo de Imagem: Imagem Informativa</t>
+  </si>
+  <si>
     <t>Contexto: O presidente da Rússia, Vladimir Putin, declarou em 9 de maio de 2026 que o conflito com a Ucrânia está "chegando ao fim", ressaltando que, embora agradeça as mediações internacionais, o acordo final diz respeito apenas às duas nações envolvidas. A afirmação ocorreu no contexto do Dia da Vitória, durante o qual um cessar-fogo de três dias foi mediado pelo presidente dos Estados Unidos, Donald Trump, incluindo uma troca de 1.000 prisioneiros e sinais de que o presidente ucraniano, Volodymyr Zelensky, estaria disposto a um encontro pessoal. Apesar do tom otimista sobre o encerramento das hostilidades, Putin utilizou seu discurso oficial para reforçar as justificativas da "operação militar especial", criticando a agressividade da Otan e mantendo a exigência de que qualquer encontro bilateral ocorra somente após a formalização de um "acordo de paz duradouro".
 Tipo de Imagem: Imagem Informativa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opção 1: Texto Alternativo Principal (Ideal para o atributo alt do leitor de tela)
+Vladimir Putin, presidente da Rússia, sentado à mesa com semblante sério e focado, segura uma caneta sobre papéis oficiais.
+Por que essa escolha? Conforme os critérios jornalísticos e de acessibilidade, este texto vai direto ao ponto em 121 caracteres. Ele prioriza o sujeito central da notícia (o líder russo), a ação relevante (despachando/assinando documentos) e a sua expressão, contextualizando perfeitamente o tom de seriedade da reportagem sem o uso de termos redundantes como "foto de".  
+Opção 2: Descrição Detalhada (Acessibilidade Avançada / longdesc)
+Fotografia em plano médio do presidente russo Vladimir Putin. Homem de pele clara, cabelos claros e ralos, veste terno escuro, camisa social branca e gravata estampada em tons de roxo e cinza. Ele está sentado atrás de uma longa mesa de tom bege claro. Com o corpo ligeiramente inclinado para a frente, ele apoia a mão esquerda sobre um bloco de papéis impressos e, com a mão direita, segura uma caneta escura, simulando o ato de escrever ou assinar os documentos. Sua expressão facial é séria, concentrada e com o olhar direcionado para o lado esquerdo. Ele está acomodado em uma cadeira presidencial de espaldar alto, estofada em tecido adamascado claro com detalhes em madeira escura e ornamentos dourados no topo. Ao fundo, à esquerda, observa-se parte de uma bandeira com faixas verticais nas cores vermelha e azul.  </t>
   </si>
   <si>
     <t>Opção 1: Texto Alternativo Principal (Ideal para o campo alt)
@@ -913,8 +1195,18 @@
     <t>Contexto: O resgate do cavalo Caramelo completou dois anos, consolidando o animal como um símbolo de resiliência da histórica enchente de maio de 2024 no Rio Grande do Sul. Flagrado pelo Globocop ilhado sobre o telhado de uma casa em Canoas, o equino passou quatro dias sem água ou comida até ser retirado em uma complexa operação interestadual conduzida pelo Corpo de Bombeiros de São Paulo, que envolveu sedação e transporte por bote. Atualmente, Caramelo vive sob os cuidados da Universidade Luterana do Brasil (Ulbra), onde recuperou cerca de 100 kg, tornou-se uma figura pública com agenda de eventos e visitas controladas, demonstrando plena recuperação física e ausência de traumas psicológicos severos, apesar da gravidade da situação em que foi encontrado.</t>
   </si>
   <si>
+    <t>URL: https://g1.globo.com/rs/rio-grande-do-sul/noticia/2026/05/09/ha-dois-anos-cavalo-caramelo-era-resgatado-de-enchente-no-rs-em-operacao-interestadual-acompanhada-em-tempo-real-relembre.ghtml
+Tipo de Imagem: Imagem Informativa</t>
+  </si>
+  <si>
     <t>Contexto: O resgate do cavalo Caramelo completou dois anos, consolidando o animal como um símbolo de resiliência da histórica enchente de maio de 2024 no Rio Grande do Sul. Flagrado pelo Globocop ilhado sobre o telhado de uma casa em Canoas, o equino passou quatro dias sem água ou comida até ser retirado em uma complexa operação interestadual conduzida pelo Corpo de Bombeiros de São Paulo, que envolveu sedação e transporte por bote. Atualmente, Caramelo vive sob os cuidados da Universidade Luterana do Brasil (Ulbra), onde recuperou cerca de 100 kg, tornou-se uma figura pública com agenda de eventos e visitas controladas, demonstrando plena recuperação física e ausência de traumas psicológicos severos, apesar da gravidade da situação em que foi encontrado.
 Tipo de Imagem: Imagem Informativa</t>
+  </si>
+  <si>
+    <t>Opção 1: Descrição Principal (Ideal para o Alt Text principal)
+    Cavalo Caramelo visto de perfil, olhando para a direita. Ele tem pelagem marrom, uma mancha branca na testa e usa um cabresto claro com seu nome gravado. Ao fundo, uma área externa ensolarada e desfocada.
+Opção 2: Descrição Detalhada (Para recursos de acessibilidade expandidos)
+    Fotografia em plano médio do cavalo Caramelo, o famoso equino resgatado nas enchentes do Rio Grande Sul. O animal possui pelagem marrom-escura brilhante e uma crina de tom caramelo mais claro que cai pelo pescoço. Ele está de perfil, voltado para a direita da imagem, exibindo uma marcação branca vertical e irregular que desce da testa até o focinho. Ele usa um cabresto de fita clara onde se lê a inscrição "ULBRA" de um lado e "CARAMELO" na focinheira. O fundo da foto está desfocado, revelando uma área verde com árvores, um lago e a fachada de um prédio de tijolos sob a luz natural do dia.</t>
   </si>
   <si>
     <t>Opção 1: Texto Alternativo Principal (Ideal para o campo alt)
@@ -957,8 +1249,18 @@
     <t>Contexto: Tiago Cheregatte Neves, ex-namorado de Elize Matsunaga, morreu no dia 5 de maio de 2026 após ser atropelado por diversos veículos na Rodovia Padre Manoel da Nóbrega, em São Vicente, no litoral paulista. De acordo com o boletim de ocorrência divulgado nesta quarta-feira (13), Tiago, que era um homem trans e cumpria pena por tentativa de homicídio contra o avô, foi atingido inicialmente por um carro que não conseguiu desviar a tempo, sendo posteriormente atropelado por outros automóveis e por uma viatura da Polícia Militar que passava pelo local. O casal se conheceu na Penitenciária de Tremembé, onde Tiago era custodiado na ala feminina por questões de segurança, mas o relacionamento havia terminado antes de Elize progredir para o regime aberto. As autoridades realizaram testes de bafômetro nos condutores envolvidos, com resultados negativos, e o caso segue sob investigação para esclarecer a dinâmica exata do acidente.</t>
   </si>
   <si>
+    <t>URL: https://g1.globo.com/sp/santos-regiao/noticia/2026/05/13/ex-de-elize-matsunaga-morre-atropelado-em-rodovia-de-sp.ghtml
+Tipo de Imagem: Imagem Informativa</t>
+  </si>
+  <si>
     <t>Contexto: Tiago Cheregatte Neves, ex-namorado de Elize Matsunaga, morreu no dia 5 de maio de 2026 após ser atropelado por diversos veículos na Rodovia Padre Manoel da Nóbrega, em São Vicente, no litoral paulista. De acordo com o boletim de ocorrência divulgado nesta quarta-feira (13), Tiago, que era um homem trans e cumpria pena por tentativa de homicídio contra o avô, foi atingido inicialmente por um carro que não conseguiu desviar a tempo, sendo posteriormente atropelado por outros automóveis e por uma viatura da Polícia Militar que passava pelo local. O casal se conheceu na Penitenciária de Tremembé, onde Tiago era custodiado na ala feminina por questões de segurança, mas o relacionamento havia terminado antes de Elize progredir para o regime aberto. As autoridades realizaram testes de bafômetro nos condutores envolvidos, com resultados negativos, e o caso segue sob investigação para esclarecer a dinâmica exata do acidente.
 Tipo de Imagem: Imagem Informativa</t>
+  </si>
+  <si>
+    <t>Opção 1: Descrição Principal (Concisa e direta ao assunto)
+    Montagem fotográfica lado a lado de Elize Matsunaga, sorrindo dentro de um veículo, e de seu ex-companheiro Tiago Medeiros, usando máscara branca e casaco vermelho.
+Opção 2: Descrição Detalhada (Nível aprofundado de conteúdo)
+    Imagem composta por duas fotografias lado a lado. À esquerda, Elize Matsunaga é retratada do peito para cima, sentada no interior de um veículo com fundo escuro. Ela tem pele clara, cabelos loiros, sorri olhando para a direita e veste um blazer cinza listrado. À direita, Tiago Medeiros é mostrado de perfil parcial, caminhando ao ar livre. Ele tem pele clara, cabelos escuros e curtos, usa uma máscara de proteção facial branca e um casaco de moletom vermelho aberto com capuz sobre uma camiseta preta. Uma tatuagem é visível em seu peito e em sua mão direita, que segura papéis brancos.</t>
   </si>
   <si>
     <t>Opção 1: Texto Alternativo Principal (Ideal para o campo alt)
@@ -999,8 +1301,22 @@
     <t>Contexto: Cerca de 40% das mulheres que realizaram aborto legal no Brasil entre janeiro de 2021 e fevereiro de 2022 precisaram se deslocar de seus municípios de residência para acessar o procedimento, com casos de pacientes percorrendo distâncias superiores a mil quilômetros devido à escassez de serviços especializados. Levantamento realizado pelo g1 aponta que, dos 1.823 procedimentos autorizados por lei no período, 711 ocorreram em cidades distintas da moradia das gestantes, evidenciando barreiras geográficas e estruturais que afetam principalmente as populações mais vulneráveis. Especialistas alertam que a falta de oferta do serviço em 96% dos municípios brasileiros, somada à burocracia hospitalar indevida — como a exigência de boletim de ocorrência em casos de estupro — e à "objeção de consciência" de profissionais de saúde, resulta em uma revitimização das mulheres, atrasando interrupções gestacionais que se tornam tecnicamente mais complexas e emocionalmente desgastantes à medida que as semanas avançam.</t>
   </si>
   <si>
+    <t>URL: https://g1.globo.com/sp/sao-paulo/noticia/2022/06/09/4-em-cada-10-abortos-legais-no-brasil-sao-feitos-fora-da-cidade-onde-a-mulher-mora-pacientes-percorreram-mais-de-1-mil-km.ghtml
+Tipo de Imagem: Imagem Complexa</t>
+  </si>
+  <si>
     <t>Contexto: Cerca de 40% das mulheres que realizaram aborto legal no Brasil entre janeiro de 2021 e fevereiro de 2022 precisaram se deslocar de seus municípios de residência para acessar o procedimento, com casos de pacientes percorrendo distâncias superiores a mil quilômetros devido à escassez de serviços especializados. Levantamento realizado pelo g1 aponta que, dos 1.823 procedimentos autorizados por lei no período, 711 ocorreram em cidades distintas da moradia das gestantes, evidenciando barreiras geográficas e estruturais que afetam principalmente as populações mais vulneráveis. Especialistas alertam que a falta de oferta do serviço em 96% dos municípios brasileiros, somada à burocracia hospitalar indevida — como a exigência de boletim de ocorrência em casos de estupro — e à "objeção de consciência" de profissionais de saúde, resulta em uma revitimização das mulheres, atrasando interrupções gestacionais que se tornam tecnicamente mais complexas e emocionalmente desgastantes à medida que as semanas avançam.
 Tipo de Imagem: Imagem Complexa</t>
+  </si>
+  <si>
+    <t>Opção 1: Descrição Principal (Ideal para o Alt Text básico)
+    Infográfico "O preço do deslocamento" mostra que o trajeto de 833 km entre Santa Maria das Barreiras e Belém custa 430 reais de ônibus.
+Opção 2: Descrição Detalhada (Aprofundada, transcrevendo os dados essenciais)
+    Infográfico intitulado "O preço do deslocamento. Trajeto entre Santa Maria das Barreiras e Belém pode custar R$ 430".
+    Na parte superior, há uma legenda indicando "Trajeto de carro" em azul e "Trajeto de ônibus" em vermelho.
+    O corpo da imagem apresenta o mapa do estado do Pará com uma rota vermelha destacada. O trajeto começa no sul do estado, em Santa Maria das Barreiras, passa por Redenção e Conceição do Araguaia, e segue em linha contínua até Belém, no norte, totalizando uma distância indicada de "833,25 km".
+    À esquerda, um balão informativo de destaque emoldurado em vermelho traz o texto: "Valor aproximado da passagem ida e volta R$ 430". Ao lado do valor, um gráfico de pizza simplificado aponta o percentual de "35,5% do valor atual do salário mínimo (R$ 1.212)".
+    No canto inferior esquerdo, há um pequeno mapa da América do Sul destacando a localização do Pará em vermelho. No rodapé, constam a assinatura do portal G1 e a fonte: "Levantamento feito pelo g1 no Ministério da Saúde, por meio da Lei de Acesso à Informação (LAI), de janeiro de 2021 ao fim de janeiro de 2022. Infográfico elaborado em: 05/05/2022".</t>
   </si>
   <si>
     <t>1. Texto Alternativo Principal (Para o campo alt do CMS)
@@ -1054,8 +1370,32 @@
     <t>Contexto: O especial do g1 Sul de Minas, publicado em comemoração aos 30 anos do "Caso ET de Varginha" em 2026, reconstrói a cronologia dos eventos de 1996 por meio de um infográfico baseado em registros da época, relatos de testemunhas e dossiês ufológicos. O marco inicial remonta a janeiro de 1996, quando as irmãs Liliane e Valquíria Silva, acompanhadas da amiga Kátia Xavier, relataram ter avistado uma criatura marrom, de pele oleosa e olhos vermelhos em um terreno baldio, narrativa que sustentam sem alterações até hoje. A linha do tempo destaca momentos críticos, como a suposta captura de seres por militares e bombeiros, a movimentação atípica em hospitais locais e a morte misteriosa do policial Marco Eli Chereze, atribuída por ufólogos ao contato com a criatura. Três décadas depois, o caso ganha novas camadas com depoimentos inéditos de médicos que afirmam ter presenciado procedimentos em seres não humanos e o lançamento de uma série documental no Globoplay, reforçando o impacto cultural do episódio que transformou a identidade da cidade mineira e permanece como um dos maiores mistérios da ufologia mundial.</t>
   </si>
   <si>
+    <t>URL: https://g1.globo.com/mg/sul-de-minas/noticia/2026/01/20/infografico-veja-a-linha-do-tempo-do-caso-et-de-varginha-que-completa-30-anos.ghtml
+Tipo de Imagem: Imagem Complexa</t>
+  </si>
+  <si>
     <t>Contexto: O especial do g1 Sul de Minas, publicado em comemoração aos 30 anos do "Caso ET de Varginha" em 2026, reconstrói a cronologia dos eventos de 1996 por meio de um infográfico baseado em registros da época, relatos de testemunhas e dossiês ufológicos. O marco inicial remonta a janeiro de 1996, quando as irmãs Liliane e Valquíria Silva, acompanhadas da amiga Kátia Xavier, relataram ter avistado uma criatura marrom, de pele oleosa e olhos vermelhos em um terreno baldio, narrativa que sustentam sem alterações até hoje. A linha do tempo destaca momentos críticos, como a suposta captura de seres por militares e bombeiros, a movimentação atípica em hospitais locais e a morte misteriosa do policial Marco Eli Chereze, atribuída por ufólogos ao contato com a criatura. Três décadas depois, o caso ganha novas camadas com depoimentos inéditos de médicos que afirmam ter presenciado procedimentos em seres não humanos e o lançamento de uma série documental no Globoplay, reforçando o impacto cultural do episódio que transformou a identidade da cidade mineira e permanece como um dos maiores mistérios da ufologia mundial.
 Tipo de Imagem: Imagem Complexa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opção 1: Descrição Principal (Concisa, focada no objetivo da imagem)
+    Infográfico com a linha do tempo dos principais relatos e fotos do caso ET de Varginha em 1996, detalhando os acontecimentos cronológicos dos dias 13, 20 e 21 de janeiro, além de desdobramentos posteriores.
+Opção 2: Descrição Detalhada (Aprofundada, transcrevendo a estrutura e dados textuais)
+    Infográfico vertical intitulado "30 anos do caso ET de Varginha - Veja os principais relatos e fotos do caso em 1996". O conteúdo é estruturado como uma linha do tempo vertical com marcadores vermelhos contendo datas e horários, acompanhados de blocos de texto e ilustrações em círculos ou retângulos:
+        Fim de tarde - 13/01/1996: Texto relata que moradores alegam ter visto uma espaçonave com problemas sobrevoando Varginha. Uma ilustração mostra um objeto cilíndrico marrom soltando fumaça sobre um campo.
+        Madrugada - 01:00: O piloto Carlos de Souza relata ter visto um objeto cortando o céu de forma irregular. Há uma foto recortada em círculo do piloto e uma ilustração de uma criatura marrom.
+        Manhã - 08:30: Texto indica que bombeiros capturaram uma criatura estranha que foi levada para o Hospital Regional. Duas ilustrações mostram militares capturando um ser em uma rede e descendo uma encosta.
+        Tarde - 13:00: Relato de uma criatura vista no Jardim Andere por três garotas. Uma ilustração em círculo mostra as testemunhas de costas observando uma figura agachada junto a um muro.
+        Fim de tarde - 15:30: Telefonemas afirmam que civis e militares avistaram uma criatura. Uma foto em preto e branco mostra as três garotas sentadas em um sofá e, ao lado, uma ilustração em roxo de pessoas olhando para o ser.
+        Noite - 17:30: PMs capturam uma segunda criatura na mata. Uma ilustração noturna mostra o interior de um carro com dois militares observando o banco de trás.
+        Noite de domingo - 21/01/1996: Texto relata a movimentação no Hospital Humanitas. Há uma fotografia da fachada do hospital histórico de Varginha.
+        Madrugada - 17:30 (provável erro de digitação do infográfico para o dia 22): Relatos de exames e necrópsia na criatura no hospital.
+        Madrugada - 05:00: Relato do transporte da criatura em comboio do exército para a Unicamp.
+        15/02/1996: O policial Marco Eli Chereze morre de infecção generalizada após participar da captura. Há uma foto oficial dele em preto e branco com traje militar.
+        Maio/1996: Ufólogos fazem conferência revelando o caso para o mundo.
+        Anos Depois: O exército conclui em IPM que o ser avistado era, na verdade, um cidadão local conhecido como "Mudinho".
+O rodapé traz a assinatura do portal G1 e créditos de arte.
+</t>
   </si>
   <si>
     <t>1. Texto Alternativo Principal (Para o campo alt do CMS)
@@ -1114,8 +1454,23 @@
     <t>Contexto: O Brasil registrou um aumento de 5% nos casos de feminicídio em 2022, atingindo a marca recorde de 1.410 mulheres mortas por questões de gênero, o que representa uma média de uma vítima a cada seis horas. De acordo com o levantamento do Monitor da Violência, realizado em parceria com o Fórum Brasileiro de Segurança Pública, 15 estados apresentaram crescimento nas taxas, com destaque para a alta em Mato Grosso do Sul e Rondônia, enquanto especialistas apontam o desmonte de políticas públicas de proteção e o corte de verbas para o enfrentamento da violência contra a mulher como fatores determinantes para o agravamento do cenário. Embora o número total de mortes violentas de mulheres tenha caído ligeiramente, o crescimento específico dos feminicídios — onde há intenção deliberada de matar pela condição de ser mulher — evidencia a persistência da violência doméstica e familiar no país.</t>
   </si>
   <si>
+    <t>URL: https://g1.globo.com/monitor-da-violencia/noticia/2023/03/08/brasil-bate-recorde-de-feminicidios-em-2022-com-uma-mulher-morta-a-cada-6-horas.ghtml
+Tipo de Imagem: Imagem Complexa</t>
+  </si>
+  <si>
     <t>Contexto: O Brasil registrou um aumento de 5% nos casos de feminicídio em 2022, atingindo a marca recorde de 1.410 mulheres mortas por questões de gênero, o que representa uma média de uma vítima a cada seis horas. De acordo com o levantamento do Monitor da Violência, realizado em parceria com o Fórum Brasileiro de Segurança Pública, 15 estados apresentaram crescimento nas taxas, com destaque para a alta em Mato Grosso do Sul e Rondônia, enquanto especialistas apontam o desmonte de políticas públicas de proteção e o corte de verbas para o enfrentamento da violência contra a mulher como fatores determinantes para o agravamento do cenário. Embora o número total de mortes violentas de mulheres tenha caído ligeiramente, o crescimento específico dos feminicídios — onde há intenção deliberada de matar pela condição de ser mulher — evidencia a persistência da violência doméstica e familiar no país.
 Tipo de Imagem: Imagem Complexa</t>
+  </si>
+  <si>
+    <t>Opção 1: Descrição Principal (Curta e Direta)
+    Infográfico "Mulheres Assassinadas" aponta recorde de 1.410 feminicídios no Brasil em 2022, um aumento de 5% em relação ao ano anterior.
+Opção 2: Descrição Detalhada (Completa para leitura aprofundada)
+    Infográfico vertical intitulado "Mulheres Assassinadas", com fundo escuro e textos em branco. O conteúdo está dividido em quatro blocos de dados:
+        Homicídios Dolosos: Um gráfico de colunas hachuradas mostra o total de assassinatos de mulheres por ano: 4.558 em 2017; 4.353 em 2018; 3.966 em 2019; 3.999 em 2020; 3.831 em 2021; e 3.930 em 2022. Uma nota indica que Mato Grosso, Rondônia e Tocantins não contabilizavam dados de feminicídio em 2017.
+        Feminicídios: Um gráfico semicircular destaca que, dos 3.930 assassinatos de 2022, 1.410 foram registros de feminicídios (quando o crime é motivado pelo fato de a vítima ser mulher). Logo abaixo, um gráfico de linha mostra a evolução histórica do feminicídio: 1.046 em 2017; 1.225 em 2018; 1.330 em 2019; 1.354 em 2020; 1.337 em 2021; atingindo o recorde de 1.410 em 2022, o que representa um aumento de 5% em relação ao ano anterior.
+        Taxas de Assassinato: Exibe o mapa do Brasil destacando os extremos. A maior taxa está em Mato Grosso do Sul, com 8,3 mortes a cada 100 mil mulheres (estado pintado em tom de rosa). A menor taxa está em São Paulo, com 1,8 a cada 100 mil mulheres (estado pintado em branco).
+        Taxas de Feminicídio: Outro mapa do Brasil destaca que a maior taxa também pertence a Mato Grosso do Sul, com 3,5 a cada 100 mil mulheres. A menor taxa é a do Ceará, com 0,6 a cada 100 mil mulheres. Uma observação informa que os dados do quarto trimestre do Rio de Janeiro estavam em fase de análise.
+    No rodapé, constam o logotipo do G1 e a informação: "Infográfico atualizado em: 07/03/2023".</t>
   </si>
   <si>
     <t>1. Texto Alternativo Principal (Para o campo alt do CMS)
@@ -1166,8 +1521,20 @@
     <t>Contexto: O Resumão Diário do Jornal Nacional de 12 de maio de 2026 destaca o anúncio da União Europeia de suspender as importações de carnes e produtos de origem animal do Brasil a partir de setembro, alegando o descumprimento de normas contra o uso de antimicrobianos na pecuária, enquanto, na esfera da segurança pública, o governo federal lançou o programa "Brasil Contra o Crime Organizado", com investimentos de R$ 11 bilhões focados em asfixia financeira de facções e reforço no sistema prisional. No Judiciário, o ministro Nunes Marques tomou posse como presidente do Tribunal Superior Eleitoral (TSE), assumindo o comando da Corte ao lado do vice-presidente André Mendonça para conduzir as eleições de outubro, em um dia também marcado pelas investigações sobre uma explosão fatal causada por vazamento de gás em São Paulo e pelo pedido de arquivamento das investigações sobre a morte do cão Orelha em Santa Catarina.</t>
   </si>
   <si>
+    <t>URL: https://g1.globo.com/podcast/resumao-diario/noticia/2026/05/12/resumao-diario-do-jn-ue-veta-importacoes-de-carne-e-produtos-de-origem-animal-do-brasil-lula-lanca-programa-para-combater-o-crime-organizado-nunes-marques-toma-posse-no-tse.ghtml
+Tipo de Imagem: Imagem de Texto</t>
+  </si>
+  <si>
     <t>Contexto: O Resumão Diário do Jornal Nacional de 12 de maio de 2026 destaca o anúncio da União Europeia de suspender as importações de carnes e produtos de origem animal do Brasil a partir de setembro, alegando o descumprimento de normas contra o uso de antimicrobianos na pecuária, enquanto, na esfera da segurança pública, o governo federal lançou o programa "Brasil Contra o Crime Organizado", com investimentos de R$ 11 bilhões focados em asfixia financeira de facções e reforço no sistema prisional. No Judiciário, o ministro Nunes Marques tomou posse como presidente do Tribunal Superior Eleitoral (TSE), assumindo o comando da Corte ao lado do vice-presidente André Mendonça para conduzir as eleições de outubro, em um dia também marcado pelas investigações sobre uma explosão fatal causada por vazamento de gás em São Paulo e pelo pedido de arquivamento das investigações sobre a morte do cão Orelha em Santa Catarina.
 Tipo de Imagem: Imagem de Texto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opção 1: Descrição Principal (Concisa, focada na transcrição do texto essencial)
+Logotipo do podcast "Resumão do JN". Texto em branco e azul sobre fundo azul escuro com a marca do portal g1 no canto inferior direito.
+Opção 2: Descrição Detalhada (Aprofundada, detalhando os elementos de design e cores)
+Imagem de texto em formato quadrado com fundo em tons de azul escuro e linhas curvas abstratas e sutis ao fundo.  No canto superior esquerdo, destaca-se o título do podcast: as palavras "Resumão" e "do" estão escritas em letras brancas de tamanho médio. Logo abaixo delas, as letras "JN" aparecem em tamanho grande, com preenchimento em um degradê que vai do azul claro ao azul escuro, contornadas por uma linha fina vermelha.  Na metade inferior da imagem, a palavra "RESUMÃO" está replicada várias vezes em letras maiúsculas azul-claras de forma diagonal e estilizada, criando um efeito de fundo. No canto inferior direito, destaca-se o logotipo oficial do portal de notícias "g1" em letras minúsculas na cor branca.  
+Opção 3: Abordagem Decorativa (Se aplicada em contextos onde o texto adjacente já repete rigorosamente o título do podcast)
+Caso esta imagem seja utilizada em uma lista onde o título "Resumão do JN" já esteja escrito logo ao lado em formato de texto acessível, ela assume função redundante ou estética. Para evitar o cansaço na leitura de telas, ela pode ser programada com o atributo alt="" (vazio) para ser ignorada pela tecnologia assistiva.  </t>
   </si>
   <si>
     <t>1. Texto Alternativo Principal (Tag alt - Conciso e Direto)
@@ -1212,8 +1579,20 @@
     <t>Contexto: É falso o comunicado atribuído à empresa Ypê que circula nas redes sociais comemorando um suposto "recorde de vendas" após a determinação de suspensão de produtos pela Anvisa em maio de 2026. Segundo a checagem do G1 Fato ou Fake, a publicação viral utiliza uma identidade visual que mimetiza informativos oficiais, mas a empresa desmentiu a emissão de qualquer balanço recente de vendas e esclareceu que não houve tal pico de consumo motivado pelo incidente. A confusão teve origem após a agência reguladora suspender e determinar o recolhimento de lotes específicos de detergentes da marca por risco de contaminação biológica; embora a Ypê tenha recorrido e obtido a liberação para comercializar novos lotes que cumprem as exigências sanitárias, a narrativa de que a crise gerou um "sucesso de vendas" em tom de desafio à agência foi fabricada para desinformar.</t>
   </si>
   <si>
+    <t>URL: https://g1.globo.com/fato-ou-fake/noticia/2026/05/12/e-fake-comunicado-da-ype-comemorando-recorde-de-vendas-apos-anvisa-determinar-suspensao.ghtml
+Tipo de Imagem: Imagem de Texto</t>
+  </si>
+  <si>
     <t>Contexto: É falso o comunicado atribuído à empresa Ypê que circula nas redes sociais comemorando um suposto "recorde de vendas" após a determinação de suspensão de produtos pela Anvisa em maio de 2026. Segundo a checagem do G1 Fato ou Fake, a publicação viral utiliza uma identidade visual que mimetiza informativos oficiais, mas a empresa desmentiu a emissão de qualquer balanço recente de vendas e esclareceu que não houve tal pico de consumo motivado pelo incidente. A confusão teve origem após a agência reguladora suspender e determinar o recolhimento de lotes específicos de detergentes da marca por risco de contaminação biológica; embora a Ypê tenha recorrido e obtido a liberação para comercializar novos lotes que cumprem as exigências sanitárias, a narrativa de que a crise gerou um "sucesso de vendas" em tom de desafio à agência foi fabricada para desinformar.
 Tipo de Imagem: Imagem de Texto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opção 1: Descrição Principal (Curta e Direta para o campo alt)
+Selo com o texto "É FAKE" em letras maiúsculas brancas sobre um retângulo azul. Ao fundo, o contorno de um ponto de exclamação dentro de um círculo.
+Opção 2: Descrição Detalhada (Completa para leitura aprofundada)
+Imagem de texto em formato retangular horizontal com fundo branco. No centro, há um retângulo azul de cantos arredondados contendo a inscrição "É FAKE" em letras maiúsculas brancas e de traços grossos. A letra "A" da palavra "FAKE" é estilizada, trazendo em seu interior o desenho de um ponto de exclamação invertido. À esquerda do retângulo azul, há o contorno fino, em linhas azuis, de um grande círculo que abriga um ponto de exclamação vertical, que fica parcialmente coberto pelo bloco de texto principal.  
+Opção 3: Abordagem de Imagem Decorativa (Redundante)
+Se esta imagem for inserida em uma posição da página onde o próprio texto do site já traga a tag textual ou a transcrição literal "Selo: É Fake", ela passa a ter um papel redundante na leitura. Em cenários assim, para evitar que seu leitor de telas repita a mesma informação em sequência, ela pode ser configurada com o atributo alt="" (vazio), permitindo que você passe direto pelo elemento sem interrupções desnecessárias.  </t>
   </si>
   <si>
     <t>1. Texto Alternativo Principal (Alt Text)
@@ -1261,8 +1640,20 @@
     <t>Contexto: O documentário "A Colisão dos Destinos", dirigido por Doriel Francisco e focado na trajetória de Jair Bolsonaro, estreou nos cinemas nesta quinta-feira (14) registrando baixa adesão de público e salas praticamente vazias em diversas capitais brasileiras. A produção adota um tom laudatório ao ex-presidente, concentrando-se em sua ascensão política e no período de seu mandato, mas chama a atenção por omitir fatos históricos relevantes, como a derrota eleitoral de 2022, os eventos de 8 de janeiro e a própria figura da ex-primeira-dama Michelle Bolsonaro. Paralelamente ao lançamento, o filme enfrenta controvérsias relacionadas ao seu financiamento, incluindo investigações sobre aportes financeiros de empresários e denúncias de condições precárias de trabalho durante as gravações, o que tem gerado desgaste político para aliados e familiares do ex-mandatário.</t>
   </si>
   <si>
+    <t>URL: https://g1.globo.com/pop-arte/cinema/noticia/2026/05/15/documentario-sobre-bolsonaro-estreia-com-sessoes-vazias-exalta-ex-presidente-ignora-michelle-e-omite-derrota-e-tentativa-de-golpe.ghtml
+Tipo de Imagem: Imagem de Texto</t>
+  </si>
+  <si>
     <t>Contexto: O documentário "A Colisão dos Destinos", dirigido por Doriel Francisco e focado na trajetória de Jair Bolsonaro, estreou nos cinemas nesta quinta-feira (14) registrando baixa adesão de público e salas praticamente vazias em diversas capitais brasileiras. A produção adota um tom laudatório ao ex-presidente, concentrando-se em sua ascensão política e no período de seu mandato, mas chama a atenção por omitir fatos históricos relevantes, como a derrota eleitoral de 2022, os eventos de 8 de janeiro e a própria figura da ex-primeira-dama Michelle Bolsonaro. Paralelamente ao lançamento, o filme enfrenta controvérsias relacionadas ao seu financiamento, incluindo investigações sobre aportes financeiros de empresários e denúncias de condições precárias de trabalho durante as gravações, o que tem gerado desgaste político para aliados e familiares do ex-mandatário.
 Tipo de Imagem: Imagem de Texto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opção 1: Descrição Principal (Concisa, focada no texto essencial)
+Cartaz do filme "Jair Messias Bolsonaro - A Colisão dos Destinos", com estreia indicada para 14 de maio nos cinemas. Centraliza o rosto do ex-presidente sobre um fundo com aparelhos de TV antigos e traz a assinatura da Dori Filmes na parte inferior.
+Opção 2: Descrição Detalhada (Aprofundada, detalhando elementos de design e composição visual)
+Cartaz promocional do documentário sobre Jair Bolsonaro. No centro, em destaque e em primeiro plano, está o rosto de Jair Bolsonaro olhando fixamente para cima e para a direita. Ele veste um terno escuro que se mistura ao fundo.  O plano de fundo é composto por uma parede preenchida por diversas telas de televisores de tubo antigos e empilhados. Nestas telas, aparecem imagens de arquivo granuladas e escuras, retratando momentos de sua trajetória, como apoiadores em manifestações, registros históricos e a bandeira do Brasil.  Na metade inferior, sobre o peito de Bolsonaro, estão dispostas as informações textuais em letras brancas e amarelas: "14 de Maio nos cinemas", seguida por "JAIR MESSIAS BOLSONARO" em letras maiúsculas. Logo abaixo, o título principal "A COLISÃO DOS" está escrito em letras garrafais amarelas, e a palavra "Destinos" aparece escrita logo abaixo em uma fonte cursiva branca, imitando caligrafia estilizada. Na base do cartaz, centralizado dentro de um retângulo verde, lê-se "DORI FILMES". 
+Opção 3: Abordagem de Imagem Decorativa (Redundante)
+Caso este cartaz esteja inserido em uma página onde o corpo do texto da notícia já transcreva e repita rigorosamente todas as informações do filme (como título completo, produtora e data de estreia), a imagem passa a ter uma função puramente estética ou redundante para o usuário de leitor de telas. Nesse contexto específico, ela deve ser configurada com o atributo alt="" (vazio) para que o seu software de leitura ignore o elemento e proporcione uma navegação mais fluida e menos cansativa.  </t>
   </si>
   <si>
     <t>Texto Alternativo Principal (Campo Alt Text)
@@ -1289,6 +1680,10 @@
   </si>
   <si>
     <t>Contexto: Investidores estrangeiros detentores de "vistos gold" iniciaram uma série de processos judiciais contra o Estado português em resposta às recentes alterações na Lei da Nacionalidade, que elevaram o tempo de residência exigido para a obtenção da cidadania de cinco para dez anos (ou sete anos para cidadãos da CPLP). A revolta do grupo baseia-se na alegação de que a mudança das regras durante o processo fere o princípio da segurança jurídica e a confiança legítima de quem realizou investimentos vultosos no país sob a promessa de um caminho mais curto para o passaporte europeu. Enquanto o governo justifica o endurecimento das normas como uma medida necessária para controlar o fluxo migratório e garantir a integridade do sistema de concessão de nacionalidade, os advogados dos investidores argumentam que a ausência de um regime de transição adequado prejudica milhares de famílias que já haviam planejado suas vidas e negócios com base na legislação anterior.</t>
+  </si>
+  <si>
+    <t>URL: https://g1.globo.com/mundo/noticia/2026/05/15/portugal-enfrenta-revolta-de-golden-visas-apos-mudancas-na-lei-da-nacionalidade.ghtml
+Tipo de Imagem: Imagem Decorativa</t>
   </si>
   <si>
     <t>Contexto: Investidores estrangeiros detentores de "vistos gold" iniciaram uma série de processos judiciais contra o Estado português em resposta às recentes alterações na Lei da Nacionalidade, que elevaram o tempo de residência exigido para a obtenção da cidadania de cinco para dez anos (ou sete anos para cidadãos da CPLP). A revolta do grupo baseia-se na alegação de que a mudança das regras durante o processo fere o princípio da segurança jurídica e a confiança legítima de quem realizou investimentos vultosos no país sob a promessa de um caminho mais curto para o passaporte europeu. Enquanto o governo justifica o endurecimento das normas como uma medida necessária para controlar o fluxo migratório e garantir a integridade do sistema de concessão de nacionalidade, os advogados dos investidores argumentam que a ausência de um regime de transição adequado prejudica milhares de famílias que já haviam planejado suas vidas e negócios com base na legislação anterior.
@@ -1322,6 +1717,10 @@
     <t>Contexto: A decisão da União Europeia de suspender as importações de carne e produtos de origem animal do Brasil a partir de 3 de setembro de 2026 deve gerar um impacto econômico estimado em quase US$ 2 bilhões anuais, afetando não apenas a carne bovina, mas também aves, ovos, mel e cavalos. O veto ocorreu porque o Brasil foi removido da lista de países que cumprem as exigências sanitárias do bloco relacionadas ao controle de antimicrobianos, especificamente a proibição do uso de antibióticos para promover o crescimento animal ou de substâncias reservadas para uso humano. Embora o governo brasileiro tenha manifestado "surpresa" e alegue que as exigências já são atendidas, analistas apontam que a medida tem um forte componente político, refletindo pressões de produtores rurais europeus (especialmente da França) contra o acordo Mercosul-UE e uma tentativa do bloco de impor padrões rigorosos de reciprocidade ambiental e sanitária. O Ministério da Agricultura e a diplomacia brasileira já iniciaram reuniões para tentar reverter a decisão antes do prazo final, argumentando que o sistema de controle nacional é robusto e que o impasse pode ser resolvido com o envio de garantias e adequações técnicas adicionais.</t>
   </si>
   <si>
+    <t>URL: https://g1.globo.com/economia/agronegocios/noticia/2026/05/13/os-impactos-da-decisao-da-ue-de-barrar-a-carne-brasileira.ghtml
+Tipo de Imagem: Imagem Decorativa</t>
+  </si>
+  <si>
     <t>Contexto: A decisão da União Europeia de suspender as importações de carne e produtos de origem animal do Brasil a partir de 3 de setembro de 2026 deve gerar um impacto econômico estimado em quase US$ 2 bilhões anuais, afetando não apenas a carne bovina, mas também aves, ovos, mel e cavalos. O veto ocorreu porque o Brasil foi removido da lista de países que cumprem as exigências sanitárias do bloco relacionadas ao controle de antimicrobianos, especificamente a proibição do uso de antibióticos para promover o crescimento animal ou de substâncias reservadas para uso humano. Embora o governo brasileiro tenha manifestado "surpresa" e alegue que as exigências já são atendidas, analistas apontam que a medida tem um forte componente político, refletindo pressões de produtores rurais europeus (especialmente da França) contra o acordo Mercosul-UE e uma tentativa do bloco de impor padrões rigorosos de reciprocidade ambiental e sanitária. O Ministério da Agricultura e a diplomacia brasileira já iniciaram reuniões para tentar reverter a decisão antes do prazo final, argumentando que o sistema de controle nacional é robusto e que o impasse pode ser resolvido com o envio de garantias e adequações técnicas adicionais.
 Tipo de Imagem: Imagem Decorativa</t>
   </si>
@@ -1353,6 +1752,10 @@
     <t>Contexto: A Coordenação de Aperfeiçoamento de Pessoal de Nível Superior (CAPES) lançou o Programa Aurora, uma iniciativa voltada a apoiar a trajetória acadêmica de professoras grávidas (a partir do 2º trimestre) ou mães de crianças de até 2 anos (ou sem limite de idade para filhos com deficiência). O programa oferece até 300 bolsas de pós-doutorado no valor de R$ 5.200,00 mensais por 24 meses, permitindo que a docente selecione um bolsista com título de doutorado para auxiliá-la em suas funções de pesquisa, aulas e orientação, garantindo que suas atividades não sejam interrompidas durante a maternidade. As inscrições para o primeiro ciclo de análise devem ser feitas exclusivamente pela internet até o dia 5 de junho de 2026, visando combater a desigualdade de gênero na ciência com um investimento total de R$ 37,4 milhões.</t>
   </si>
   <si>
+    <t>URL: https://g1.globo.com/educacao/noticia/2026/05/13/maes-professoras-podem-se-inscrever-em-bolsas-de-estudo-de-r-52-mil-mensais-em-novo-programa-da-capes.ghtml
+Tipo de Imagem: Imagem Decorativa</t>
+  </si>
+  <si>
     <t>Contexto: A Coordenação de Aperfeiçoamento de Pessoal de Nível Superior (CAPES) lançou o Programa Aurora, uma iniciativa voltada a apoiar a trajetória acadêmica de professoras grávidas (a partir do 2º trimestre) ou mães de crianças de até 2 anos (ou sem limite de idade para filhos com deficiência). O programa oferece até 300 bolsas de pós-doutorado no valor de R$ 5.200,00 mensais por 24 meses, permitindo que a docente selecione um bolsista com título de doutorado para auxiliá-la em suas funções de pesquisa, aulas e orientação, garantindo que suas atividades não sejam interrompidas durante a maternidade. As inscrições para o primeiro ciclo de análise devem ser feitas exclusivamente pela internet até o dia 5 de junho de 2026, visando combater a desigualdade de gênero na ciência com um investimento total de R$ 37,4 milhões.
 Tipo de Imagem: Imagem Decorativa</t>
   </si>
@@ -1387,6 +1790,10 @@
     <t>Contexto: A bancada do Partido dos Trabalhadores retomou a estratégia digital de classificar o Congresso Nacional como "inimigo do povo" como forma de reagir a recentes derrotas legislativas e reforçar um discurso antissistema que ecoa o posicionamento do presidente Luiz Inácio Lula da Silva. A tática mira prioritariamente o Senado e estende-se também a críticas contra o Banco Central e seu presidente, Gabriel Galípolo, buscando personificar a responsabilidade pelos juros altos sob o rótulo de "traidor". Internamente, a sigla avalia que a retomada desse mote é essencial para recuperar as raízes do partido e mobilizar a base eleitoral em torno de pautas populares, como a aprovação do fim da escala de trabalho 6x1, equilibrando a retórica de enfrentamento à elite financeira com a necessidade pragmática de apoio parlamentar para materializar projetos de impacto social.</t>
   </si>
   <si>
+    <t>URL: https://www.cnnbrasil.com.br/blogs/isabel-mega/politica/petistas-retomam-mote-de-congresso-inimigo-do-povo/
+Tipo de Imagem: Imagem Informativa</t>
+  </si>
+  <si>
     <t>Contexto: A bancada do Partido dos Trabalhadores retomou a estratégia digital de classificar o Congresso Nacional como "inimigo do povo" como forma de reagir a recentes derrotas legislativas e reforçar um discurso antissistema que ecoa o posicionamento do presidente Luiz Inácio Lula da Silva. A tática mira prioritariamente o Senado e estende-se também a críticas contra o Banco Central e seu presidente, Gabriel Galípolo, buscando personificar a responsabilidade pelos juros altos sob o rótulo de "traidor". Internamente, a sigla avalia que a retomada desse mote é essencial para recuperar as raízes do partido e mobilizar a base eleitoral em torno de pautas populares, como a aprovação do fim da escala de trabalho 6x1, equilibrando a retórica de enfrentamento à elite financeira com a necessidade pragmática de apoio parlamentar para materializar projetos de impacto social.
 Tipo de Imagem: Informativa</t>
   </si>
@@ -1418,6 +1825,10 @@
     <t>Context: Uma criança de cinco anos foi internada no Hospital Monsenhor Walfredo Gurgel, em Natal, com suspeita de intoxicação e lesões na boca após utilizar um detergente durante o banho na última quarta-feira. O incidente ocorreu em uma residência no bairro das Quintas, na zona Oeste da capital potiguar, onde familiares relataram que o produto teria causado reações imediatas após o contato com a mucosa oral. A Polícia Civil do Rio Grande do Norte iniciou as investigações para apurar se houve falha na composição do produto de limpeza ou se o caso configura negligência por parte dos responsáveis. O estado de saúde da vítima é considerado estável, mas ela permanece sob observação médica para monitoramento de possíveis danos internos causados pela substância química.</t>
   </si>
   <si>
+    <t>URL: https://www.cnnbrasil.com.br/nacional/nordeste/rn/crianca-e-internada-por-suspeita-de-contaminacao-apos-uso-de-detergente/
+Tipo de Imagem: Imagem Informativa</t>
+  </si>
+  <si>
     <t xml:space="preserve">Context: Uma criança de cinco anos foi internada no Hospital Monsenhor Walfredo Gurgel, em Natal, com suspeita de intoxicação e lesões na boca após utilizar um detergente durante o banho na última quarta-feira. O incidente ocorreu em uma residência no bairro das Quintas, na zona Oeste da capital potiguar, onde familiares relataram que o produto teria causado reações imediatas após o contato com a mucosa oral. A Polícia Civil do Rio Grande do Norte iniciou as investigações para apurar se houve falha na composição do produto de limpeza ou se o caso configura negligência por parte dos responsáveis. O estado de saúde da vítima é considerado estável, mas ela permanece sob observação médica para monitoramento de possíveis danos internos causados pela substância química.
 Tipo de Imagem: Informativa
 </t>
@@ -1446,6 +1857,10 @@
     <t>Contexto: O Ministério da Justiça e Segurança Pública fundamentou a elevação da classificação indicativa do YouTube para 16 anos citando, entre outros fatores, a popularização das "novelas das frutas", produções criadas por inteligência artificial que utilizam personagens antropomórficos visualmente atrativos para crianças, mas com enredos de conteúdo adulto. Segundo a análise técnica, essas tramas abordam temas sensíveis como violência doméstica, consumo de entorpecentes, apelo sexual e assassinatos com realismo imagético, o que representa riscos à formação do público infanto-juvenil por mimetizar a estética de animações infantis consagradas enquanto veiculam situações de criminalidade e preconceito. A decisão, baseada nas diretrizes do ECA Digital, também aponta a presença de linguagens de baixo calão, tortura e relatos libidinosos em diversos formatos de vídeo na plataforma, reforçando a necessidade de uma indicação etária mais rigorosa para mitigar a exposição precoce de adolescentes a conteúdos de alta complexidade e impacto emocional.</t>
   </si>
   <si>
+    <t>URL: https://www.cnnbrasil.com.br/tecnologia/governo-cita-novela-das-frutas-ao-subir-classificacao-do-youtube-entenda/
+Tipo de Imagem: Imagem Informativa</t>
+  </si>
+  <si>
     <t>Contexto: O Ministério da Justiça e Segurança Pública fundamentou a elevação da classificação indicativa do YouTube para 16 anos citando, entre outros fatores, a popularização das "novelas das frutas", produções criadas por inteligência artificial que utilizam personagens antropomórficos visualmente atrativos para crianças, mas com enredos de conteúdo adulto. Segundo a análise técnica, essas tramas abordam temas sensíveis como violência doméstica, consumo de entorpecentes, apelo sexual e assassinatos com realismo imagético, o que representa riscos à formação do público infanto-juvenil por mimetizar a estética de animações infantis consagradas enquanto veiculam situações de criminalidade e preconceito. A decisão, baseada nas diretrizes do ECA Digital, também aponta a presença de linguagens de baixo calão, tortura e relatos libidinosos em diversos formatos de vídeo na plataforma, reforçando a necessidade de uma indicação etária mais rigorosa para mitigar a exposição precoce de adolescentes a conteúdos de alta complexidade e impacto emocional.
 Tipo de Imagem: Imagem Informativa</t>
   </si>
@@ -1482,6 +1897,10 @@
   </si>
   <si>
     <t>Contexto: A pandemia de Covid-19 provocou a crise econômica global mais severa desde a Grande Depressão, resultando em uma contração de 4,4% no PIB mundial em 2020 e elevando drasticamente as taxas de desemprego nas principais economias do mundo. De acordo com levantamento baseado em dados do FMI e índices de mercado, setores como turismo, hotelaria e varejo físico foram os mais atingidos devido aos lockdowns e restrições de viagens, com estimativas de que a aviação internacional só retorne aos níveis pré-pandemia por volta de 2025. Enquanto a China foi a única grande economia a registrar crescimento em 2020, o cenário global foi marcado por quedas históricas nas bolsas de valores, reduções nas taxas de juros por bancos centrais para estimular o consumo e uma migração acelerada para o varejo online, paralelamente à valorização de empresas farmacêuticas envolvidas no desenvolvimento de vacinas.</t>
+  </si>
+  <si>
+    <t>URL: https://g1.globo.com/economia/noticia/2021/02/02/coronavirus-8-graficos-para-entender-como-a-pandemia-de-covid-19-afetou-as-maiores-economias-do-mundo.ghtml
+Tipo de Imagem: Imagem Complexa</t>
   </si>
   <si>
     <t>Contexto: A pandemia de Covid-19 provocou a crise econômica global mais severa desde a Grande Depressão, resultando em uma contração de 4,4% no PIB mundial em 2020 e elevando drasticamente as taxas de desemprego nas principais economias do mundo. De acordo com levantamento baseado em dados do FMI e índices de mercado, setores como turismo, hotelaria e varejo físico foram os mais atingidos devido aos lockdowns e restrições de viagens, com estimativas de que a aviação internacional só retorne aos níveis pré-pandemia por volta de 2025. Enquanto a China foi a única grande economia a registrar crescimento em 2020, o cenário global foi marcado por quedas históricas nas bolsas de valores, reduções nas taxas de juros por bancos centrais para estimular o consumo e uma migração acelerada para o varejo online, paralelamente à valorização de empresas farmacêuticas envolvidas no desenvolvimento de vacinas.
@@ -1538,6 +1957,10 @@
     <t>Contexto: Estatísticas do Observatório de Segurança Pública de Minas Gerais indicam que o "roubo consumado" foi o crime violento mais frequente no estado desde 2012, representando mais de 860 mil das 1,1 milhão de ocorrências totais registradas no período. O levantamento destaca 2016 como o ano de maior incidência, com 132.362 casos, seguido por uma redução progressiva que atingiu cerca de 90% até 2025, enquanto Belo Horizonte e Contagem lideram o ranking de municípios com o maior volume de registros criminais. De acordo com os dados, os delitos ocorrem predominantemente em vias públicas durante o turno da noite, frequentemente mediante o uso de armas de fogo, motivando o governo estadual a intensificar estratégias de inteligência e ações integradas das forças de segurança para dar continuidade à tendência de queda nos indicadores.</t>
   </si>
   <si>
+    <t>URL: https://www.cnnbrasil.com.br/nacional/sudeste/mg/roubo-foi-o-crime-mais-registrado-em-mg-desde-2012-veja-numeros/
+Tipo de Imagem: Imagem Complexa</t>
+  </si>
+  <si>
     <t>Contexto: Estatísticas do Observatório de Segurança Pública de Minas Gerais indicam que o "roubo consumado" foi o crime violento mais frequente no estado desde 2012, representando mais de 860 mil das 1,1 milhão de ocorrências totais registradas no período. O levantamento destaca 2016 como o ano de maior incidência, com 132.362 casos, seguido por uma redução progressiva que atingiu cerca de 90% até 2025, enquanto Belo Horizonte e Contagem lideram o ranking de municípios com o maior volume de registros criminais. De acordo com os dados, os delitos ocorrem predominantemente em vias públicas durante o turno da noite, frequentemente mediante o uso de armas de fogo, motivando o governo estadual a intensificar estratégias de inteligência e ações integradas das forças de segurança para dar continuidade à tendência de queda nos indicadores.
 Tipo de Imagem: Imagem Complexa</t>
   </si>
@@ -1590,6 +2013,10 @@
     <t>Contexto: A nova campanha da CNN Brasil consolida a emissora como o maior canal multiplataforma de notícias do país após cinco anos de operação, registrando um alcance mensal superior a 80 milhões de pessoas no último trimestre de 2024. O levantamento destaca a liderança da rede sobre a concorrente GloboNews em diversos segmentos digitais, com 35 milhões de acessos mensais no portal e presença expressiva no YouTube e redes sociais, além da distribuição em plataformas como Samsung TV Plus e sinal de banda KU. Ao somar todas as frentes de transmissão e excluir as sobreposições de público, a CNN totaliza um alcance democratizado que reafirma sua estratégia de distribuição abrangente e jornalismo imparcial em múltiplas telas.</t>
   </si>
   <si>
+    <t>URL: https://www.cnnbrasil.com.br/nacional/brasil/numeros-cnn/
+Tipo de Imagem: Imagem Complexa</t>
+  </si>
+  <si>
     <t>Contexto: A nova campanha da CNN Brasil consolida a emissora como o maior canal multiplataforma de notícias do país após cinco anos de operação, registrando um alcance mensal superior a 80 milhões de pessoas no último trimestre de 2024. O levantamento destaca a liderança da rede sobre a concorrente GloboNews em diversos segmentos digitais, com 35 milhões de acessos mensais no portal e presença expressiva no YouTube e redes sociais, além da distribuição em plataformas como Samsung TV Plus e sinal de banda KU. Ao somar todas as frentes de transmissão e excluir as sobreposições de público, a CNN totaliza um alcance democratizado que reafirma sua estratégia de distribuição abrangente e jornalismo imparcial em múltiplas telas.
 Tipo de Imagem: Imagem Complexa</t>
   </si>
@@ -1639,6 +2066,10 @@
     <t>Contexto: O programa CNN Sinais Vitais, apresentado pelo cardiologista Roberto Kalil, aborda os impactos deletérios do uso excessivo de tecnologias digitais, destacando prejuízos físicos e cognitivos que afetam prioritariamente crianças e adolescentes. Especialistas convidados alertam para problemas que vão desde danos à coluna cervical e ombros, causados pela má postura ao utilizar dispositivos, até o comprometimento do desenvolvimento da fala, da linguagem e do raciocínio lógico devido à substituição de interações humanas por telas. O conteúdo enfatiza que o mecanismo de recompensa do cérebro ao acessar jogos e redes sociais libera substâncias como dopamina e serotonina, assemelhando-se ao processo de dependência química, o que exige um controle rigoroso do tempo de exposição conforme as recomendações da Sociedade Brasileira de Pediatria para mitigar riscos como a redução do quociente de inteligência (QI) e o isolamento social.</t>
   </si>
   <si>
+    <t>URL: https://www.cnnbrasil.com.br/saude/cnn-sinais-vitais-discute-riscos-a-saude-do-uso-em-excesso-da-tecnologia-digital/
+Tipo de Imagem: Imagem de Texto</t>
+  </si>
+  <si>
     <t>Contexto: O programa CNN Sinais Vitais, apresentado pelo cardiologista Roberto Kalil, aborda os impactos deletérios do uso excessivo de tecnologias digitais, destacando prejuízos físicos e cognitivos que afetam prioritariamente crianças e adolescentes. Especialistas convidados alertam para problemas que vão desde danos à coluna cervical e ombros, causados pela má postura ao utilizar dispositivos, até o comprometimento do desenvolvimento da fala, da linguagem e do raciocínio lógico devido à substituição de interações humanas por telas. O conteúdo enfatiza que o mecanismo de recompensa do cérebro ao acessar jogos e redes sociais libera substâncias como dopamina e serotonina, assemelhando-se ao processo de dependência química, o que exige um controle rigoroso do tempo de exposição conforme as recomendações da Sociedade Brasileira de Pediatria para mitigar riscos como a redução do quociente de inteligência (QI) e o isolamento social.
 Tipo de Imagem: Imagem de Texto</t>
   </si>
@@ -1681,6 +2112,10 @@
     <t>Contexto: A CNN Brasil lançou uma nova identidade visual e a assinatura "CNN Brasil. Você por dentro de tudo", marcando uma etapa estratégica de consolidação após dois anos de sua estreia no país e reforçando seu compromisso com a imparcialidade e a precisão dos fatos. Criada pela agência AlmapBBDO, a campanha utiliza a simbologia de um polígrafo e o conceito "Nem uma linha além dos fatos" em peças publicitárias para TV, rádio e plataformas digitais, destacando-se em um ano de cobertura eleitoral decisiva e crescimento recorde de audiência digital. Segundo a então CEO Renata Afonso, a iniciativa visa estreitar o vínculo com o público em um cenário de expansão da vida digital e desinformação, posicionando a emissora como uma referência de credibilidade para a audiência e um parceiro de negócios estratégico para marcas que buscam associar-se a conteúdos jornalísticos qualificados e multiplataforma.</t>
   </si>
   <si>
+    <t>URL: https://www.cnnbrasil.com.br/nacional/cnn-brasil-lanca-nova-campanha-e-nova-assinatura/
+Tipo de Imagem: Imagem de Texto</t>
+  </si>
+  <si>
     <t>Contexto: A CNN Brasil lançou uma nova identidade visual e a assinatura "CNN Brasil. Você por dentro de tudo", marcando uma etapa estratégica de consolidação após dois anos de sua estreia no país e reforçando seu compromisso com a imparcialidade e a precisão dos fatos. Criada pela agência AlmapBBDO, a campanha utiliza a simbologia de um polígrafo e o conceito "Nem uma linha além dos fatos" em peças publicitárias para TV, rádio e plataformas digitais, destacando-se em um ano de cobertura eleitoral decisiva e crescimento recorde de audiência digital. Segundo a então CEO Renata Afonso, a iniciativa visa estreitar o vínculo com o público em um cenário de expansão da vida digital e desinformação, posicionando a emissora como uma referência de credibilidade para a audiência e um parceiro de negócios estratégico para marcas que buscam associar-se a conteúdos jornalísticos qualificados e multiplataforma.
 Tipo de Imagem: Imagem de Texto</t>
   </si>
@@ -1696,6 +2131,15 @@
         Parte Inferior Central: Nova assinatura da marca em letras menores: "CNN Brasil. Você por dentro de tudo."</t>
   </si>
   <si>
+    <t>Opções de Texto Alternativo (Alt Text)
+Opção 1: Texto Alternativo Principal (Direto e Conciso)
+    Logotipo da CNN em vermelho sobre fundo preto, acompanhado do texto em letras brancas: 'CNN. Onde a notícia acontece primeiro.'
+    Por que funciona? Vai direto ao ponto, não utiliza termos redundantes como "imagem de" ou "foto de", e descreve a informação essencial de maneira rápida para o leitor de tela.
+Opção 2: Descrição Longa / Informativa Completa
+Se o sistema permitir um detalhamento maior ou se a imagem for tratada de forma altamente informativa no corpo da matéria, use:
+    Logotipo com as letras 'CNN' em vermelho e traço duplo estilizado posicionado no centro esquerdo. À direita, a frase em letras maiúsculas e na cor branca diz: 'ONDE A NOTÍCIA ACONTECE PRIMEIRO.' O fundo de toda a composição é inteiramente preto.</t>
+  </si>
+  <si>
     <t>Propostas de Texto Alternativo (Alt Text)
 Opção 1: Transcrição Factual e Estruturada (Recomendado)
     Peça publicitária da CNN Brasil sobre fundo cinza-claro. No centro, o desenho de uma linha vermelha contínua oscila horizontalmente, assemelhando-se ao traçado de um polígrafo. Em letras pretas, lê-se o texto destacado: 'Nem uma linha além dos fatos.' Logo abaixo, o logotipo vermelho da CNN e a assinatura: 'CNN Brasil. Você por dentro de tudo.'
@@ -1723,6 +2167,11 @@
   </si>
   <si>
     <t>Contexto: O canal CNN Money, em parceria com o portal NeoFeed, estreia nesta sexta-feira (15) o programa "Números Falam", uma atração quinzenal apresentada pelo jornalista Márcio Kroehn que visa decodificar balanços corporativos e indicadores macroeconômicos por meio de entrevistas com lideranças empresariais. No episódio de estreia, que vai ao ar às 19h45, o convidado é o CFO da Gerdau, Rafael Japur, que analisa o desempenho financeiro da companhia e destaca a relevância das operações na América do Norte, responsáveis por 75% do Ebitda trimestral da empresa, além de comentar as perspectivas para o fluxo de caixa futuro. O lançamento consolida a expansão da grade do canal dedicada ao mercado financeiro e ao mundo dos negócios, reforçando a estratégia de oferecer análises técnicas e profundas para investidores e tomadores de decisão.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">URL: https://www.cnnbrasil.com.br/economia/negocios/numeros-falam-estreia-nesta-sexta-feira-15-no-cnn-money-saiba-mais/
+Tipo de Imagem: Imagem de Texto
+</t>
   </si>
   <si>
     <t>Contexto: O canal CNN Money, em parceria com o portal NeoFeed, estreia nesta sexta-feira (15) o programa "Números Falam", uma atração quinzenal apresentada pelo jornalista Márcio Kroehn que visa decodificar balanços corporativos e indicadores macroeconômicos por meio de entrevistas com lideranças empresariais. No episódio de estreia, que vai ao ar às 19h45, o convidado é o CFO da Gerdau, Rafael Japur, que analisa o desempenho financeiro da companhia e destaca a relevância das operações na América do Norte, responsáveis por 75% do Ebitda trimestral da empresa, além de comentar as perspectivas para o fluxo de caixa futuro. O lançamento consolida a expansão da grade do canal dedicada ao mercado financeiro e ao mundo dos negócios, reforçando a estratégia de oferecer análises técnicas e profundas para investidores e tomadores de decisão.
@@ -1740,6 +2189,16 @@
         Convidado do Episódio: Rafael Japur (CFO da Gerdau).
         Horário e Exibição: Sexta-feira, às 19h45.
         Destaque de Conteúdo (Quadro Informativo): "Operações na América do Norte representam 75% do Ebitda trimestral da Gerdau e impulsionam perspectivas para o fluxo de caixa."</t>
+  </si>
+  <si>
+    <t>Opção 1: Texto Alternativo Principal (Curto e Direto ao Ponto)
+Seguindo o limite técnico ideal de caracteres (geralmente entre 125 e 150 caracteres para manter a leitura do bloco fluida), priorizamos o nome do programa, a parceria institucional e as informações fundamentais de exibição:
+    Texto Alternativo Sugerido: Logotipo do programa Números Falam, uma parceria entre a CNN Money e o NeoFeed. Exibido na lateral esquerda, o logo da CNN Money.
+Opção 2: Descrição Longa (Ideal para Transcrição Completa da Arte)
+Se a arte digital contiver informações detalhadas sobre a data, horário de estreia, o nome do apresentador ou slogans cruciais estampados na imagem, é fundamental realizar uma descrição longa ou transcrever o texto diretamente no corpo da notícia (ou por meio de atributos complementares):
+    Texto Alternativo Longo Sugerido:
+    Arte digital com fundo conceitual de mercado financeiro. No centro, o título em destaque "Números Falam", novo programa produzido pelo NeoFeed em parceria com a CNN Money. Apresentado por Márcio Kroehn, o programa foca na análise de empresas e estratégias corporativas, indo ao ar às sextas-feiras, às 19h45.
+(Nota: Seguindo o nosso padrão, fomos direto à descrição textual do conteúdo sem utilizar marcadores redundantes como "Imagem com texto" ou "Foto da arte", otimizando a experiência do usuário do leitor de tela).</t>
   </si>
   <si>
     <t>Proposta de Texto Alternativo (Alt Text)
@@ -1781,6 +2240,10 @@
     <t>Contexto: O governo federal, por meio do Ministério da Justiça e Segurança Pública, elevou a classificação indicativa do YouTube de 14 para 16 anos, fundamentando a decisão na identificação de conteúdos contendo violência extrema, linguagem imprópria, drogas e temas sexuais prejudiciais a menores. A medida, oficializada via Diário Oficial da União e integrante das novas diretrizes do ECA Digital para a proteção online de crianças e adolescentes, possui caráter informativo e obriga a plataforma a exibir o selo etário e as justificativas da restrição de forma visível em todos os seus pontos de acesso. Embora não configure censura ou remoção de vídeos, a reclassificação impõe um rigor maior na indicação de faixa etária, alinhando o YouTube a outras redes sociais, como TikTok e Instagram, que também tiveram suas idades recomendadas ajustadas para 16 anos sob a mesma política de regulação.</t>
   </si>
   <si>
+    <t>URL: https://www.cnnbrasil.com.br/tecnologia/governo-aumenta-classificacao-indicativa-do-youtube-para-16-anos-entenda/
+Tipo de Imagem: Imagem Decorativa</t>
+  </si>
+  <si>
     <t>Contexto: O governo federal, por meio do Ministério da Justiça e Segurança Pública, elevou a classificação indicativa do YouTube de 14 para 16 anos, fundamentando a decisão na identificação de conteúdos contendo violência extrema, linguagem imprópria, drogas e temas sexuais prejudiciais a menores. A medida, oficializada via Diário Oficial da União e integrante das novas diretrizes do ECA Digital para a proteção online de crianças e adolescentes, possui caráter informativo e obriga a plataforma a exibir o selo etário e as justificativas da restrição de forma visível em todos os seus pontos de acesso. Embora não configure censura ou remoção de vídeos, a reclassificação impõe um rigor maior na indicação de faixa etária, alinhando o YouTube a outras redes sociais, como TikTok e Instagram, que também tiveram suas idades recomendadas ajustadas para 16 anos sob a mesma política de regulação.
 Tipo de Imagem: Imagem Decorativa</t>
   </si>
@@ -1799,6 +2262,17 @@
         Selo oficial de classificação indicativa de 16 anos, ilustrando a nova regulamentação do governo federal para o YouTube.</t>
   </si>
   <si>
+    <t>Opção 1: Tratamento Técnico como Elemento Puramente Decorativo (Recomendado)
+Se a imagem cumpre apenas um papel estético (como uma imagem genérica de banco de dados ou um detalhe de layout) e sua ausência não altera em nada o entendimento da decisão do governo sobre a plataforma, o ideal é instruir o leitor de tela a ignorá-la. Para isso, o campo alt deve conter apenas aspas vazias, evitando que o sintetizador de voz leia códigos desnecessários.
+    Texto Alternativo (Código Alt Sugerido): ""
+    Comportamento no Leitor de Tela: O leitor passará direto pelo elemento, mantendo o foco do usuário totalmente no texto da notícia.
+Opção 2: Tratamento Editorial de Banco de Dados (Contexto de Tecnologia)
+Se a política do portal exigir o preenchimento descritivo mesmo para imagens ilustrativas, a fim de contextualizar visualmente o tema "YouTube" ou "redes sociais", a descrição deve ser direta e concisa:
+    Texto Alternativo Sugerido (até 150 caracteres):
+    Logotipo do YouTube exibido na tela iluminada de um smartphone segurado por uma pessoa.
+(Nota: Mantendo nosso padrão jornalístico de acessibilidade, fomos direto ao assunto visual sem usar os termos redundantes "Imagem de" ou "Foto de").</t>
+  </si>
+  <si>
     <t>Opção 1: Descrição Curta Informativa (Recomendada para Portais de Notícias)
 Se o nosso manual de estilo interno exigir que toda imagem de artigo editorial pintada na tela tenha uma descrição textual para SEO e contextualização de tela:
     Texto Descritivo:
@@ -1837,6 +2311,11 @@
     <t>Contexto: O consumo de ovos no Brasil deve atingir o recorde de 320 unidades per capita em 2026, consolidando um crescimento de 166% nos últimos dezessete anos e refletindo uma mudança profunda nos hábitos alimentares da população. Segundo dados do Instituto Ovos Brasil, esse avanço é impulsionado pela desmistificação científica do alimento em relação ao colesterol, pela busca por proteínas de alto valor biológico e baixo custo, e pela crescente demanda associada a dietas fitness, low carb e ao uso de medicamentos para emagrecimento que exigem a preservação da massa muscular. Com uma produção nacional superior a 250 milhões de unidades diárias, o setor destina 98% de sua oferta ao mercado interno, sustentado pela praticidade do produto e pelo envelhecimento da população, que prioriza a longevidade saudável por meio de alimentos nutricionalmente densos.</t>
   </si>
   <si>
+    <t xml:space="preserve">URL: https://www.cnnbrasil.com.br/agro/consumo-de-ovos-no-brasil-cresce-166-em-dezessete-anos/
+Tipo de Imagem: Imagem Decorativa
+</t>
+  </si>
+  <si>
     <t>Contexto: O consumo de ovos no Brasil deve atingir o recorde de 320 unidades per capita em 2026, consolidando um crescimento de 166% nos últimos dezessete anos e refletindo uma mudança profunda nos hábitos alimentares da população. Segundo dados do Instituto Ovos Brasil, esse avanço é impulsionado pela desmistificação científica do alimento em relação ao colesterol, pela busca por proteínas de alto valor biológico e baixo custo, e pela crescente demanda associada a dietas fitness, low carb e ao uso de medicamentos para emagrecimento que exigem a preservação da massa muscular. Com uma produção nacional superior a 250 milhões de unidades diárias, o setor destina 98% de sua oferta ao mercado interno, sustentado pela praticidade do produto e pelo envelhecimento da população, que prioriza a longevidade saudável por meio de alimentos nutricionalmente densos.
 Tipo de Imagem: Decorativa</t>
   </si>
@@ -1852,6 +2331,16 @@
 Se por acaso essa imagem for usada no topo da matéria (banner principal) e você queira dar um tom mais jornalístico e contextualizado à fotografia:
     Texto Alternativo Principal (Atributo alt):
         Cartela de ovos brancos em destaque, ilustrando o crescimento recorde do consumo do alimento no Brasil.</t>
+  </si>
+  <si>
+    <t>Opção 1: Tratamento técnico como Elemento Puramente Decorativo (Recomendado)
+Se a imagem de banco de dados (stock image) serve puramente para ilustrar a matéria esteticamente ou criar uma quebra visual no texto, sem adicionar fatos novos à notícia, o padrão ideal é ocultá-la das tecnologias assistivas. Para fazer isso de forma correta e limpa, o campo de texto alternativo deve conter aspas vazias. Isso instrui o leitor de tela a ignorar o elemento de forma fluida, impedindo que ele leia códigos de programação ou nomes de arquivos confusos como "35.jpg".
+    Texto Alternativo (Código Alt Sugerido): ""
+    Comportamento no Leitor de Tela: O sintetizador de voz passará direto pela imagem, otimizando o tempo e o foco da sua leitura.
+Opção 2: Tratamento como Imagem de Banco de Dados de Contexto (Equidade Editorial)
+Caso a política do portal de notícias exija que imagens ilustrativas de banco de dados (como fotos de ovos ou granjas) também recebam uma descrição para fornecer uma experiência equivalente de ambientação sobre o tema (o agronegócio de ovos), o texto descritivo deve ser muito conciso e ir direto ao ponto, respeitando o limite ideal de caracteres:
+    Texto Alternativo Sugerido (até 150 caracteres):
+    Vários ovos de galinha brancos e vermelhos organizados lado a lado em uma bandeja de papelão.</t>
   </si>
   <si>
     <t>Opção 1: Descrição Sucinta Editorial (Padrão Recomendado da BBC para Equidade)
@@ -1896,6 +2385,10 @@
     <t>Contexto: O setor gastronômico de São Paulo prepara-se para o Dia das Mães com expectativas de aumento no faturamento entre 30% e 50%, conforme dados da Abrasel, motivando diversos estabelecimentos a oferecerem menus exclusivos e cortesias para a celebração. A seleção de restaurantes na capital abrange desde a culinária francesa e italiana, com pratos como pernil de cordeiro e massas frescas artesanais, até opções de gastronomia chinesa, portuguesa e brasileira, incluindo menus fechados em três tempos e pratos para compartilhamento familiar. Além das propostas culinárias específicas, como o tradicional bacalhau e receitas com frutos do mar, algumas casas promovem experiências sensoriais com música ao vivo e brindes de boas-vindas, como taças de vinho e espumante, visando atrair o público que busca celebrar a data em ambientes que variam do rústico ao sofisticado nos principais polos gastronômicos da cidade, como Jardins, Itaim Bibi e Pinheiros.</t>
   </si>
   <si>
+    <t>URL: https://www.cnnbrasil.com.br/viagemegastronomia/gastronomia/dia-das-maes-em-sao-paulo-confira-restaurantes-para-celebrar-a-data/
+Tipo de Imagem: Imagem Decorativa</t>
+  </si>
+  <si>
     <t>Contexto: O setor gastronômico de São Paulo prepara-se para o Dia das Mães com expectativas de aumento no faturamento entre 30% e 50%, conforme dados da Abrasel, motivando diversos estabelecimentos a oferecerem menus exclusivos e cortesias para a celebração. A seleção de restaurantes na capital abrange desde a culinária francesa e italiana, com pratos como pernil de cordeiro e massas frescas artesanais, até opções de gastronomia chinesa, portuguesa e brasileira, incluindo menus fechados em três tempos e pratos para compartilhamento familiar. Além das propostas culinárias específicas, como o tradicional bacalhau e receitas com frutos do mar, algumas casas promovem experiências sensoriais com música ao vivo e brindes de boas-vindas, como taças de vinho e espumante, visando atrair o público que busca celebrar a data em ambientes que variam do rústico ao sofisticado nos principais polos gastronômicos da cidade, como Jardins, Itaim Bibi e Pinheiros.
 Tipo de Imagem: Imagem Decorativa</t>
   </si>
@@ -1904,6 +2397,13 @@
     Prato de massa artesanal com molho de tomate, manjericão e queijo ralado, servido em mesa de madeira rústica com taças de vinho ao fundo.
 Opção 2: Descrição Longa (Se a imagem for central à experiência sensorial)
     Em um ambiente de iluminação quente e acolhedora, um prato fundo de cerâmica branca destaca uma massa longa envolta em molho de tomate vibrante. Sobre o prato, folhas de manjericão fresco e lascas de queijo. Ao fundo, de forma levemente desfocada, duas taças de vinho tinto e talheres de prata sobre uma mesa de madeira escura, sugerindo um almoço festivo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opção 1: Tratamento estrito como Imagem Puramente Decorativa (Recomendado)
+Se a imagem cumpre uma função estritamente estética no layout da página (como quebra de texto, borda ou elemento de design redundante) e sua ausência não altera o entendimento do artigo , a diretriz indica que o campo de texto alternativo não deve ser deixado em branco, mas sim preenchido com aspas vazias para instruir o leitor de tela a ignorá-la. Isso evita a leitura desnecessária de códigos ou caminhos de arquivos confusos.  
+Código Alt Sugerido: ""   Comportamento do Leitor de Tela: O sintetizador de voz passará diretamente pela imagem de forma fluida, sem anúncios desnecessários.  
+Opção 2: Tratamento contextualizado como Banco de Imagens (Stock Photo)
+Em portais de notícias brasileiros, muitas fotos ilustrativas de pratos de comida ou restaurantes são utilizadas para "quebrar o texto" ou ilustrar matérias de gastronomia. Para garantir uma experiência de igualdade para os usuários que apreciam saber o tom e a ambientação da matéria , podemos fornecer uma descrição concisa do conteúdo visual presente no arquivo enviado (36.jpg) focado no contexto do Dia das Mães:  Texto Alternativo Sugerido (até 150 caracteres):Prato gourmet de massa fresca decorado com folhas de manjericão, servido em uma mesa iluminada de restaurante.   </t>
   </si>
   <si>
     <t>Opção 1: Descrição Sucinta de Ambiente (Padrão Recomendado pela BBC)
@@ -1930,23 +2430,27 @@
 Trabalho limpo e focado na usabilidade! Se tiver mais imagens dessa cobertura ou de outras editorias, manda para cá.</t>
   </si>
   <si>
-    <t>Tipo de Prompt 1</t>
-  </si>
-  <si>
-    <t>Zero-Shot Prompting</t>
-  </si>
-  <si>
-    <t>Tipo de Prompt 2</t>
-  </si>
-  <si>
-    <t>Tipo de Prompt 3</t>
+    <t>Prompt Base</t>
+  </si>
+  <si>
+    <t>Analise primeiramente a imagem anexada. Use a URL https://www.cnnbrasil.com.br/nacional/cnn-brasil-lanca-nova-campanha-e-nova-assinatura/ e o tipo de imagem Imagem de Texto apenas como contexto extra para entender onde ela está inserida, mas descreva estritamente o que está visível no arquivo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gere um alt text para a imagem analisando seu conteúdo visual, o contexto obtido pela URL associada, o tipo de imagem e a diretrizes de acessibilidade da BBC. Produza uma descrição objetiva, acessível e contextualizada, destacando apenas as informações essenciais para a compreensão da imagem.  Sua resposta deve consistir em apenas nos alt texts gerados.
+</t>
+  </si>
+  <si>
+    <t>Gere um alt text para a imagem analisando seu conteúdo visual, o contexto obtido pela URL associada, o tipo de imagem e as Diretrizes da Carolina. Produza uma descrição objetiva, acessível e contextualizada, destacando apenas as informações essenciais para a compreensão da imagem. Sua resposta deve consistir em apenas nos alt texts gerados.</t>
+  </si>
+  <si>
+    <t>Gere um alt text para a imagem analisando seu conteúdo visual, o contexto obtido pela URL associada, o tipo de imagem e as Guidelines do Section 508. Produza uma descrição objetiva, acessível e contextualizada, destacando apenas as informações essenciais para a compreensão da imagem. Sua resposta deve consistir em apenas nos alt texts gerados.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -1966,11 +2470,12 @@
     </font>
     <font>
       <u/>
-      <color rgb="FF0000FF"/>
+      <color rgb="FF434343"/>
       <name val="Roboto"/>
     </font>
     <font>
       <u/>
+      <sz val="11.0"/>
       <color rgb="FF434343"/>
       <name val="Roboto"/>
     </font>
@@ -1978,6 +2483,17 @@
       <u/>
       <color rgb="FF0000FF"/>
       <name val="Roboto"/>
+    </font>
+    <font>
+      <u/>
+      <color rgb="FF0000FF"/>
+      <name val="Roboto"/>
+    </font>
+    <font>
+      <sz val="10.0"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <color theme="1"/>
@@ -1998,7 +2514,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="26">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -2029,6 +2545,9 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="49" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="49" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
@@ -2050,14 +2569,29 @@
     <xf borderId="0" fillId="0" fontId="5" numFmtId="49" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="49" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="7" numFmtId="49" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="49" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf quotePrefix="1" borderId="0" fillId="0" fontId="1" numFmtId="49" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2144,8 +2678,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:P37" displayName="Tabela_1" name="Tabela_1" id="1">
-  <tableColumns count="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:V37" displayName="Tabela_1" name="Tabela_1" id="1">
+  <tableColumns count="22">
     <tableColumn name="ID" id="1"/>
     <tableColumn name="Título Noticia" id="2"/>
     <tableColumn name="Portal Originario" id="3"/>
@@ -2157,18 +2691,24 @@
     <tableColumn name="Alt Text Original" id="9"/>
     <tableColumn name="Caption Imagem" id="10"/>
     <tableColumn name="Resumo da Noticia" id="11"/>
-    <tableColumn name="Prompt sem Contexto" id="12"/>
-    <tableColumn name="Prompt com Contexto" id="13"/>
-    <tableColumn name="Alt Text IA 1 - Tese da Carolina" id="14"/>
-    <tableColumn name="Alt Text IA 2 - BBC" id="15"/>
-    <tableColumn name="Alt Text IA 3 - Section 508" id="16"/>
+    <tableColumn name="Prompt para Gemini Sem Gems" id="12"/>
+    <tableColumn name="Prompt com URL" id="13"/>
+    <tableColumn name="Prompt com Contexto" id="14"/>
+    <tableColumn name="Alt Text 1 - Tese da Carolina" id="15"/>
+    <tableColumn name="Alt Text 1 URL - Tese da Carolina" id="16"/>
+    <tableColumn name="Alt Text IA 1 Contexto - Tese da Carolina" id="17"/>
+    <tableColumn name="Alt Text 2 URL - BBC" id="18"/>
+    <tableColumn name="Alt Text IA 2 - BBC" id="19"/>
+    <tableColumn name="Alt Text 3 - Section 508" id="20"/>
+    <tableColumn name="Alt Text 3 URL - Section 508" id="21"/>
+    <tableColumn name="Alt Text IA 3 Contexto - Section 508" id="22"/>
   </tableColumns>
   <tableStyleInfo name="Página1-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="S2:U3" displayName="Tabela_2" name="Tabela_2" id="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="Y2:AA3" displayName="Tabela_2" name="Tabela_2" id="2">
   <tableColumns count="3">
     <tableColumn name="Instruções do Gems - Tese da Carolina" id="1"/>
     <tableColumn name="Instruções do Gems - BCC News" id="2"/>
@@ -2376,6 +2916,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
@@ -2389,14 +2930,14 @@
     <col customWidth="1" min="9" max="9" width="21.0"/>
     <col customWidth="1" min="10" max="10" width="22.88"/>
     <col customWidth="1" min="11" max="11" width="23.63"/>
-    <col customWidth="1" min="12" max="12" width="27.75"/>
+    <col customWidth="1" min="12" max="12" width="33.63"/>
     <col customWidth="1" min="13" max="13" width="35.13"/>
-    <col customWidth="1" min="14" max="14" width="23.25"/>
+    <col customWidth="1" min="14" max="14" width="34.38"/>
     <col customWidth="1" min="15" max="15" width="35.13"/>
     <col customWidth="1" min="16" max="16" width="34.88"/>
     <col customWidth="1" min="17" max="17" width="29.63"/>
-    <col customWidth="1" min="18" max="18" width="26.38"/>
-    <col customWidth="1" min="19" max="19" width="24.38"/>
+    <col customWidth="1" min="18" max="18" width="45.63"/>
+    <col customWidth="1" min="19" max="19" width="40.13"/>
     <col customWidth="1" min="20" max="20" width="43.13"/>
     <col customWidth="1" min="21" max="21" width="40.13"/>
     <col customWidth="1" min="22" max="22" width="36.88"/>
@@ -2439,17 +2980,35 @@
       <c r="L1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="M1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="4" t="s">
+      <c r="O1" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="4" t="s">
+      <c r="P1" s="3" t="s">
         <v>15</v>
+      </c>
+      <c r="Q1" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" s="4" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="2" ht="22.5" customHeight="1">
@@ -2457,1745 +3016,2110 @@
         <v>1.0</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="K2" s="6" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="L2" s="9"/>
       <c r="M2" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="N2" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="O2" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="P2" s="9" t="s">
-        <v>29</v>
+        <v>32</v>
+      </c>
+      <c r="N2" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="O2" s="10"/>
+      <c r="P2" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q2" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="R2" s="10" t="s">
+        <v>36</v>
       </c>
       <c r="S2" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="T2" s="10" t="s">
-        <v>31</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="T2" s="10"/>
       <c r="U2" s="10" t="s">
-        <v>32</v>
+        <v>38</v>
+      </c>
+      <c r="V2" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="Y2" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="Z2" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="AA2" s="11" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="3" ht="22.5" customHeight="1">
-      <c r="A3" s="11">
+      <c r="A3" s="12">
         <f t="shared" ref="A3:A37" si="1">A2+1</f>
         <v>2</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D3" s="12" t="s">
-        <v>34</v>
+        <v>23</v>
+      </c>
+      <c r="D3" s="13" t="s">
+        <v>44</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="J3" s="6" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="K3" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="L3" s="9"/>
-      <c r="M3" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="N3" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="O3" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="P3" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="S3" s="13" t="s">
-        <v>44</v>
-      </c>
-      <c r="T3" s="13" t="s">
-        <v>45</v>
-      </c>
-      <c r="U3" s="13" t="s">
-        <v>46</v>
+        <v>49</v>
+      </c>
+      <c r="L3" s="10"/>
+      <c r="M3" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="N3" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="O3" s="10"/>
+      <c r="P3" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q3" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="R3" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="S3" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="T3" s="10"/>
+      <c r="U3" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="V3" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="Y3" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="Z3" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="AA3" s="14" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="4" ht="22.5" customHeight="1">
-      <c r="A4" s="11">
+      <c r="A4" s="12">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
-      <c r="B4" s="14" t="s">
-        <v>47</v>
-      </c>
-      <c r="C4" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4" s="16" t="s">
-        <v>48</v>
-      </c>
-      <c r="E4" s="16" t="s">
-        <v>49</v>
-      </c>
-      <c r="F4" s="15" t="s">
-        <v>20</v>
+      <c r="B4" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="C4" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="E4" s="17" t="s">
+        <v>63</v>
+      </c>
+      <c r="F4" s="16" t="s">
+        <v>26</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>50</v>
+        <v>64</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>51</v>
+        <v>65</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="J4" s="14" t="s">
-        <v>53</v>
+        <v>66</v>
+      </c>
+      <c r="J4" s="15" t="s">
+        <v>67</v>
       </c>
       <c r="K4" s="6" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="L4" s="9"/>
       <c r="M4" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="N4" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="O4" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="P4" s="9" t="s">
-        <v>58</v>
+        <v>69</v>
+      </c>
+      <c r="N4" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="O4" s="10"/>
+      <c r="P4" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q4" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="R4" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="S4" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="T4" s="10"/>
+      <c r="U4" s="10"/>
+      <c r="V4" s="10" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="5" ht="243.0" customHeight="1">
-      <c r="A5" s="11">
+      <c r="A5" s="12">
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>59</v>
+        <v>76</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="E5" s="12" t="s">
-        <v>61</v>
+        <v>23</v>
+      </c>
+      <c r="D5" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>78</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>62</v>
+        <v>79</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>63</v>
+        <v>80</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>64</v>
+        <v>81</v>
       </c>
       <c r="J5" s="6" t="s">
-        <v>64</v>
+        <v>81</v>
       </c>
       <c r="K5" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="L5" s="6"/>
-      <c r="M5" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="N5" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="O5" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="P5" s="9" t="s">
-        <v>69</v>
+        <v>82</v>
+      </c>
+      <c r="L5" s="10"/>
+      <c r="M5" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="N5" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="O5" s="6"/>
+      <c r="P5" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="Q5" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="R5" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="S5" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="T5" s="10"/>
+      <c r="U5" s="10"/>
+      <c r="V5" s="10" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="6" ht="22.5" customHeight="1">
-      <c r="A6" s="11">
+      <c r="A6" s="12">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D6" s="12" t="s">
-        <v>71</v>
-      </c>
-      <c r="E6" s="12" t="s">
-        <v>72</v>
+        <v>23</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>92</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>62</v>
+        <v>79</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>73</v>
+        <v>93</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>50</v>
+        <v>64</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>74</v>
+        <v>94</v>
       </c>
       <c r="J6" s="6" t="s">
-        <v>75</v>
+        <v>95</v>
       </c>
       <c r="K6" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="L6" s="6"/>
-      <c r="M6" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="N6" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="O6" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="P6" s="9" t="s">
-        <v>80</v>
+        <v>96</v>
+      </c>
+      <c r="L6" s="10"/>
+      <c r="M6" s="10" t="s">
+        <v>97</v>
+      </c>
+      <c r="N6" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="O6" s="6"/>
+      <c r="P6" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="Q6" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="R6" s="6"/>
+      <c r="S6" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="T6" s="10"/>
+      <c r="U6" s="10"/>
+      <c r="V6" s="10" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="7" ht="22.5" customHeight="1">
-      <c r="A7" s="11">
+      <c r="A7" s="12">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="C7" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="E7" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="F7" s="15" t="s">
-        <v>62</v>
+        <v>103</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="D7" s="13" t="s">
+        <v>104</v>
+      </c>
+      <c r="E7" s="18" t="s">
+        <v>105</v>
+      </c>
+      <c r="F7" s="16" t="s">
+        <v>79</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>84</v>
+        <v>106</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>85</v>
+        <v>107</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>86</v>
+        <v>108</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>86</v>
+        <v>108</v>
       </c>
       <c r="K7" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="L7" s="6"/>
-      <c r="M7" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="N7" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="O7" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="P7" s="9" t="s">
-        <v>91</v>
+        <v>109</v>
+      </c>
+      <c r="L7" s="15"/>
+      <c r="M7" s="15" t="s">
+        <v>110</v>
+      </c>
+      <c r="N7" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="O7" s="10"/>
+      <c r="P7" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="Q7" s="10" t="s">
+        <v>113</v>
+      </c>
+      <c r="R7" s="6"/>
+      <c r="S7" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="T7" s="10"/>
+      <c r="U7" s="10"/>
+      <c r="V7" s="10" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="8" ht="22.5" customHeight="1">
-      <c r="A8" s="11">
+      <c r="A8" s="12">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>92</v>
+        <v>116</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>93</v>
-      </c>
-      <c r="E8" s="8" t="s">
-        <v>94</v>
+        <v>23</v>
+      </c>
+      <c r="D8" s="18" t="s">
+        <v>117</v>
+      </c>
+      <c r="E8" s="18" t="s">
+        <v>118</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>95</v>
+        <v>119</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>96</v>
+        <v>120</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>50</v>
+        <v>64</v>
       </c>
       <c r="I8" s="6" t="s">
-        <v>97</v>
+        <v>121</v>
       </c>
       <c r="J8" s="6" t="s">
-        <v>98</v>
+        <v>122</v>
       </c>
       <c r="K8" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="L8" s="6"/>
-      <c r="M8" s="9" t="s">
-        <v>100</v>
-      </c>
-      <c r="N8" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="O8" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="P8" s="9" t="s">
-        <v>103</v>
+        <v>123</v>
+      </c>
+      <c r="L8" s="10"/>
+      <c r="M8" s="10" t="s">
+        <v>124</v>
+      </c>
+      <c r="N8" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="O8" s="6"/>
+      <c r="P8" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="Q8" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="R8" s="6"/>
+      <c r="S8" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="T8" s="10"/>
+      <c r="U8" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="V8" s="10" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="9" ht="22.5" customHeight="1">
-      <c r="A9" s="11">
+      <c r="A9" s="12">
         <f t="shared" si="1"/>
         <v>8</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>104</v>
+        <v>131</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>105</v>
-      </c>
-      <c r="E9" s="8" t="s">
-        <v>106</v>
+        <v>23</v>
+      </c>
+      <c r="D9" s="18" t="s">
+        <v>132</v>
+      </c>
+      <c r="E9" s="18" t="s">
+        <v>133</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>95</v>
+        <v>119</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>107</v>
+        <v>134</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>107</v>
+        <v>134</v>
       </c>
       <c r="I9" s="6" t="s">
-        <v>108</v>
+        <v>135</v>
       </c>
       <c r="J9" s="6" t="s">
-        <v>109</v>
+        <v>136</v>
       </c>
       <c r="K9" s="6" t="s">
-        <v>110</v>
-      </c>
-      <c r="L9" s="6"/>
-      <c r="M9" s="9" t="s">
-        <v>111</v>
-      </c>
-      <c r="N9" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="O9" s="6" t="s">
-        <v>113</v>
-      </c>
-      <c r="P9" s="9" t="s">
-        <v>114</v>
+        <v>137</v>
+      </c>
+      <c r="L9" s="10"/>
+      <c r="M9" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="N9" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="O9" s="6"/>
+      <c r="P9" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="Q9" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="R9" s="6"/>
+      <c r="S9" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="T9" s="10"/>
+      <c r="U9" s="10"/>
+      <c r="V9" s="10" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="10" ht="22.5" customHeight="1">
-      <c r="A10" s="11">
+      <c r="A10" s="12">
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>115</v>
-      </c>
-      <c r="C10" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="D10" s="16" t="s">
-        <v>116</v>
-      </c>
-      <c r="E10" s="16" t="s">
-        <v>117</v>
-      </c>
-      <c r="F10" s="15" t="s">
-        <v>95</v>
+        <v>144</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="D10" s="17" t="s">
+        <v>145</v>
+      </c>
+      <c r="E10" s="17" t="s">
+        <v>146</v>
+      </c>
+      <c r="F10" s="16" t="s">
+        <v>119</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>118</v>
+        <v>147</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>85</v>
+        <v>107</v>
       </c>
       <c r="I10" s="6" t="s">
-        <v>119</v>
+        <v>148</v>
       </c>
       <c r="J10" s="6" t="s">
-        <v>119</v>
+        <v>148</v>
       </c>
       <c r="K10" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="L10" s="6"/>
-      <c r="M10" s="9" t="s">
-        <v>121</v>
-      </c>
-      <c r="N10" s="9" t="s">
-        <v>122</v>
-      </c>
-      <c r="O10" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="P10" s="9"/>
+        <v>149</v>
+      </c>
+      <c r="L10" s="10"/>
+      <c r="M10" s="10" t="s">
+        <v>150</v>
+      </c>
+      <c r="N10" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="O10" s="10"/>
+      <c r="P10" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="Q10" s="10" t="s">
+        <v>153</v>
+      </c>
+      <c r="R10" s="6"/>
+      <c r="S10" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="T10" s="10"/>
+      <c r="U10" s="10"/>
+      <c r="V10" s="10"/>
     </row>
     <row r="11" ht="22.5" customHeight="1">
-      <c r="A11" s="11">
+      <c r="A11" s="12">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>124</v>
+        <v>155</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D11" s="8" t="s">
-        <v>125</v>
-      </c>
-      <c r="E11" s="8" t="s">
-        <v>126</v>
+        <v>23</v>
+      </c>
+      <c r="D11" s="18" t="s">
+        <v>156</v>
+      </c>
+      <c r="E11" s="18" t="s">
+        <v>157</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>127</v>
+        <v>158</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>50</v>
+        <v>64</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>50</v>
+        <v>64</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>128</v>
+        <v>159</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>129</v>
+        <v>160</v>
       </c>
       <c r="K11" s="6" t="s">
-        <v>130</v>
-      </c>
-      <c r="L11" s="6"/>
-      <c r="M11" s="9" t="s">
-        <v>131</v>
-      </c>
-      <c r="N11" s="6" t="s">
-        <v>132</v>
-      </c>
-      <c r="O11" s="6" t="s">
-        <v>133</v>
-      </c>
-      <c r="P11" s="9"/>
+        <v>161</v>
+      </c>
+      <c r="L11" s="10"/>
+      <c r="M11" s="10" t="s">
+        <v>162</v>
+      </c>
+      <c r="N11" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="O11" s="6"/>
+      <c r="P11" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="Q11" s="6" t="s">
+        <v>165</v>
+      </c>
+      <c r="R11" s="6"/>
+      <c r="S11" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="T11" s="10"/>
+      <c r="U11" s="10"/>
+      <c r="V11" s="10"/>
     </row>
     <row r="12" ht="22.5" customHeight="1">
-      <c r="A12" s="11">
+      <c r="A12" s="12">
         <f t="shared" si="1"/>
         <v>11</v>
       </c>
       <c r="B12" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D12" s="17" t="s">
+        <v>168</v>
+      </c>
+      <c r="E12" s="18" t="s">
+        <v>169</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="G12" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="C12" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D12" s="16" t="s">
-        <v>135</v>
-      </c>
-      <c r="E12" s="8" t="s">
-        <v>136</v>
-      </c>
-      <c r="F12" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="G12" s="6" t="s">
-        <v>107</v>
-      </c>
       <c r="H12" s="6" t="s">
-        <v>107</v>
+        <v>134</v>
       </c>
       <c r="I12" s="6" t="s">
-        <v>137</v>
+        <v>170</v>
       </c>
       <c r="J12" s="6" t="s">
-        <v>138</v>
+        <v>171</v>
       </c>
       <c r="K12" s="6" t="s">
-        <v>139</v>
-      </c>
-      <c r="L12" s="6"/>
-      <c r="M12" s="9" t="s">
-        <v>140</v>
-      </c>
-      <c r="N12" s="6" t="s">
-        <v>141</v>
-      </c>
-      <c r="O12" s="6" t="s">
-        <v>142</v>
-      </c>
-      <c r="P12" s="9"/>
+        <v>172</v>
+      </c>
+      <c r="L12" s="10"/>
+      <c r="M12" s="10" t="s">
+        <v>173</v>
+      </c>
+      <c r="N12" s="10" t="s">
+        <v>174</v>
+      </c>
+      <c r="O12" s="6"/>
+      <c r="P12" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="Q12" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="R12" s="6"/>
+      <c r="S12" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="T12" s="10"/>
+      <c r="U12" s="10"/>
+      <c r="V12" s="10"/>
     </row>
     <row r="13" ht="22.5" customHeight="1">
-      <c r="A13" s="11">
+      <c r="A13" s="12">
         <f t="shared" si="1"/>
         <v>12</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="C13" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="D13" s="16" t="s">
-        <v>144</v>
-      </c>
-      <c r="E13" s="16" t="s">
-        <v>145</v>
-      </c>
-      <c r="F13" s="15" t="s">
-        <v>127</v>
+        <v>178</v>
+      </c>
+      <c r="C13" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="D13" s="17" t="s">
+        <v>179</v>
+      </c>
+      <c r="E13" s="17" t="s">
+        <v>180</v>
+      </c>
+      <c r="F13" s="16" t="s">
+        <v>158</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>85</v>
+        <v>107</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>85</v>
+        <v>107</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>146</v>
+        <v>181</v>
       </c>
       <c r="J13" s="6" t="s">
-        <v>147</v>
+        <v>182</v>
       </c>
       <c r="K13" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="L13" s="9"/>
-      <c r="M13" s="9" t="s">
-        <v>149</v>
-      </c>
-      <c r="N13" s="9" t="s">
-        <v>150</v>
-      </c>
-      <c r="O13" s="6" t="s">
-        <v>151</v>
-      </c>
-      <c r="P13" s="17"/>
+        <v>183</v>
+      </c>
+      <c r="L13" s="10"/>
+      <c r="M13" s="10" t="s">
+        <v>184</v>
+      </c>
+      <c r="N13" s="10" t="s">
+        <v>185</v>
+      </c>
+      <c r="O13" s="19"/>
+      <c r="P13" s="19" t="s">
+        <v>186</v>
+      </c>
+      <c r="Q13" s="10" t="s">
+        <v>187</v>
+      </c>
+      <c r="R13" s="6"/>
+      <c r="S13" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="T13" s="20"/>
+      <c r="U13" s="20"/>
+      <c r="V13" s="20"/>
     </row>
     <row r="14" ht="22.5" customHeight="1">
-      <c r="A14" s="11">
+      <c r="A14" s="12">
         <f t="shared" si="1"/>
         <v>13</v>
       </c>
-      <c r="B14" s="18" t="s">
-        <v>152</v>
+      <c r="B14" s="21" t="s">
+        <v>189</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>153</v>
-      </c>
-      <c r="D14" s="8" t="s">
-        <v>154</v>
-      </c>
-      <c r="E14" s="8" t="s">
-        <v>155</v>
+        <v>190</v>
+      </c>
+      <c r="D14" s="18" t="s">
+        <v>191</v>
+      </c>
+      <c r="E14" s="18" t="s">
+        <v>192</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>50</v>
+        <v>64</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>50</v>
+        <v>64</v>
       </c>
       <c r="I14" s="6" t="s">
-        <v>156</v>
+        <v>193</v>
       </c>
       <c r="J14" s="6" t="s">
-        <v>156</v>
+        <v>193</v>
       </c>
       <c r="K14" s="6" t="s">
-        <v>157</v>
-      </c>
-      <c r="L14" s="9"/>
-      <c r="M14" s="9" t="s">
-        <v>158</v>
-      </c>
-      <c r="N14" s="9" t="s">
-        <v>159</v>
-      </c>
-      <c r="O14" s="6" t="s">
-        <v>160</v>
-      </c>
-      <c r="P14" s="17"/>
+        <v>194</v>
+      </c>
+      <c r="L14" s="10"/>
+      <c r="M14" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="N14" s="10" t="s">
+        <v>196</v>
+      </c>
+      <c r="O14" s="19"/>
+      <c r="P14" s="19" t="s">
+        <v>197</v>
+      </c>
+      <c r="Q14" s="10" t="s">
+        <v>198</v>
+      </c>
+      <c r="R14" s="6"/>
+      <c r="S14" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="T14" s="20"/>
+      <c r="U14" s="20"/>
+      <c r="V14" s="20"/>
     </row>
     <row r="15" ht="22.5" customHeight="1">
-      <c r="A15" s="11">
+      <c r="A15" s="12">
         <f t="shared" si="1"/>
         <v>14</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>161</v>
+        <v>200</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>153</v>
-      </c>
-      <c r="D15" s="8" t="s">
-        <v>162</v>
-      </c>
-      <c r="E15" s="8" t="s">
-        <v>163</v>
+        <v>190</v>
+      </c>
+      <c r="D15" s="18" t="s">
+        <v>201</v>
+      </c>
+      <c r="E15" s="18" t="s">
+        <v>202</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>50</v>
+        <v>64</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>50</v>
+        <v>64</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>164</v>
+        <v>203</v>
       </c>
       <c r="J15" s="6" t="s">
-        <v>164</v>
+        <v>203</v>
       </c>
       <c r="K15" s="6" t="s">
-        <v>165</v>
-      </c>
-      <c r="L15" s="9"/>
-      <c r="M15" s="9" t="s">
-        <v>166</v>
-      </c>
-      <c r="N15" s="9" t="s">
-        <v>167</v>
-      </c>
-      <c r="O15" s="6" t="s">
-        <v>168</v>
-      </c>
-      <c r="P15" s="17"/>
+        <v>204</v>
+      </c>
+      <c r="L15" s="10"/>
+      <c r="M15" s="10" t="s">
+        <v>205</v>
+      </c>
+      <c r="N15" s="10" t="s">
+        <v>206</v>
+      </c>
+      <c r="O15" s="10"/>
+      <c r="P15" s="10" t="s">
+        <v>207</v>
+      </c>
+      <c r="Q15" s="10" t="s">
+        <v>208</v>
+      </c>
+      <c r="R15" s="6"/>
+      <c r="S15" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="T15" s="20"/>
+      <c r="U15" s="20"/>
+      <c r="V15" s="20"/>
     </row>
     <row r="16" ht="22.5" customHeight="1">
-      <c r="A16" s="11">
+      <c r="A16" s="12">
         <f t="shared" si="1"/>
         <v>15</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>169</v>
+        <v>210</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>153</v>
-      </c>
-      <c r="D16" s="16" t="s">
-        <v>170</v>
-      </c>
-      <c r="E16" s="16" t="s">
-        <v>171</v>
-      </c>
-      <c r="F16" s="15" t="s">
-        <v>20</v>
+        <v>190</v>
+      </c>
+      <c r="D16" s="17" t="s">
+        <v>211</v>
+      </c>
+      <c r="E16" s="17" t="s">
+        <v>212</v>
+      </c>
+      <c r="F16" s="16" t="s">
+        <v>26</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>172</v>
+        <v>213</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>51</v>
+        <v>65</v>
       </c>
       <c r="I16" s="6" t="s">
-        <v>173</v>
+        <v>214</v>
       </c>
       <c r="J16" s="6" t="s">
-        <v>174</v>
+        <v>215</v>
       </c>
       <c r="K16" s="6" t="s">
-        <v>175</v>
-      </c>
-      <c r="L16" s="9"/>
-      <c r="M16" s="9" t="s">
-        <v>176</v>
-      </c>
-      <c r="N16" s="9" t="s">
-        <v>177</v>
-      </c>
-      <c r="O16" s="6" t="s">
-        <v>178</v>
-      </c>
-      <c r="P16" s="17"/>
+        <v>216</v>
+      </c>
+      <c r="L16" s="10"/>
+      <c r="M16" s="10" t="s">
+        <v>217</v>
+      </c>
+      <c r="N16" s="10" t="s">
+        <v>218</v>
+      </c>
+      <c r="O16" s="10"/>
+      <c r="P16" s="10" t="s">
+        <v>219</v>
+      </c>
+      <c r="Q16" s="10" t="s">
+        <v>220</v>
+      </c>
+      <c r="R16" s="6"/>
+      <c r="S16" s="6" t="s">
+        <v>221</v>
+      </c>
+      <c r="T16" s="20"/>
+      <c r="U16" s="20"/>
+      <c r="V16" s="20"/>
     </row>
     <row r="17" ht="22.5" customHeight="1">
-      <c r="A17" s="11">
+      <c r="A17" s="12">
         <f t="shared" si="1"/>
         <v>16</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>179</v>
+        <v>222</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>153</v>
-      </c>
-      <c r="D17" s="8" t="s">
-        <v>180</v>
-      </c>
-      <c r="E17" s="8" t="s">
-        <v>181</v>
+        <v>190</v>
+      </c>
+      <c r="D17" s="18" t="s">
+        <v>223</v>
+      </c>
+      <c r="E17" s="18" t="s">
+        <v>224</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>62</v>
+        <v>79</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>182</v>
+        <v>225</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>50</v>
+        <v>64</v>
       </c>
       <c r="I17" s="6" t="s">
-        <v>183</v>
+        <v>226</v>
       </c>
       <c r="J17" s="6" t="s">
-        <v>183</v>
+        <v>226</v>
       </c>
       <c r="K17" s="6" t="s">
-        <v>184</v>
-      </c>
-      <c r="L17" s="9"/>
-      <c r="M17" s="9" t="s">
-        <v>185</v>
-      </c>
-      <c r="N17" s="9" t="s">
-        <v>186</v>
-      </c>
-      <c r="O17" s="6" t="s">
-        <v>187</v>
-      </c>
-      <c r="P17" s="17"/>
+        <v>227</v>
+      </c>
+      <c r="L17" s="10"/>
+      <c r="M17" s="10" t="s">
+        <v>228</v>
+      </c>
+      <c r="N17" s="10" t="s">
+        <v>229</v>
+      </c>
+      <c r="O17" s="10"/>
+      <c r="P17" s="10" t="s">
+        <v>230</v>
+      </c>
+      <c r="Q17" s="10" t="s">
+        <v>231</v>
+      </c>
+      <c r="R17" s="6"/>
+      <c r="S17" s="6" t="s">
+        <v>232</v>
+      </c>
+      <c r="T17" s="20"/>
+      <c r="U17" s="20"/>
+      <c r="V17" s="20"/>
     </row>
     <row r="18" ht="22.5" customHeight="1">
-      <c r="A18" s="11">
+      <c r="A18" s="12">
         <f t="shared" si="1"/>
         <v>17</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>188</v>
+        <v>233</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>153</v>
-      </c>
-      <c r="D18" s="8" t="s">
-        <v>189</v>
-      </c>
-      <c r="E18" s="8" t="s">
         <v>190</v>
       </c>
+      <c r="D18" s="13" t="s">
+        <v>234</v>
+      </c>
+      <c r="E18" s="18" t="s">
+        <v>235</v>
+      </c>
       <c r="F18" s="7" t="s">
-        <v>62</v>
+        <v>79</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>191</v>
+        <v>236</v>
       </c>
       <c r="H18" s="6" t="s">
-        <v>50</v>
+        <v>64</v>
       </c>
       <c r="I18" s="6" t="s">
-        <v>192</v>
+        <v>237</v>
       </c>
       <c r="J18" s="6" t="s">
-        <v>192</v>
+        <v>237</v>
       </c>
       <c r="K18" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="L18" s="9"/>
-      <c r="M18" s="9" t="s">
-        <v>194</v>
-      </c>
-      <c r="N18" s="9" t="s">
-        <v>195</v>
-      </c>
-      <c r="O18" s="6" t="s">
-        <v>196</v>
-      </c>
-      <c r="P18" s="17"/>
+        <v>238</v>
+      </c>
+      <c r="L18" s="10"/>
+      <c r="M18" s="10" t="s">
+        <v>239</v>
+      </c>
+      <c r="N18" s="10" t="s">
+        <v>240</v>
+      </c>
+      <c r="O18" s="10"/>
+      <c r="P18" s="10" t="s">
+        <v>241</v>
+      </c>
+      <c r="Q18" s="10" t="s">
+        <v>242</v>
+      </c>
+      <c r="R18" s="6"/>
+      <c r="S18" s="6" t="s">
+        <v>243</v>
+      </c>
+      <c r="T18" s="20"/>
+      <c r="U18" s="20"/>
+      <c r="V18" s="20"/>
     </row>
     <row r="19" ht="22.5" customHeight="1">
-      <c r="A19" s="11">
+      <c r="A19" s="12">
         <f t="shared" si="1"/>
         <v>18</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>197</v>
+        <v>244</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>153</v>
-      </c>
-      <c r="D19" s="16" t="s">
-        <v>198</v>
-      </c>
-      <c r="E19" s="16" t="s">
-        <v>199</v>
-      </c>
-      <c r="F19" s="15" t="s">
-        <v>62</v>
+        <v>190</v>
+      </c>
+      <c r="D19" s="13" t="s">
+        <v>245</v>
+      </c>
+      <c r="E19" s="17" t="s">
+        <v>246</v>
+      </c>
+      <c r="F19" s="16" t="s">
+        <v>79</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>200</v>
+        <v>247</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>51</v>
+        <v>65</v>
       </c>
       <c r="I19" s="6" t="s">
-        <v>201</v>
+        <v>248</v>
       </c>
       <c r="J19" s="6" t="s">
-        <v>202</v>
+        <v>249</v>
       </c>
       <c r="K19" s="6" t="s">
-        <v>203</v>
-      </c>
-      <c r="L19" s="9"/>
-      <c r="M19" s="9" t="s">
-        <v>204</v>
-      </c>
-      <c r="N19" s="9" t="s">
-        <v>205</v>
-      </c>
-      <c r="O19" s="6" t="s">
-        <v>206</v>
-      </c>
-      <c r="P19" s="17"/>
+        <v>250</v>
+      </c>
+      <c r="L19" s="10"/>
+      <c r="M19" s="10" t="s">
+        <v>251</v>
+      </c>
+      <c r="N19" s="10" t="s">
+        <v>252</v>
+      </c>
+      <c r="O19" s="10"/>
+      <c r="P19" s="10" t="s">
+        <v>253</v>
+      </c>
+      <c r="Q19" s="10" t="s">
+        <v>254</v>
+      </c>
+      <c r="R19" s="6"/>
+      <c r="S19" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="T19" s="20"/>
+      <c r="U19" s="20"/>
+      <c r="V19" s="20"/>
     </row>
     <row r="20" ht="22.5" customHeight="1">
-      <c r="A20" s="11">
+      <c r="A20" s="12">
         <f t="shared" si="1"/>
         <v>19</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>207</v>
+        <v>256</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>153</v>
-      </c>
-      <c r="D20" s="16" t="s">
-        <v>208</v>
-      </c>
-      <c r="E20" s="8" t="s">
-        <v>209</v>
+        <v>190</v>
+      </c>
+      <c r="D20" s="13" t="s">
+        <v>257</v>
+      </c>
+      <c r="E20" s="18" t="s">
+        <v>258</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>95</v>
+        <v>119</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>107</v>
+        <v>134</v>
       </c>
       <c r="H20" s="6" t="s">
-        <v>107</v>
+        <v>134</v>
       </c>
       <c r="I20" s="6" t="s">
-        <v>210</v>
+        <v>259</v>
       </c>
       <c r="J20" s="6" t="s">
-        <v>210</v>
+        <v>259</v>
       </c>
       <c r="K20" s="6" t="s">
-        <v>211</v>
-      </c>
-      <c r="L20" s="9"/>
-      <c r="M20" s="9" t="s">
-        <v>212</v>
-      </c>
-      <c r="N20" s="9" t="s">
-        <v>213</v>
-      </c>
-      <c r="O20" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="P20" s="17"/>
+        <v>260</v>
+      </c>
+      <c r="L20" s="10"/>
+      <c r="M20" s="10" t="s">
+        <v>261</v>
+      </c>
+      <c r="N20" s="10" t="s">
+        <v>262</v>
+      </c>
+      <c r="O20" s="10"/>
+      <c r="P20" s="10" t="s">
+        <v>263</v>
+      </c>
+      <c r="Q20" s="10" t="s">
+        <v>264</v>
+      </c>
+      <c r="R20" s="6"/>
+      <c r="S20" s="6" t="s">
+        <v>265</v>
+      </c>
+      <c r="T20" s="20"/>
+      <c r="U20" s="20"/>
+      <c r="V20" s="20"/>
     </row>
     <row r="21" ht="22.5" customHeight="1">
-      <c r="A21" s="11">
+      <c r="A21" s="12">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>215</v>
+        <v>266</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>153</v>
-      </c>
-      <c r="D21" s="8" t="s">
-        <v>216</v>
-      </c>
-      <c r="E21" s="8" t="s">
-        <v>217</v>
+        <v>190</v>
+      </c>
+      <c r="D21" s="13" t="s">
+        <v>267</v>
+      </c>
+      <c r="E21" s="18" t="s">
+        <v>268</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>95</v>
+        <v>119</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>107</v>
+        <v>134</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>107</v>
+        <v>134</v>
       </c>
       <c r="I21" s="6" t="s">
-        <v>218</v>
+        <v>269</v>
       </c>
       <c r="J21" s="6" t="s">
-        <v>218</v>
+        <v>269</v>
       </c>
       <c r="K21" s="6" t="s">
-        <v>219</v>
-      </c>
-      <c r="L21" s="9"/>
-      <c r="M21" s="9" t="s">
-        <v>220</v>
-      </c>
-      <c r="N21" s="9" t="s">
-        <v>221</v>
-      </c>
-      <c r="O21" s="6" t="s">
-        <v>222</v>
-      </c>
-      <c r="P21" s="17"/>
+        <v>270</v>
+      </c>
+      <c r="L21" s="10"/>
+      <c r="M21" s="10" t="s">
+        <v>271</v>
+      </c>
+      <c r="N21" s="10" t="s">
+        <v>272</v>
+      </c>
+      <c r="O21" s="10"/>
+      <c r="P21" s="10" t="s">
+        <v>273</v>
+      </c>
+      <c r="Q21" s="10" t="s">
+        <v>274</v>
+      </c>
+      <c r="R21" s="6"/>
+      <c r="S21" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="T21" s="20"/>
+      <c r="U21" s="20"/>
+      <c r="V21" s="20"/>
     </row>
     <row r="22" ht="22.5" customHeight="1">
-      <c r="A22" s="11">
+      <c r="A22" s="12">
         <f t="shared" si="1"/>
         <v>21</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>223</v>
+        <v>276</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>153</v>
-      </c>
-      <c r="D22" s="16" t="s">
-        <v>224</v>
-      </c>
-      <c r="E22" s="16" t="s">
-        <v>225</v>
-      </c>
-      <c r="F22" s="15" t="s">
-        <v>95</v>
+        <v>190</v>
+      </c>
+      <c r="D22" s="17" t="s">
+        <v>277</v>
+      </c>
+      <c r="E22" s="17" t="s">
+        <v>278</v>
+      </c>
+      <c r="F22" s="16" t="s">
+        <v>119</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>85</v>
+        <v>107</v>
       </c>
       <c r="H22" s="6" t="s">
-        <v>85</v>
+        <v>107</v>
       </c>
       <c r="I22" s="6" t="s">
-        <v>226</v>
+        <v>279</v>
       </c>
       <c r="J22" s="6" t="s">
-        <v>226</v>
+        <v>279</v>
       </c>
       <c r="K22" s="6" t="s">
-        <v>227</v>
-      </c>
-      <c r="L22" s="9"/>
-      <c r="M22" s="9" t="s">
-        <v>228</v>
-      </c>
-      <c r="N22" s="17"/>
-      <c r="O22" s="6" t="s">
-        <v>229</v>
-      </c>
-      <c r="P22" s="17"/>
+        <v>280</v>
+      </c>
+      <c r="L22" s="10"/>
+      <c r="M22" s="10" t="s">
+        <v>281</v>
+      </c>
+      <c r="N22" s="10" t="s">
+        <v>282</v>
+      </c>
+      <c r="O22" s="6"/>
+      <c r="P22" s="6" t="s">
+        <v>283</v>
+      </c>
+      <c r="Q22" s="20"/>
+      <c r="R22" s="6"/>
+      <c r="S22" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="T22" s="20"/>
+      <c r="U22" s="20"/>
+      <c r="V22" s="20"/>
     </row>
     <row r="23" ht="22.5" customHeight="1">
-      <c r="A23" s="11">
+      <c r="A23" s="12">
         <f t="shared" si="1"/>
         <v>22</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>230</v>
+        <v>285</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>153</v>
-      </c>
-      <c r="D23" s="8" t="s">
-        <v>231</v>
-      </c>
-      <c r="E23" s="16" t="s">
-        <v>232</v>
+        <v>190</v>
+      </c>
+      <c r="D23" s="18" t="s">
+        <v>286</v>
+      </c>
+      <c r="E23" s="17" t="s">
+        <v>287</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>127</v>
+        <v>158</v>
       </c>
       <c r="G23" s="6" t="s">
-        <v>85</v>
+        <v>107</v>
       </c>
       <c r="H23" s="6" t="s">
-        <v>85</v>
+        <v>107</v>
       </c>
       <c r="I23" s="6" t="s">
-        <v>233</v>
+        <v>288</v>
       </c>
       <c r="J23" s="6" t="s">
-        <v>234</v>
+        <v>289</v>
       </c>
       <c r="K23" s="6" t="s">
-        <v>235</v>
-      </c>
-      <c r="L23" s="6"/>
-      <c r="M23" s="6" t="s">
-        <v>236</v>
-      </c>
-      <c r="N23" s="17"/>
-      <c r="O23" s="6" t="s">
-        <v>237</v>
-      </c>
-      <c r="P23" s="17"/>
+        <v>290</v>
+      </c>
+      <c r="L23" s="10"/>
+      <c r="M23" s="10" t="s">
+        <v>291</v>
+      </c>
+      <c r="N23" s="10" t="s">
+        <v>292</v>
+      </c>
+      <c r="O23" s="20"/>
+      <c r="P23" s="20"/>
+      <c r="Q23" s="20"/>
+      <c r="R23" s="6"/>
+      <c r="S23" s="6" t="s">
+        <v>293</v>
+      </c>
+      <c r="T23" s="20"/>
+      <c r="U23" s="20"/>
+      <c r="V23" s="20"/>
     </row>
     <row r="24" ht="22.5" customHeight="1">
-      <c r="A24" s="11">
+      <c r="A24" s="12">
         <f t="shared" si="1"/>
         <v>23</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>238</v>
+        <v>294</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>153</v>
-      </c>
-      <c r="D24" s="8" t="s">
-        <v>239</v>
-      </c>
-      <c r="E24" s="8" t="s">
-        <v>240</v>
+        <v>190</v>
+      </c>
+      <c r="D24" s="18" t="s">
+        <v>295</v>
+      </c>
+      <c r="E24" s="18" t="s">
+        <v>296</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>127</v>
+        <v>158</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>172</v>
+        <v>213</v>
       </c>
       <c r="H24" s="6" t="s">
-        <v>172</v>
+        <v>213</v>
       </c>
       <c r="I24" s="6" t="s">
-        <v>241</v>
+        <v>297</v>
       </c>
       <c r="J24" s="6" t="s">
-        <v>241</v>
+        <v>297</v>
       </c>
       <c r="K24" s="6" t="s">
-        <v>242</v>
-      </c>
-      <c r="L24" s="6"/>
-      <c r="M24" s="6" t="s">
-        <v>243</v>
-      </c>
-      <c r="N24" s="17"/>
-      <c r="O24" s="6" t="s">
-        <v>244</v>
-      </c>
-      <c r="P24" s="17"/>
+        <v>298</v>
+      </c>
+      <c r="L24" s="10"/>
+      <c r="M24" s="10" t="s">
+        <v>299</v>
+      </c>
+      <c r="N24" s="6" t="s">
+        <v>300</v>
+      </c>
+      <c r="O24" s="20"/>
+      <c r="P24" s="20"/>
+      <c r="Q24" s="20"/>
+      <c r="R24" s="6"/>
+      <c r="S24" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="T24" s="20"/>
+      <c r="U24" s="20"/>
+      <c r="V24" s="20"/>
     </row>
     <row r="25" ht="22.5" customHeight="1">
-      <c r="A25" s="11">
+      <c r="A25" s="12">
         <f t="shared" si="1"/>
         <v>24</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>245</v>
+        <v>302</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>153</v>
-      </c>
-      <c r="D25" s="8" t="s">
-        <v>246</v>
-      </c>
-      <c r="E25" s="8" t="s">
-        <v>247</v>
+        <v>190</v>
+      </c>
+      <c r="D25" s="13" t="s">
+        <v>303</v>
+      </c>
+      <c r="E25" s="18" t="s">
+        <v>304</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>127</v>
+        <v>158</v>
       </c>
       <c r="G25" s="6" t="s">
-        <v>172</v>
+        <v>213</v>
       </c>
       <c r="H25" s="6" t="s">
-        <v>172</v>
+        <v>213</v>
       </c>
       <c r="I25" s="6" t="s">
-        <v>248</v>
+        <v>305</v>
       </c>
       <c r="J25" s="6" t="s">
-        <v>248</v>
+        <v>305</v>
       </c>
       <c r="K25" s="6" t="s">
-        <v>249</v>
-      </c>
-      <c r="L25" s="6"/>
-      <c r="M25" s="6" t="s">
-        <v>250</v>
-      </c>
-      <c r="N25" s="17"/>
-      <c r="O25" s="6" t="s">
-        <v>251</v>
-      </c>
-      <c r="P25" s="17"/>
+        <v>306</v>
+      </c>
+      <c r="L25" s="10"/>
+      <c r="M25" s="10" t="s">
+        <v>307</v>
+      </c>
+      <c r="N25" s="6" t="s">
+        <v>308</v>
+      </c>
+      <c r="O25" s="20"/>
+      <c r="P25" s="20"/>
+      <c r="Q25" s="20"/>
+      <c r="R25" s="6"/>
+      <c r="S25" s="6" t="s">
+        <v>309</v>
+      </c>
+      <c r="T25" s="20"/>
+      <c r="U25" s="20"/>
+      <c r="V25" s="20"/>
     </row>
     <row r="26" ht="22.5" customHeight="1">
-      <c r="A26" s="11">
+      <c r="A26" s="12">
         <f t="shared" si="1"/>
         <v>25</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>252</v>
+        <v>310</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="D26" s="8" t="s">
-        <v>254</v>
-      </c>
-      <c r="E26" s="8" t="s">
-        <v>255</v>
+        <v>311</v>
+      </c>
+      <c r="D26" s="18" t="s">
+        <v>312</v>
+      </c>
+      <c r="E26" s="18" t="s">
+        <v>313</v>
       </c>
       <c r="F26" s="7" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="H26" s="6" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="I26" s="6" t="s">
-        <v>86</v>
+        <v>108</v>
       </c>
       <c r="J26" s="6" t="s">
-        <v>256</v>
+        <v>314</v>
       </c>
       <c r="K26" s="6" t="s">
-        <v>257</v>
-      </c>
-      <c r="L26" s="6"/>
-      <c r="M26" s="6" t="s">
-        <v>258</v>
-      </c>
-      <c r="N26" s="17"/>
-      <c r="O26" s="6" t="s">
-        <v>259</v>
-      </c>
-      <c r="P26" s="17"/>
+        <v>315</v>
+      </c>
+      <c r="L26" s="10"/>
+      <c r="M26" s="10" t="s">
+        <v>316</v>
+      </c>
+      <c r="N26" s="6" t="s">
+        <v>317</v>
+      </c>
+      <c r="O26" s="20"/>
+      <c r="P26" s="20"/>
+      <c r="Q26" s="20"/>
+      <c r="R26" s="6"/>
+      <c r="S26" s="6" t="s">
+        <v>318</v>
+      </c>
+      <c r="T26" s="20"/>
+      <c r="U26" s="20"/>
+      <c r="V26" s="20"/>
     </row>
     <row r="27" ht="22.5" customHeight="1">
-      <c r="A27" s="11">
+      <c r="A27" s="12">
         <f t="shared" si="1"/>
         <v>26</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>260</v>
-      </c>
-      <c r="C27" s="15" t="s">
-        <v>253</v>
-      </c>
-      <c r="D27" s="16" t="s">
-        <v>261</v>
-      </c>
-      <c r="E27" s="8" t="s">
-        <v>262</v>
-      </c>
-      <c r="F27" s="15" t="s">
-        <v>20</v>
+        <v>319</v>
+      </c>
+      <c r="C27" s="16" t="s">
+        <v>311</v>
+      </c>
+      <c r="D27" s="17" t="s">
+        <v>320</v>
+      </c>
+      <c r="E27" s="18" t="s">
+        <v>321</v>
+      </c>
+      <c r="F27" s="16" t="s">
+        <v>26</v>
       </c>
       <c r="G27" s="6" t="s">
-        <v>51</v>
+        <v>65</v>
       </c>
       <c r="H27" s="6" t="s">
-        <v>85</v>
+        <v>107</v>
       </c>
       <c r="I27" s="6" t="s">
-        <v>86</v>
+        <v>108</v>
       </c>
       <c r="J27" s="6" t="s">
-        <v>263</v>
+        <v>322</v>
       </c>
       <c r="K27" s="6" t="s">
-        <v>264</v>
-      </c>
-      <c r="L27" s="6"/>
-      <c r="M27" s="6" t="s">
-        <v>265</v>
-      </c>
-      <c r="N27" s="17"/>
-      <c r="O27" s="6" t="s">
-        <v>266</v>
-      </c>
-      <c r="P27" s="17"/>
+        <v>323</v>
+      </c>
+      <c r="L27" s="9"/>
+      <c r="M27" s="9" t="s">
+        <v>324</v>
+      </c>
+      <c r="N27" s="6" t="s">
+        <v>325</v>
+      </c>
+      <c r="O27" s="20"/>
+      <c r="P27" s="20"/>
+      <c r="Q27" s="20"/>
+      <c r="R27" s="6"/>
+      <c r="S27" s="6" t="s">
+        <v>326</v>
+      </c>
+      <c r="T27" s="20"/>
+      <c r="U27" s="20"/>
+      <c r="V27" s="20"/>
     </row>
     <row r="28" ht="22.5" customHeight="1">
-      <c r="A28" s="11">
+      <c r="A28" s="12">
         <f t="shared" si="1"/>
         <v>27</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>267</v>
+        <v>327</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="D28" s="8" t="s">
-        <v>268</v>
-      </c>
-      <c r="E28" s="8" t="s">
-        <v>269</v>
+        <v>311</v>
+      </c>
+      <c r="D28" s="13" t="s">
+        <v>328</v>
+      </c>
+      <c r="E28" s="18" t="s">
+        <v>329</v>
       </c>
       <c r="F28" s="7" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="G28" s="6" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="H28" s="6" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="I28" s="6" t="s">
-        <v>270</v>
+        <v>330</v>
       </c>
       <c r="J28" s="6" t="s">
-        <v>270</v>
+        <v>330</v>
       </c>
       <c r="K28" s="6" t="s">
-        <v>271</v>
-      </c>
-      <c r="L28" s="9"/>
-      <c r="M28" s="9" t="s">
-        <v>272</v>
-      </c>
-      <c r="N28" s="9" t="s">
-        <v>273</v>
-      </c>
-      <c r="O28" s="6" t="s">
-        <v>274</v>
-      </c>
-      <c r="P28" s="17"/>
+        <v>331</v>
+      </c>
+      <c r="L28" s="10"/>
+      <c r="M28" s="10" t="s">
+        <v>332</v>
+      </c>
+      <c r="N28" s="10" t="s">
+        <v>333</v>
+      </c>
+      <c r="O28" s="10"/>
+      <c r="P28" s="10"/>
+      <c r="Q28" s="10" t="s">
+        <v>334</v>
+      </c>
+      <c r="R28" s="6"/>
+      <c r="S28" s="6" t="s">
+        <v>335</v>
+      </c>
+      <c r="T28" s="20"/>
+      <c r="U28" s="20"/>
+      <c r="V28" s="20"/>
     </row>
     <row r="29" ht="22.5" customHeight="1">
-      <c r="A29" s="11">
+      <c r="A29" s="12">
         <f t="shared" si="1"/>
         <v>28</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>275</v>
+        <v>336</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="D29" s="12" t="s">
-        <v>276</v>
-      </c>
-      <c r="E29" s="8" t="s">
-        <v>277</v>
+        <v>311</v>
+      </c>
+      <c r="D29" s="8" t="s">
+        <v>337</v>
+      </c>
+      <c r="E29" s="18" t="s">
+        <v>338</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>62</v>
+        <v>79</v>
       </c>
       <c r="G29" s="6" t="s">
-        <v>278</v>
+        <v>339</v>
       </c>
       <c r="H29" s="6" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="I29" s="6" t="s">
-        <v>279</v>
+        <v>340</v>
       </c>
       <c r="J29" s="6" t="s">
-        <v>279</v>
+        <v>340</v>
       </c>
       <c r="K29" s="6" t="s">
-        <v>280</v>
-      </c>
-      <c r="L29" s="9"/>
-      <c r="M29" s="9" t="s">
-        <v>281</v>
-      </c>
-      <c r="N29" s="9" t="s">
-        <v>282</v>
-      </c>
-      <c r="O29" s="6" t="s">
-        <v>283</v>
-      </c>
-      <c r="P29" s="17"/>
+        <v>341</v>
+      </c>
+      <c r="L29" s="10"/>
+      <c r="M29" s="10" t="s">
+        <v>342</v>
+      </c>
+      <c r="N29" s="10" t="s">
+        <v>343</v>
+      </c>
+      <c r="O29" s="10"/>
+      <c r="P29" s="10"/>
+      <c r="Q29" s="10" t="s">
+        <v>344</v>
+      </c>
+      <c r="R29" s="6"/>
+      <c r="S29" s="6" t="s">
+        <v>345</v>
+      </c>
+      <c r="T29" s="20"/>
+      <c r="U29" s="20"/>
+      <c r="V29" s="20"/>
     </row>
     <row r="30" ht="22.5" customHeight="1">
-      <c r="A30" s="11">
+      <c r="A30" s="12">
         <f t="shared" si="1"/>
         <v>29</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>284</v>
+        <v>346</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="D30" s="8" t="s">
-        <v>285</v>
-      </c>
-      <c r="E30" s="8" t="s">
-        <v>286</v>
+        <v>311</v>
+      </c>
+      <c r="D30" s="13" t="s">
+        <v>347</v>
+      </c>
+      <c r="E30" s="13" t="s">
+        <v>348</v>
       </c>
       <c r="F30" s="7" t="s">
-        <v>62</v>
+        <v>79</v>
       </c>
       <c r="G30" s="6" t="s">
-        <v>287</v>
+        <v>349</v>
       </c>
       <c r="H30" s="6" t="s">
-        <v>287</v>
+        <v>349</v>
       </c>
       <c r="I30" s="6" t="s">
-        <v>288</v>
+        <v>350</v>
       </c>
       <c r="J30" s="6" t="s">
-        <v>288</v>
+        <v>350</v>
       </c>
       <c r="K30" s="6" t="s">
-        <v>289</v>
-      </c>
-      <c r="L30" s="9"/>
-      <c r="M30" s="9" t="s">
-        <v>290</v>
-      </c>
-      <c r="N30" s="9" t="s">
-        <v>291</v>
-      </c>
-      <c r="O30" s="6" t="s">
-        <v>292</v>
-      </c>
-      <c r="P30" s="17"/>
+        <v>351</v>
+      </c>
+      <c r="L30" s="10"/>
+      <c r="M30" s="10" t="s">
+        <v>352</v>
+      </c>
+      <c r="N30" s="10" t="s">
+        <v>353</v>
+      </c>
+      <c r="O30" s="10"/>
+      <c r="P30" s="10"/>
+      <c r="Q30" s="10" t="s">
+        <v>354</v>
+      </c>
+      <c r="R30" s="6"/>
+      <c r="S30" s="6" t="s">
+        <v>355</v>
+      </c>
+      <c r="T30" s="20"/>
+      <c r="U30" s="20"/>
+      <c r="V30" s="20"/>
     </row>
     <row r="31" ht="22.5" customHeight="1">
-      <c r="A31" s="11">
+      <c r="A31" s="12">
         <f t="shared" si="1"/>
         <v>30</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>293</v>
-      </c>
-      <c r="C31" s="15" t="s">
-        <v>253</v>
-      </c>
-      <c r="D31" s="16" t="s">
-        <v>294</v>
-      </c>
-      <c r="E31" s="16" t="s">
-        <v>295</v>
-      </c>
-      <c r="F31" s="15" t="s">
-        <v>62</v>
+        <v>356</v>
+      </c>
+      <c r="C31" s="16" t="s">
+        <v>311</v>
+      </c>
+      <c r="D31" s="13" t="s">
+        <v>357</v>
+      </c>
+      <c r="E31" s="13" t="s">
+        <v>358</v>
+      </c>
+      <c r="F31" s="16" t="s">
+        <v>79</v>
       </c>
       <c r="G31" s="6" t="s">
-        <v>296</v>
+        <v>359</v>
       </c>
       <c r="H31" s="6" t="s">
-        <v>85</v>
+        <v>107</v>
       </c>
       <c r="I31" s="6" t="s">
-        <v>297</v>
+        <v>360</v>
       </c>
       <c r="J31" s="6" t="s">
-        <v>297</v>
+        <v>360</v>
       </c>
       <c r="K31" s="6" t="s">
-        <v>298</v>
-      </c>
-      <c r="L31" s="9"/>
-      <c r="M31" s="9" t="s">
-        <v>299</v>
-      </c>
-      <c r="N31" s="9" t="s">
-        <v>300</v>
-      </c>
-      <c r="O31" s="6" t="s">
-        <v>301</v>
-      </c>
-      <c r="P31" s="17"/>
+        <v>361</v>
+      </c>
+      <c r="L31" s="10"/>
+      <c r="M31" s="10" t="s">
+        <v>362</v>
+      </c>
+      <c r="N31" s="10" t="s">
+        <v>363</v>
+      </c>
+      <c r="O31" s="10"/>
+      <c r="P31" s="10"/>
+      <c r="Q31" s="10" t="s">
+        <v>364</v>
+      </c>
+      <c r="R31" s="6"/>
+      <c r="S31" s="6" t="s">
+        <v>365</v>
+      </c>
+      <c r="T31" s="20"/>
+      <c r="U31" s="20"/>
+      <c r="V31" s="20"/>
     </row>
     <row r="32" ht="22.5" customHeight="1">
-      <c r="A32" s="11">
+      <c r="A32" s="12">
         <f t="shared" si="1"/>
         <v>31</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>302</v>
+        <v>366</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="D32" s="8" t="s">
-        <v>303</v>
-      </c>
-      <c r="E32" s="8" t="s">
-        <v>304</v>
+        <v>311</v>
+      </c>
+      <c r="D32" s="18" t="s">
+        <v>367</v>
+      </c>
+      <c r="E32" s="18" t="s">
+        <v>368</v>
       </c>
       <c r="F32" s="7" t="s">
-        <v>95</v>
+        <v>119</v>
       </c>
       <c r="G32" s="6" t="s">
-        <v>305</v>
+        <v>369</v>
       </c>
       <c r="H32" s="6" t="s">
-        <v>50</v>
+        <v>64</v>
       </c>
       <c r="I32" s="6" t="s">
-        <v>306</v>
+        <v>370</v>
       </c>
       <c r="J32" s="6" t="s">
-        <v>306</v>
+        <v>370</v>
       </c>
       <c r="K32" s="6" t="s">
-        <v>307</v>
-      </c>
-      <c r="L32" s="9"/>
-      <c r="M32" s="9" t="s">
-        <v>308</v>
-      </c>
-      <c r="N32" s="9" t="s">
-        <v>309</v>
-      </c>
-      <c r="O32" s="6" t="s">
-        <v>310</v>
-      </c>
-      <c r="P32" s="17"/>
+        <v>371</v>
+      </c>
+      <c r="L32" s="10"/>
+      <c r="M32" s="10" t="s">
+        <v>372</v>
+      </c>
+      <c r="N32" s="10" t="s">
+        <v>373</v>
+      </c>
+      <c r="O32" s="10"/>
+      <c r="P32" s="10"/>
+      <c r="Q32" s="10" t="s">
+        <v>374</v>
+      </c>
+      <c r="R32" s="6"/>
+      <c r="S32" s="6" t="s">
+        <v>375</v>
+      </c>
+      <c r="T32" s="20"/>
+      <c r="U32" s="20"/>
+      <c r="V32" s="20"/>
     </row>
     <row r="33" ht="22.5" customHeight="1">
-      <c r="A33" s="11">
+      <c r="A33" s="12">
         <f t="shared" si="1"/>
         <v>32</v>
       </c>
       <c r="B33" s="6" t="s">
+        <v>376</v>
+      </c>
+      <c r="C33" s="7" t="s">
         <v>311</v>
       </c>
-      <c r="C33" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="D33" s="8" t="s">
-        <v>312</v>
-      </c>
-      <c r="E33" s="8" t="s">
-        <v>313</v>
+      <c r="D33" s="18" t="s">
+        <v>377</v>
+      </c>
+      <c r="E33" s="18" t="s">
+        <v>378</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>95</v>
+        <v>119</v>
       </c>
       <c r="G33" s="6" t="s">
-        <v>314</v>
+        <v>379</v>
       </c>
       <c r="H33" s="6" t="s">
-        <v>172</v>
+        <v>213</v>
       </c>
       <c r="I33" s="6" t="s">
-        <v>315</v>
+        <v>380</v>
       </c>
       <c r="J33" s="6" t="s">
-        <v>315</v>
+        <v>380</v>
       </c>
       <c r="K33" s="6" t="s">
-        <v>316</v>
-      </c>
-      <c r="L33" s="9"/>
-      <c r="M33" s="9" t="s">
-        <v>317</v>
-      </c>
-      <c r="N33" s="9" t="s">
-        <v>318</v>
-      </c>
-      <c r="O33" s="6" t="s">
-        <v>319</v>
-      </c>
-      <c r="P33" s="17"/>
+        <v>381</v>
+      </c>
+      <c r="L33" s="10"/>
+      <c r="M33" s="10" t="s">
+        <v>382</v>
+      </c>
+      <c r="N33" s="10" t="s">
+        <v>383</v>
+      </c>
+      <c r="O33" s="10"/>
+      <c r="P33" s="10"/>
+      <c r="Q33" s="10" t="s">
+        <v>384</v>
+      </c>
+      <c r="R33" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="S33" s="6" t="s">
+        <v>386</v>
+      </c>
+      <c r="T33" s="20"/>
+      <c r="U33" s="20"/>
+      <c r="V33" s="20"/>
     </row>
     <row r="34" ht="22.5" customHeight="1">
-      <c r="A34" s="11">
+      <c r="A34" s="12">
         <f t="shared" si="1"/>
         <v>33</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>320</v>
-      </c>
-      <c r="C34" s="15" t="s">
-        <v>253</v>
-      </c>
-      <c r="D34" s="8" t="s">
-        <v>321</v>
-      </c>
-      <c r="E34" s="8" t="s">
-        <v>322</v>
-      </c>
-      <c r="F34" s="15" t="s">
-        <v>95</v>
+        <v>387</v>
+      </c>
+      <c r="C34" s="16" t="s">
+        <v>311</v>
+      </c>
+      <c r="D34" s="18" t="s">
+        <v>388</v>
+      </c>
+      <c r="E34" s="18" t="s">
+        <v>389</v>
+      </c>
+      <c r="F34" s="16" t="s">
+        <v>119</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>323</v>
+        <v>390</v>
       </c>
       <c r="H34" s="6" t="s">
-        <v>85</v>
+        <v>107</v>
       </c>
       <c r="I34" s="6" t="s">
-        <v>324</v>
+        <v>391</v>
       </c>
       <c r="J34" s="6" t="s">
-        <v>325</v>
+        <v>392</v>
       </c>
       <c r="K34" s="6" t="s">
-        <v>326</v>
-      </c>
-      <c r="L34" s="9"/>
-      <c r="M34" s="9" t="s">
-        <v>327</v>
-      </c>
-      <c r="N34" s="9" t="s">
-        <v>328</v>
-      </c>
-      <c r="O34" s="6" t="s">
-        <v>329</v>
-      </c>
-      <c r="P34" s="6" t="s">
-        <v>330</v>
+        <v>393</v>
+      </c>
+      <c r="L34" s="10"/>
+      <c r="M34" s="10" t="s">
+        <v>394</v>
+      </c>
+      <c r="N34" s="10" t="s">
+        <v>395</v>
+      </c>
+      <c r="O34" s="10"/>
+      <c r="P34" s="10"/>
+      <c r="Q34" s="10" t="s">
+        <v>396</v>
+      </c>
+      <c r="R34" s="6" t="s">
+        <v>397</v>
+      </c>
+      <c r="S34" s="6" t="s">
+        <v>398</v>
+      </c>
+      <c r="T34" s="6"/>
+      <c r="U34" s="6"/>
+      <c r="V34" s="6" t="s">
+        <v>399</v>
       </c>
     </row>
     <row r="35" ht="22.5" customHeight="1">
-      <c r="A35" s="11">
+      <c r="A35" s="12">
         <f t="shared" si="1"/>
         <v>34</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>331</v>
+        <v>400</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="D35" s="8" t="s">
-        <v>332</v>
-      </c>
-      <c r="E35" s="8" t="s">
-        <v>333</v>
+        <v>311</v>
+      </c>
+      <c r="D35" s="18" t="s">
+        <v>401</v>
+      </c>
+      <c r="E35" s="18" t="s">
+        <v>402</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>127</v>
+        <v>158</v>
       </c>
       <c r="G35" s="6" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="H35" s="6" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="I35" s="6" t="s">
-        <v>334</v>
+        <v>403</v>
       </c>
       <c r="J35" s="6" t="s">
-        <v>335</v>
+        <v>404</v>
       </c>
       <c r="K35" s="6" t="s">
-        <v>336</v>
-      </c>
-      <c r="L35" s="9"/>
-      <c r="M35" s="9" t="s">
-        <v>337</v>
-      </c>
-      <c r="N35" s="9" t="s">
-        <v>338</v>
-      </c>
-      <c r="O35" s="6" t="s">
-        <v>339</v>
-      </c>
-      <c r="P35" s="6" t="s">
-        <v>340</v>
+        <v>405</v>
+      </c>
+      <c r="L35" s="10"/>
+      <c r="M35" s="10" t="s">
+        <v>406</v>
+      </c>
+      <c r="N35" s="10" t="s">
+        <v>407</v>
+      </c>
+      <c r="O35" s="10"/>
+      <c r="P35" s="10"/>
+      <c r="Q35" s="10" t="s">
+        <v>408</v>
+      </c>
+      <c r="R35" s="6" t="s">
+        <v>409</v>
+      </c>
+      <c r="S35" s="6" t="s">
+        <v>410</v>
+      </c>
+      <c r="T35" s="6"/>
+      <c r="U35" s="6"/>
+      <c r="V35" s="6" t="s">
+        <v>411</v>
       </c>
     </row>
     <row r="36" ht="22.5" customHeight="1">
-      <c r="A36" s="11">
+      <c r="A36" s="12">
         <f t="shared" si="1"/>
         <v>35</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>341</v>
-      </c>
-      <c r="C36" s="15" t="s">
-        <v>253</v>
-      </c>
-      <c r="D36" s="8" t="s">
-        <v>342</v>
-      </c>
-      <c r="E36" s="16" t="s">
-        <v>343</v>
-      </c>
-      <c r="F36" s="15" t="s">
-        <v>127</v>
+        <v>412</v>
+      </c>
+      <c r="C36" s="16" t="s">
+        <v>311</v>
+      </c>
+      <c r="D36" s="18" t="s">
+        <v>413</v>
+      </c>
+      <c r="E36" s="17" t="s">
+        <v>414</v>
+      </c>
+      <c r="F36" s="16" t="s">
+        <v>158</v>
       </c>
       <c r="G36" s="6" t="s">
-        <v>85</v>
+        <v>107</v>
       </c>
       <c r="H36" s="6" t="s">
-        <v>85</v>
+        <v>107</v>
       </c>
       <c r="I36" s="6" t="s">
-        <v>86</v>
+        <v>108</v>
       </c>
       <c r="J36" s="6" t="s">
-        <v>344</v>
+        <v>415</v>
       </c>
       <c r="K36" s="6" t="s">
-        <v>345</v>
+        <v>416</v>
       </c>
       <c r="L36" s="9"/>
       <c r="M36" s="9" t="s">
-        <v>346</v>
-      </c>
-      <c r="N36" s="9" t="s">
-        <v>347</v>
-      </c>
-      <c r="O36" s="6" t="s">
-        <v>348</v>
-      </c>
-      <c r="P36" s="6" t="s">
-        <v>349</v>
+        <v>417</v>
+      </c>
+      <c r="N36" s="10" t="s">
+        <v>418</v>
+      </c>
+      <c r="O36" s="10"/>
+      <c r="P36" s="10"/>
+      <c r="Q36" s="10" t="s">
+        <v>419</v>
+      </c>
+      <c r="R36" s="6" t="s">
+        <v>420</v>
+      </c>
+      <c r="S36" s="6" t="s">
+        <v>421</v>
+      </c>
+      <c r="T36" s="6"/>
+      <c r="U36" s="6"/>
+      <c r="V36" s="6" t="s">
+        <v>422</v>
       </c>
     </row>
     <row r="37" ht="22.5" customHeight="1">
-      <c r="A37" s="11">
+      <c r="A37" s="12">
         <f t="shared" si="1"/>
         <v>36</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>350</v>
+        <v>423</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="D37" s="8" t="s">
-        <v>351</v>
-      </c>
-      <c r="E37" s="8" t="s">
-        <v>352</v>
+        <v>311</v>
+      </c>
+      <c r="D37" s="18" t="s">
+        <v>424</v>
+      </c>
+      <c r="E37" s="18" t="s">
+        <v>425</v>
       </c>
       <c r="F37" s="7" t="s">
-        <v>127</v>
+        <v>158</v>
       </c>
       <c r="G37" s="6" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="H37" s="6" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="I37" s="6" t="s">
-        <v>353</v>
+        <v>426</v>
       </c>
       <c r="J37" s="6" t="s">
-        <v>354</v>
+        <v>427</v>
       </c>
       <c r="K37" s="6" t="s">
-        <v>355</v>
-      </c>
-      <c r="L37" s="6"/>
-      <c r="M37" s="6" t="s">
-        <v>356</v>
+        <v>428</v>
+      </c>
+      <c r="L37" s="10"/>
+      <c r="M37" s="10" t="s">
+        <v>429</v>
       </c>
       <c r="N37" s="6" t="s">
-        <v>357</v>
-      </c>
-      <c r="O37" s="6" t="s">
-        <v>358</v>
-      </c>
-      <c r="P37" s="6" t="s">
-        <v>359</v>
+        <v>430</v>
+      </c>
+      <c r="O37" s="6"/>
+      <c r="P37" s="6"/>
+      <c r="Q37" s="6" t="s">
+        <v>431</v>
+      </c>
+      <c r="R37" s="6" t="s">
+        <v>432</v>
+      </c>
+      <c r="S37" s="6" t="s">
+        <v>433</v>
+      </c>
+      <c r="T37" s="6"/>
+      <c r="U37" s="6"/>
+      <c r="V37" s="6" t="s">
+        <v>434</v>
       </c>
     </row>
     <row r="40">
-      <c r="C40" s="19" t="s">
-        <v>360</v>
-      </c>
-      <c r="D40" s="19"/>
-      <c r="F40" s="19"/>
-      <c r="G40" s="19" t="s">
-        <v>361</v>
-      </c>
+      <c r="C40" s="22"/>
+      <c r="D40" s="22"/>
+      <c r="F40" s="22"/>
+      <c r="G40" s="22"/>
     </row>
     <row r="41">
-      <c r="C41" s="19" t="s">
-        <v>362</v>
-      </c>
-      <c r="D41" s="19"/>
-      <c r="F41" s="19"/>
+      <c r="C41" s="22"/>
+      <c r="D41" s="22"/>
+      <c r="F41" s="22"/>
     </row>
     <row r="42">
-      <c r="C42" s="19" t="s">
-        <v>363</v>
-      </c>
-      <c r="D42" s="19"/>
-      <c r="F42" s="19"/>
+      <c r="C42" s="23" t="s">
+        <v>435</v>
+      </c>
+      <c r="D42" s="24" t="s">
+        <v>436</v>
+      </c>
+      <c r="F42" s="22"/>
+    </row>
+    <row r="44">
+      <c r="D44" s="25" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="D45" s="25" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="D47" s="25" t="s">
+        <v>439</v>
+      </c>
     </row>
   </sheetData>
   <dataValidations>
@@ -4208,7 +5132,7 @@
     <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="A2:A37">
       <formula1>AND(ISNUMBER(A2),(NOT(OR(NOT(ISERROR(DATEVALUE(A2))), AND(ISNUMBER(A2), LEFT(CELL("format", A2))="D")))))</formula1>
     </dataValidation>
-    <dataValidation allowBlank="1" showDropDown="1" sqref="B2:B37 D2:E37 I2:J37 M2:P37"/>
+    <dataValidation allowBlank="1" showDropDown="1" sqref="B2:B37 D2:E37 I2:J37 N2:N37 Q2:Q37 S2:S37 V2:V37"/>
   </dataValidations>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="D2"/>
@@ -4284,6 +5208,9 @@
     <hyperlink r:id="rId71" ref="D37"/>
     <hyperlink r:id="rId72" ref="E37"/>
   </hyperlinks>
+  <printOptions gridLines="1" horizontalCentered="1"/>
+  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
+  <pageSetup fitToHeight="0" paperSize="9" cellComments="atEnd" orientation="portrait" pageOrder="overThenDown"/>
   <drawing r:id="rId73"/>
   <tableParts count="2">
     <tablePart r:id="rId76"/>

</xml_diff>